<commit_message>
Atualiza dados — extração 14/10/2026 13:56 (via painel)
</commit_message>
<xml_diff>
--- a/dados/prontuario-equipamentos_1.xlsx
+++ b/dados/prontuario-equipamentos_1.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1130" uniqueCount="1130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1123" uniqueCount="1123">
   <si>
     <t>Geração:</t>
   </si>
@@ -3382,27 +3382,6 @@
   </si>
   <si>
     <t>VOLVO/FH 400 6X2T / VOLVO/FH 400 6X2T</t>
-  </si>
-  <si>
-    <t>SR/LIBRELATO SRCT 2E / SR/LIBRELATO SRCT 2E</t>
-  </si>
-  <si>
-    <t>SR/LIBRELATO SRCD 2E / SR/LIBRELATO SRCD 2E</t>
-  </si>
-  <si>
-    <t>REB/RANDON SR GR TR / REB/RANDON SR GR TR</t>
-  </si>
-  <si>
-    <t>MARCONI BELO SOBRINHO</t>
-  </si>
-  <si>
-    <t>00729704203 / 00729704203</t>
-  </si>
-  <si>
-    <t>SR/RANDON / SR CA</t>
-  </si>
-  <si>
-    <t>VOLVO / FH 460 6X2T</t>
   </si>
 </sst>
 </file>
@@ -3594,7 +3573,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3">
-        <v>46309.34970878472</v>
+        <v>46309.58092883102</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -11175,13 +11154,13 @@
         <v>39</v>
       </c>
       <c r="J89" s="11">
-        <v>46335.125</v>
+        <v>46391.125</v>
       </c>
       <c r="K89" s="0" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="L89" s="0" t="s">
-        <v>209</v>
+        <v>39</v>
       </c>
       <c r="M89" s="0" t="s">
         <v>39</v>
@@ -11190,13 +11169,13 @@
         <v>42</v>
       </c>
       <c r="O89" s="11">
-        <v>46751.125</v>
+        <v>46721.125</v>
       </c>
       <c r="Q89" s="0" t="s">
         <v>42</v>
       </c>
       <c r="R89" s="11">
-        <v>46335.125</v>
+        <v>46491.125</v>
       </c>
       <c r="T89" s="0" t="s">
         <v>43</v>
@@ -46168,7 +46147,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="16384" width="9.140625" customWidth="1"/>
@@ -47486,422 +47465,6 @@
         <v>56</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="0" t="s">
-        <v>388</v>
-      </c>
-      <c r="B42" s="0" t="s">
-        <v>1123</v>
-      </c>
-      <c r="C42" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="D42" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="E42" s="11">
-        <v>46249</v>
-      </c>
-      <c r="F42" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="G42" s="11">
-        <v>46429.125</v>
-      </c>
-      <c r="H42" s="0" t="s">
-        <v>1100</v>
-      </c>
-      <c r="I42" s="0" t="s">
-        <v>1093</v>
-      </c>
-      <c r="J42" s="0" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="0" t="s">
-        <v>390</v>
-      </c>
-      <c r="B43" s="0" t="s">
-        <v>1124</v>
-      </c>
-      <c r="C43" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="D43" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="E43" s="11">
-        <v>46249</v>
-      </c>
-      <c r="F43" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="G43" s="11">
-        <v>46429.125</v>
-      </c>
-      <c r="H43" s="0" t="s">
-        <v>1100</v>
-      </c>
-      <c r="I43" s="0" t="s">
-        <v>1093</v>
-      </c>
-      <c r="J43" s="0" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="0" t="s">
-        <v>700</v>
-      </c>
-      <c r="B44" s="0" t="s">
-        <v>1112</v>
-      </c>
-      <c r="C44" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="D44" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="E44" s="11">
-        <v>46249</v>
-      </c>
-      <c r="F44" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="G44" s="11">
-        <v>46429.125</v>
-      </c>
-      <c r="H44" s="0" t="s">
-        <v>1100</v>
-      </c>
-      <c r="I44" s="0" t="s">
-        <v>1093</v>
-      </c>
-      <c r="J44" s="0" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="0" t="s">
-        <v>1050</v>
-      </c>
-      <c r="B45" s="0" t="s">
-        <v>1125</v>
-      </c>
-      <c r="C45" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="D45" s="0" t="s">
-        <v>29</v>
-      </c>
-      <c r="E45" s="11">
-        <v>46249</v>
-      </c>
-      <c r="F45" s="0" t="s">
-        <v>1097</v>
-      </c>
-      <c r="G45" s="11">
-        <v>46429.125</v>
-      </c>
-      <c r="H45" s="0" t="s">
-        <v>1126</v>
-      </c>
-      <c r="I45" s="0" t="s">
-        <v>1099</v>
-      </c>
-      <c r="J45" s="0" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="0" t="s">
-        <v>1051</v>
-      </c>
-      <c r="B46" s="0" t="s">
-        <v>1125</v>
-      </c>
-      <c r="C46" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="D46" s="0" t="s">
-        <v>29</v>
-      </c>
-      <c r="E46" s="11">
-        <v>46249</v>
-      </c>
-      <c r="F46" s="0" t="s">
-        <v>1097</v>
-      </c>
-      <c r="G46" s="11">
-        <v>46429.125</v>
-      </c>
-      <c r="H46" s="0" t="s">
-        <v>1126</v>
-      </c>
-      <c r="I46" s="0" t="s">
-        <v>1099</v>
-      </c>
-      <c r="J46" s="0" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="0" t="s">
-        <v>1048</v>
-      </c>
-      <c r="B47" s="0" t="s">
-        <v>1127</v>
-      </c>
-      <c r="C47" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="D47" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="E47" s="11">
-        <v>46249</v>
-      </c>
-      <c r="F47" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="G47" s="11">
-        <v>46429.125</v>
-      </c>
-      <c r="H47" s="0" t="s">
-        <v>1121</v>
-      </c>
-      <c r="I47" s="0" t="s">
-        <v>1093</v>
-      </c>
-      <c r="J47" s="0" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="0" t="s">
-        <v>1051</v>
-      </c>
-      <c r="B48" s="0" t="s">
-        <v>1125</v>
-      </c>
-      <c r="C48" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="D48" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="E48" s="11">
-        <v>46249</v>
-      </c>
-      <c r="F48" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="G48" s="11">
-        <v>46429.125</v>
-      </c>
-      <c r="H48" s="0" t="s">
-        <v>1121</v>
-      </c>
-      <c r="I48" s="0" t="s">
-        <v>1093</v>
-      </c>
-      <c r="J48" s="0" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="0" t="s">
-        <v>1050</v>
-      </c>
-      <c r="B49" s="0" t="s">
-        <v>1125</v>
-      </c>
-      <c r="C49" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="D49" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="E49" s="11">
-        <v>46249</v>
-      </c>
-      <c r="F49" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="G49" s="11">
-        <v>46429.125</v>
-      </c>
-      <c r="H49" s="0" t="s">
-        <v>1121</v>
-      </c>
-      <c r="I49" s="0" t="s">
-        <v>1093</v>
-      </c>
-      <c r="J49" s="0" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="B50" s="0" t="s">
-        <v>1128</v>
-      </c>
-      <c r="C50" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="D50" s="0" t="s">
-        <v>29</v>
-      </c>
-      <c r="E50" s="11">
-        <v>46249</v>
-      </c>
-      <c r="F50" s="0" t="s">
-        <v>1097</v>
-      </c>
-      <c r="G50" s="11">
-        <v>46429.125</v>
-      </c>
-      <c r="H50" s="0" t="s">
-        <v>1126</v>
-      </c>
-      <c r="I50" s="0" t="s">
-        <v>1099</v>
-      </c>
-      <c r="J50" s="0" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="B51" s="0" t="s">
-        <v>1128</v>
-      </c>
-      <c r="C51" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="D51" s="0" t="s">
-        <v>29</v>
-      </c>
-      <c r="E51" s="11">
-        <v>46249</v>
-      </c>
-      <c r="F51" s="0" t="s">
-        <v>1097</v>
-      </c>
-      <c r="G51" s="11">
-        <v>46429.125</v>
-      </c>
-      <c r="H51" s="0" t="s">
-        <v>1126</v>
-      </c>
-      <c r="I51" s="0" t="s">
-        <v>1099</v>
-      </c>
-      <c r="J51" s="0" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="B52" s="0" t="s">
-        <v>1128</v>
-      </c>
-      <c r="C52" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="D52" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="E52" s="11">
-        <v>46249</v>
-      </c>
-      <c r="F52" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="G52" s="11">
-        <v>46429.125</v>
-      </c>
-      <c r="H52" s="0" t="s">
-        <v>1100</v>
-      </c>
-      <c r="I52" s="0" t="s">
-        <v>1093</v>
-      </c>
-      <c r="J52" s="0" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="B53" s="0" t="s">
-        <v>1128</v>
-      </c>
-      <c r="C53" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="D53" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="E53" s="11">
-        <v>46249</v>
-      </c>
-      <c r="F53" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="G53" s="11">
-        <v>46429.125</v>
-      </c>
-      <c r="H53" s="0" t="s">
-        <v>1100</v>
-      </c>
-      <c r="I53" s="0" t="s">
-        <v>1093</v>
-      </c>
-      <c r="J53" s="0" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="0" t="s">
-        <v>57</v>
-      </c>
-      <c r="B54" s="0" t="s">
-        <v>1129</v>
-      </c>
-      <c r="C54" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="D54" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="E54" s="11">
-        <v>46249</v>
-      </c>
-      <c r="F54" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="G54" s="11">
-        <v>46429.125</v>
-      </c>
-      <c r="H54" s="0" t="s">
-        <v>1100</v>
-      </c>
-      <c r="I54" s="0" t="s">
-        <v>1093</v>
-      </c>
-      <c r="J54" s="0" t="s">
-        <v>45</v>
-      </c>
-    </row>
   </sheetData>
   <headerFooter/>
 </worksheet>

</xml_diff>

<commit_message>
Atualiza dados — extração 15/10/2026 08:21 (via painel)
</commit_message>
<xml_diff>
--- a/dados/prontuario-equipamentos_1.xlsx
+++ b/dados/prontuario-equipamentos_1.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1123" uniqueCount="1123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1122" uniqueCount="1122">
   <si>
     <t>Geração:</t>
   </si>
@@ -1230,7 +1230,7 @@
     <t>APK0H88</t>
   </si>
   <si>
-    <t>Inspeção Checklist de Qualidade vencida / Documento CRLV vencendo</t>
+    <t>Documento CRLV ausente ou vencido / Inspeção Checklist de Qualidade vencida</t>
   </si>
   <si>
     <t>KDH8F64</t>
@@ -2548,9 +2548,6 @@
   </si>
   <si>
     <t>AVV6018</t>
-  </si>
-  <si>
-    <t>Inspeções Checklist de Segurança SESMT a vencer / Documento CRLV vencendo</t>
   </si>
   <si>
     <t>BDV6I85</t>
@@ -3573,7 +3570,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3">
-        <v>46309.58092883102</v>
+        <v>46310.34958142361</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -8568,10 +8565,10 @@
         <v>46310.125</v>
       </c>
       <c r="K59" s="0" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="L59" s="0" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="M59" s="0" t="s">
         <v>39</v>
@@ -16499,7 +16496,7 @@
         <v>39</v>
       </c>
       <c r="N151" s="0" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="O151" s="11">
         <v>46309.125</v>
@@ -21396,13 +21393,13 @@
         <v>70</v>
       </c>
       <c r="L208" s="0" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="M208" s="0" t="s">
         <v>39</v>
       </c>
       <c r="N208" s="0" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="O208" s="11">
         <v>46309.125</v>
@@ -24043,20 +24040,18 @@
       <c r="H239" s="0" t="s">
         <v>589</v>
       </c>
-      <c r="J239" s="11">
-        <v>46309.125</v>
-      </c>
+      <c r="J239" s="11"/>
       <c r="K239" s="0" t="s">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="L239" s="0" t="s">
-        <v>41</v>
+        <v>71</v>
       </c>
       <c r="M239" s="0" t="s">
         <v>39</v>
       </c>
       <c r="N239" s="0" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="O239" s="11">
         <v>46309.125</v>
@@ -35154,10 +35149,10 @@
         <v>46310.125</v>
       </c>
       <c r="K370" s="0" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="L370" s="0" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="M370" s="0" t="s">
         <v>39</v>
@@ -35742,14 +35737,12 @@
       <c r="H377" s="0" t="s">
         <v>718</v>
       </c>
-      <c r="J377" s="11">
-        <v>46309</v>
-      </c>
+      <c r="J377" s="11"/>
       <c r="K377" s="0" t="s">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="L377" s="0" t="s">
-        <v>845</v>
+        <v>684</v>
       </c>
       <c r="M377" s="0" t="s">
         <v>39</v>
@@ -35811,7 +35804,7 @@
         <v>644</v>
       </c>
       <c r="C378" s="0" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="D378" s="0" t="s">
         <v>111</v>
@@ -35897,13 +35890,13 @@
         <v>644</v>
       </c>
       <c r="C379" s="0" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="D379" s="0" t="s">
         <v>62</v>
       </c>
       <c r="E379" s="0" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="F379" s="0" t="s">
         <v>136</v>
@@ -35912,7 +35905,7 @@
         <v>325</v>
       </c>
       <c r="H379" s="0" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="J379" s="11">
         <v>46341.125</v>
@@ -35983,7 +35976,7 @@
         <v>48</v>
       </c>
       <c r="C380" s="0" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="D380" s="0" t="s">
         <v>201</v>
@@ -36066,10 +36059,10 @@
         <v>643</v>
       </c>
       <c r="B381" s="0" t="s">
+        <v>850</v>
+      </c>
+      <c r="C381" s="0" t="s">
         <v>851</v>
-      </c>
-      <c r="C381" s="0" t="s">
-        <v>852</v>
       </c>
       <c r="D381" s="0" t="s">
         <v>62</v>
@@ -36123,7 +36116,7 @@
         <v>43</v>
       </c>
       <c r="AC381" s="0" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="AD381" s="11">
         <v>46037.467388136574</v>
@@ -36152,16 +36145,16 @@
         <v>643</v>
       </c>
       <c r="B382" s="0" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="C382" s="0" t="s">
+        <v>853</v>
+      </c>
+      <c r="D382" s="0" t="s">
         <v>854</v>
       </c>
-      <c r="D382" s="0" t="s">
+      <c r="E382" s="0" t="s">
         <v>855</v>
-      </c>
-      <c r="E382" s="0" t="s">
-        <v>856</v>
       </c>
       <c r="F382" s="0" t="s">
         <v>59</v>
@@ -36170,14 +36163,14 @@
         <v>136</v>
       </c>
       <c r="H382" s="0" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J382" s="11"/>
       <c r="K382" s="0" t="s">
         <v>70</v>
       </c>
       <c r="L382" s="0" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="M382" s="0" t="s">
         <v>39</v>
@@ -36198,7 +36191,7 @@
         <v>43</v>
       </c>
       <c r="AC382" s="0" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="AD382" s="11">
         <v>46038.63016152778</v>
@@ -36230,19 +36223,19 @@
         <v>48</v>
       </c>
       <c r="C383" s="0" t="s">
+        <v>857</v>
+      </c>
+      <c r="D383" s="0" t="s">
         <v>858</v>
       </c>
-      <c r="D383" s="0" t="s">
+      <c r="E383" s="0" t="s">
+        <v>858</v>
+      </c>
+      <c r="F383" s="0" t="s">
         <v>859</v>
       </c>
-      <c r="E383" s="0" t="s">
+      <c r="G383" s="0" t="s">
         <v>859</v>
-      </c>
-      <c r="F383" s="0" t="s">
-        <v>860</v>
-      </c>
-      <c r="G383" s="0" t="s">
-        <v>860</v>
       </c>
       <c r="H383" s="0" t="s">
         <v>134</v>
@@ -36310,25 +36303,25 @@
     </row>
     <row r="384">
       <c r="A384" s="0" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="B384" s="0" t="s">
         <v>807</v>
       </c>
       <c r="C384" s="0" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="D384" s="0" t="s">
         <v>525</v>
       </c>
       <c r="E384" s="0" t="s">
+        <v>862</v>
+      </c>
+      <c r="F384" s="0" t="s">
+        <v>859</v>
+      </c>
+      <c r="G384" s="0" t="s">
         <v>863</v>
-      </c>
-      <c r="F384" s="0" t="s">
-        <v>860</v>
-      </c>
-      <c r="G384" s="0" t="s">
-        <v>864</v>
       </c>
       <c r="J384" s="11">
         <v>46409.125</v>
@@ -36387,25 +36380,25 @@
     </row>
     <row r="385">
       <c r="A385" s="0" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="B385" s="0" t="s">
         <v>807</v>
       </c>
       <c r="C385" s="0" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="D385" s="0" t="s">
         <v>525</v>
       </c>
       <c r="E385" s="0" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="F385" s="0" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="G385" s="0" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="J385" s="11">
         <v>46413.125</v>
@@ -36467,7 +36460,7 @@
         <v>34</v>
       </c>
       <c r="C386" s="0" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="D386" s="0" t="s">
         <v>50</v>
@@ -36551,7 +36544,7 @@
         <v>34</v>
       </c>
       <c r="C387" s="0" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="D387" s="0" t="s">
         <v>36</v>
@@ -36637,13 +36630,13 @@
         <v>60</v>
       </c>
       <c r="C388" s="0" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="D388" s="0" t="s">
         <v>218</v>
       </c>
       <c r="E388" s="0" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="F388" s="0" t="s">
         <v>203</v>
@@ -36656,7 +36649,7 @@
         <v>70</v>
       </c>
       <c r="L388" s="0" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="M388" s="0" t="s">
         <v>39</v>
@@ -36714,13 +36707,13 @@
         <v>60</v>
       </c>
       <c r="C389" s="0" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="D389" s="0" t="s">
         <v>218</v>
       </c>
       <c r="E389" s="0" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="F389" s="0" t="s">
         <v>203</v>
@@ -36733,7 +36726,7 @@
         <v>70</v>
       </c>
       <c r="L389" s="0" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="M389" s="0" t="s">
         <v>39</v>
@@ -36785,25 +36778,25 @@
     </row>
     <row r="390">
       <c r="A390" s="0" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="B390" s="0" t="s">
+        <v>874</v>
+      </c>
+      <c r="C390" s="0" t="s">
         <v>875</v>
-      </c>
-      <c r="C390" s="0" t="s">
-        <v>876</v>
       </c>
       <c r="D390" s="0" t="s">
         <v>587</v>
       </c>
       <c r="E390" s="0" t="s">
+        <v>876</v>
+      </c>
+      <c r="F390" s="0" t="s">
         <v>877</v>
       </c>
-      <c r="F390" s="0" t="s">
-        <v>878</v>
-      </c>
       <c r="G390" s="0" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="J390" s="11">
         <v>46401.125</v>
@@ -36836,7 +36829,7 @@
         <v>44</v>
       </c>
       <c r="AC390" s="0" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="AD390" s="11">
         <v>46104.56253545139</v>
@@ -36868,7 +36861,7 @@
         <v>644</v>
       </c>
       <c r="C391" s="0" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="D391" s="0" t="s">
         <v>111</v>
@@ -36954,13 +36947,13 @@
         <v>644</v>
       </c>
       <c r="C392" s="0" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="D392" s="0" t="s">
         <v>62</v>
       </c>
       <c r="E392" s="0" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="F392" s="0" t="s">
         <v>326</v>
@@ -37040,13 +37033,13 @@
         <v>60</v>
       </c>
       <c r="C393" s="0" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="D393" s="0" t="s">
         <v>62</v>
       </c>
       <c r="E393" s="0" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="F393" s="0" t="s">
         <v>59</v>
@@ -37059,7 +37052,7 @@
         <v>70</v>
       </c>
       <c r="L393" s="0" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="M393" s="0" t="s">
         <v>39</v>
@@ -37121,7 +37114,7 @@
         <v>644</v>
       </c>
       <c r="C394" s="0" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="D394" s="0" t="s">
         <v>111</v>
@@ -37207,7 +37200,7 @@
         <v>34</v>
       </c>
       <c r="C395" s="0" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="D395" s="0" t="s">
         <v>201</v>
@@ -37293,13 +37286,13 @@
         <v>48</v>
       </c>
       <c r="C396" s="0" t="s">
+        <v>886</v>
+      </c>
+      <c r="D396" s="0" t="s">
         <v>887</v>
       </c>
-      <c r="D396" s="0" t="s">
-        <v>888</v>
-      </c>
       <c r="E396" s="0" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="F396" s="0" t="s">
         <v>243</v>
@@ -37308,7 +37301,7 @@
         <v>243</v>
       </c>
       <c r="H396" s="0" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="J396" s="11">
         <v>46413.125</v>
@@ -37379,13 +37372,13 @@
         <v>48</v>
       </c>
       <c r="C397" s="0" t="s">
+        <v>889</v>
+      </c>
+      <c r="D397" s="0" t="s">
         <v>890</v>
       </c>
-      <c r="D397" s="0" t="s">
-        <v>891</v>
-      </c>
       <c r="E397" s="0" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="F397" s="0" t="s">
         <v>52</v>
@@ -37394,7 +37387,7 @@
         <v>53</v>
       </c>
       <c r="H397" s="0" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="J397" s="11">
         <v>46357.125</v>
@@ -37465,7 +37458,7 @@
         <v>34</v>
       </c>
       <c r="C398" s="0" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="D398" s="0" t="s">
         <v>164</v>
@@ -37480,7 +37473,7 @@
         <v>53</v>
       </c>
       <c r="H398" s="0" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="J398" s="11">
         <v>46361.125</v>
@@ -37551,7 +37544,7 @@
         <v>34</v>
       </c>
       <c r="C399" s="0" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="D399" s="0" t="s">
         <v>50</v>
@@ -37566,7 +37559,7 @@
         <v>152</v>
       </c>
       <c r="H399" s="0" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="J399" s="11">
         <v>46365.125</v>
@@ -37637,7 +37630,7 @@
         <v>34</v>
       </c>
       <c r="C400" s="0" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="D400" s="0" t="s">
         <v>50</v>
@@ -37652,7 +37645,7 @@
         <v>136</v>
       </c>
       <c r="H400" s="0" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="J400" s="11">
         <v>46365.125</v>
@@ -37723,7 +37716,7 @@
         <v>34</v>
       </c>
       <c r="C401" s="0" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="D401" s="0" t="s">
         <v>36</v>
@@ -37738,7 +37731,7 @@
         <v>136</v>
       </c>
       <c r="H401" s="0" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="J401" s="11"/>
       <c r="K401" s="0" t="s">
@@ -37807,13 +37800,13 @@
         <v>48</v>
       </c>
       <c r="C402" s="0" t="s">
+        <v>898</v>
+      </c>
+      <c r="D402" s="0" t="s">
         <v>899</v>
       </c>
-      <c r="D402" s="0" t="s">
-        <v>900</v>
-      </c>
       <c r="E402" s="0" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="F402" s="0" t="s">
         <v>53</v>
@@ -37822,7 +37815,7 @@
         <v>53</v>
       </c>
       <c r="H402" s="0" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="J402" s="11">
         <v>46365.125</v>
@@ -37893,7 +37886,7 @@
         <v>48</v>
       </c>
       <c r="C403" s="0" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="D403" s="0" t="s">
         <v>321</v>
@@ -37908,7 +37901,7 @@
         <v>136</v>
       </c>
       <c r="H403" s="0" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="J403" s="11">
         <v>46362.125</v>
@@ -37979,13 +37972,13 @@
         <v>34</v>
       </c>
       <c r="C404" s="0" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="D404" s="0" t="s">
         <v>79</v>
       </c>
       <c r="E404" s="0" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="F404" s="0" t="s">
         <v>64</v>
@@ -38065,7 +38058,7 @@
         <v>34</v>
       </c>
       <c r="C405" s="0" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="D405" s="0" t="s">
         <v>36</v>
@@ -38151,7 +38144,7 @@
         <v>34</v>
       </c>
       <c r="C406" s="0" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="D406" s="0" t="s">
         <v>36</v>
@@ -38237,13 +38230,13 @@
         <v>34</v>
       </c>
       <c r="C407" s="0" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="D407" s="0" t="s">
         <v>79</v>
       </c>
       <c r="E407" s="0" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="F407" s="0" t="s">
         <v>438</v>
@@ -38252,7 +38245,7 @@
         <v>438</v>
       </c>
       <c r="H407" s="0" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="J407" s="11"/>
       <c r="K407" s="0" t="s">
@@ -38321,13 +38314,13 @@
         <v>34</v>
       </c>
       <c r="C408" s="0" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="D408" s="0" t="s">
         <v>74</v>
       </c>
       <c r="E408" s="0" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="F408" s="0" t="s">
         <v>136</v>
@@ -38336,7 +38329,7 @@
         <v>136</v>
       </c>
       <c r="H408" s="0" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="J408" s="11">
         <v>46310.125</v>
@@ -38407,7 +38400,7 @@
         <v>34</v>
       </c>
       <c r="C409" s="0" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="D409" s="0" t="s">
         <v>74</v>
@@ -38496,7 +38489,7 @@
         <v>34</v>
       </c>
       <c r="C410" s="0" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="D410" s="0" t="s">
         <v>50</v>
@@ -38511,7 +38504,7 @@
         <v>338</v>
       </c>
       <c r="H410" s="0" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="J410" s="11">
         <v>46356.125</v>
@@ -38585,13 +38578,13 @@
         <v>34</v>
       </c>
       <c r="C411" s="0" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="D411" s="0" t="s">
         <v>142</v>
       </c>
       <c r="E411" s="0" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="F411" s="0" t="s">
         <v>144</v>
@@ -38600,7 +38593,7 @@
         <v>144</v>
       </c>
       <c r="H411" s="0" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="J411" s="11"/>
       <c r="K411" s="0" t="s">
@@ -38672,13 +38665,13 @@
         <v>34</v>
       </c>
       <c r="C412" s="0" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="D412" s="0" t="s">
         <v>164</v>
       </c>
       <c r="E412" s="0" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="F412" s="0" t="s">
         <v>95</v>
@@ -38687,7 +38680,7 @@
         <v>95</v>
       </c>
       <c r="H412" s="0" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="J412" s="11">
         <v>46310.125</v>
@@ -38761,7 +38754,7 @@
         <v>34</v>
       </c>
       <c r="C413" s="0" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="D413" s="0" t="s">
         <v>125</v>
@@ -38776,7 +38769,7 @@
         <v>59</v>
       </c>
       <c r="H413" s="0" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="J413" s="11">
         <v>46310.125</v>
@@ -38847,7 +38840,7 @@
         <v>34</v>
       </c>
       <c r="C414" s="0" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="D414" s="0" t="s">
         <v>125</v>
@@ -38862,7 +38855,7 @@
         <v>59</v>
       </c>
       <c r="H414" s="0" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="J414" s="11">
         <v>46310.125</v>
@@ -38933,13 +38926,13 @@
         <v>48</v>
       </c>
       <c r="C415" s="0" t="s">
+        <v>922</v>
+      </c>
+      <c r="D415" s="0" t="s">
         <v>923</v>
       </c>
-      <c r="D415" s="0" t="s">
-        <v>924</v>
-      </c>
       <c r="E415" s="0" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="F415" s="0" t="s">
         <v>203</v>
@@ -39016,7 +39009,7 @@
         <v>34</v>
       </c>
       <c r="C416" s="0" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="D416" s="0" t="s">
         <v>62</v>
@@ -39102,7 +39095,7 @@
         <v>34</v>
       </c>
       <c r="C417" s="0" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="D417" s="0" t="s">
         <v>36</v>
@@ -39117,14 +39110,14 @@
         <v>38</v>
       </c>
       <c r="H417" s="0" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="J417" s="11"/>
       <c r="K417" s="0" t="s">
         <v>70</v>
       </c>
       <c r="L417" s="0" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="M417" s="0" t="s">
         <v>39</v>
@@ -39189,7 +39182,7 @@
         <v>34</v>
       </c>
       <c r="C418" s="0" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="D418" s="0" t="s">
         <v>36</v>
@@ -39204,14 +39197,14 @@
         <v>38</v>
       </c>
       <c r="H418" s="0" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="J418" s="11"/>
       <c r="K418" s="0" t="s">
         <v>70</v>
       </c>
       <c r="L418" s="0" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="M418" s="0" t="s">
         <v>39</v>
@@ -39276,13 +39269,13 @@
         <v>48</v>
       </c>
       <c r="C419" s="0" t="s">
+        <v>929</v>
+      </c>
+      <c r="D419" s="0" t="s">
         <v>930</v>
       </c>
-      <c r="D419" s="0" t="s">
-        <v>931</v>
-      </c>
       <c r="E419" s="0" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="F419" s="0" t="s">
         <v>64</v>
@@ -39359,7 +39352,7 @@
         <v>48</v>
       </c>
       <c r="C420" s="0" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="D420" s="0" t="s">
         <v>321</v>
@@ -39442,13 +39435,13 @@
         <v>34</v>
       </c>
       <c r="C421" s="0" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="D421" s="0" t="s">
         <v>314</v>
       </c>
       <c r="E421" s="0" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="F421" s="0" t="s">
         <v>95</v>
@@ -39457,14 +39450,14 @@
         <v>38</v>
       </c>
       <c r="H421" s="0" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="J421" s="11"/>
       <c r="K421" s="0" t="s">
         <v>70</v>
       </c>
       <c r="L421" s="0" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="M421" s="0" t="s">
         <v>39</v>
@@ -39529,7 +39522,7 @@
         <v>48</v>
       </c>
       <c r="C422" s="0" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="D422" s="0" t="s">
         <v>387</v>
@@ -39612,13 +39605,13 @@
         <v>48</v>
       </c>
       <c r="C423" s="0" t="s">
+        <v>936</v>
+      </c>
+      <c r="D423" s="0" t="s">
         <v>937</v>
       </c>
-      <c r="D423" s="0" t="s">
-        <v>938</v>
-      </c>
       <c r="E423" s="0" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="F423" s="0" t="s">
         <v>152</v>
@@ -39695,7 +39688,7 @@
         <v>60</v>
       </c>
       <c r="C424" s="0" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="D424" s="0" t="s">
         <v>50</v>
@@ -39710,7 +39703,7 @@
         <v>170</v>
       </c>
       <c r="H424" s="0" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="J424" s="11">
         <v>46310.125</v>
@@ -39781,13 +39774,13 @@
         <v>60</v>
       </c>
       <c r="C425" s="0" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="D425" s="0" t="s">
         <v>79</v>
       </c>
       <c r="E425" s="0" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="F425" s="0" t="s">
         <v>331</v>
@@ -39796,7 +39789,7 @@
         <v>331</v>
       </c>
       <c r="H425" s="0" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="J425" s="11">
         <v>46373.125</v>
@@ -39867,7 +39860,7 @@
         <v>60</v>
       </c>
       <c r="C426" s="0" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="D426" s="0" t="s">
         <v>79</v>
@@ -39882,7 +39875,7 @@
         <v>523</v>
       </c>
       <c r="H426" s="0" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="J426" s="11">
         <v>46310.125</v>
@@ -39956,13 +39949,13 @@
         <v>60</v>
       </c>
       <c r="C427" s="0" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="D427" s="0" t="s">
         <v>164</v>
       </c>
       <c r="E427" s="0" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="F427" s="0" t="s">
         <v>171</v>
@@ -40045,7 +40038,7 @@
         <v>60</v>
       </c>
       <c r="C428" s="0" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="D428" s="0" t="s">
         <v>79</v>
@@ -40060,7 +40053,7 @@
         <v>53</v>
       </c>
       <c r="H428" s="0" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="J428" s="11">
         <v>46373.125</v>
@@ -40131,13 +40124,13 @@
         <v>60</v>
       </c>
       <c r="C429" s="0" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="D429" s="0" t="s">
         <v>164</v>
       </c>
       <c r="E429" s="0" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="F429" s="0" t="s">
         <v>257</v>
@@ -40146,7 +40139,7 @@
         <v>257</v>
       </c>
       <c r="H429" s="0" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="J429" s="11">
         <v>46310.125</v>
@@ -40217,7 +40210,7 @@
         <v>60</v>
       </c>
       <c r="C430" s="0" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="D430" s="0" t="s">
         <v>50</v>
@@ -40232,7 +40225,7 @@
         <v>152</v>
       </c>
       <c r="H430" s="0" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="J430" s="11">
         <v>46373.125</v>
@@ -40303,13 +40296,13 @@
         <v>60</v>
       </c>
       <c r="C431" s="0" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="D431" s="0" t="s">
         <v>730</v>
       </c>
       <c r="E431" s="0" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="F431" s="0" t="s">
         <v>212</v>
@@ -40389,7 +40382,7 @@
         <v>60</v>
       </c>
       <c r="C432" s="0" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="D432" s="0" t="s">
         <v>249</v>
@@ -40404,7 +40397,7 @@
         <v>326</v>
       </c>
       <c r="H432" s="0" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="J432" s="11">
         <v>46310.125</v>
@@ -40475,7 +40468,7 @@
         <v>60</v>
       </c>
       <c r="C433" s="0" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="D433" s="0" t="s">
         <v>259</v>
@@ -40490,7 +40483,7 @@
         <v>95</v>
       </c>
       <c r="H433" s="0" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="J433" s="11">
         <v>46310.125</v>
@@ -40561,13 +40554,13 @@
         <v>60</v>
       </c>
       <c r="C434" s="0" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="D434" s="0" t="s">
         <v>259</v>
       </c>
       <c r="E434" s="0" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="F434" s="0" t="s">
         <v>170</v>
@@ -40576,7 +40569,7 @@
         <v>170</v>
       </c>
       <c r="H434" s="0" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="J434" s="11">
         <v>46310.125</v>
@@ -40650,7 +40643,7 @@
         <v>60</v>
       </c>
       <c r="C435" s="0" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="D435" s="0" t="s">
         <v>249</v>
@@ -40739,13 +40732,13 @@
         <v>60</v>
       </c>
       <c r="C436" s="0" t="s">
+        <v>961</v>
+      </c>
+      <c r="D436" s="0" t="s">
         <v>962</v>
       </c>
-      <c r="D436" s="0" t="s">
+      <c r="E436" s="0" t="s">
         <v>963</v>
-      </c>
-      <c r="E436" s="0" t="s">
-        <v>964</v>
       </c>
       <c r="F436" s="0" t="s">
         <v>293</v>
@@ -40825,7 +40818,7 @@
         <v>60</v>
       </c>
       <c r="C437" s="0" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="D437" s="0" t="s">
         <v>259</v>
@@ -40914,7 +40907,7 @@
         <v>60</v>
       </c>
       <c r="C438" s="0" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="D438" s="0" t="s">
         <v>411</v>
@@ -40929,7 +40922,7 @@
         <v>171</v>
       </c>
       <c r="H438" s="0" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="J438" s="11">
         <v>46373.125</v>
@@ -41000,7 +40993,7 @@
         <v>60</v>
       </c>
       <c r="C439" s="0" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
       <c r="D439" s="0" t="s">
         <v>259</v>
@@ -41086,7 +41079,7 @@
         <v>60</v>
       </c>
       <c r="C440" s="0" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="D440" s="0" t="s">
         <v>259</v>
@@ -41172,7 +41165,7 @@
         <v>60</v>
       </c>
       <c r="C441" s="0" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="D441" s="0" t="s">
         <v>411</v>
@@ -41187,7 +41180,7 @@
         <v>326</v>
       </c>
       <c r="H441" s="0" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="J441" s="11">
         <v>46373.125</v>
@@ -41258,7 +41251,7 @@
         <v>60</v>
       </c>
       <c r="C442" s="0" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="D442" s="0" t="s">
         <v>259</v>
@@ -41273,7 +41266,7 @@
         <v>76</v>
       </c>
       <c r="H442" s="0" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="J442" s="11">
         <v>46310.125</v>
@@ -41344,7 +41337,7 @@
         <v>60</v>
       </c>
       <c r="C443" s="0" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="D443" s="0" t="s">
         <v>259</v>
@@ -41433,7 +41426,7 @@
         <v>60</v>
       </c>
       <c r="C444" s="0" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="D444" s="0" t="s">
         <v>411</v>
@@ -41448,7 +41441,7 @@
         <v>171</v>
       </c>
       <c r="H444" s="0" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="J444" s="11">
         <v>46373.125</v>
@@ -41519,7 +41512,7 @@
         <v>60</v>
       </c>
       <c r="C445" s="0" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="D445" s="0" t="s">
         <v>259</v>
@@ -41605,7 +41598,7 @@
         <v>60</v>
       </c>
       <c r="C446" s="0" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="D446" s="0" t="s">
         <v>164</v>
@@ -41620,7 +41613,7 @@
         <v>179</v>
       </c>
       <c r="H446" s="0" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="J446" s="11">
         <v>46310.125</v>
@@ -41691,13 +41684,13 @@
         <v>60</v>
       </c>
       <c r="C447" s="0" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="D447" s="0" t="s">
         <v>164</v>
       </c>
       <c r="E447" s="0" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="F447" s="0" t="s">
         <v>501</v>
@@ -41706,7 +41699,7 @@
         <v>501</v>
       </c>
       <c r="H447" s="0" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="J447" s="11">
         <v>46373.125</v>
@@ -41777,7 +41770,7 @@
         <v>60</v>
       </c>
       <c r="C448" s="0" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="D448" s="0" t="s">
         <v>164</v>
@@ -41792,7 +41785,7 @@
         <v>517</v>
       </c>
       <c r="H448" s="0" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="J448" s="11">
         <v>46310.125</v>
@@ -41863,13 +41856,13 @@
         <v>60</v>
       </c>
       <c r="C449" s="0" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="D449" s="0" t="s">
         <v>164</v>
       </c>
       <c r="E449" s="0" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="F449" s="0" t="s">
         <v>331</v>
@@ -41878,7 +41871,7 @@
         <v>331</v>
       </c>
       <c r="H449" s="0" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="J449" s="11">
         <v>46310.125</v>
@@ -41952,7 +41945,7 @@
         <v>60</v>
       </c>
       <c r="C450" s="0" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="D450" s="0" t="s">
         <v>164</v>
@@ -41967,7 +41960,7 @@
         <v>331</v>
       </c>
       <c r="H450" s="0" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="J450" s="11"/>
       <c r="K450" s="0" t="s">
@@ -42030,25 +42023,25 @@
     </row>
     <row r="451">
       <c r="A451" s="0" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="B451" s="0" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="C451" s="0" t="s">
+        <v>986</v>
+      </c>
+      <c r="D451" s="0" t="s">
         <v>987</v>
       </c>
-      <c r="D451" s="0" t="s">
-        <v>988</v>
-      </c>
       <c r="E451" s="0" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="F451" s="0" t="s">
         <v>299</v>
       </c>
       <c r="G451" s="0" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="J451" s="11">
         <v>46310.125</v>
@@ -42081,7 +42074,7 @@
         <v>44</v>
       </c>
       <c r="AC451" s="0" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="AD451" s="11">
         <v>46203.65469700231</v>
@@ -42113,13 +42106,13 @@
         <v>644</v>
       </c>
       <c r="C452" s="0" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="D452" s="0" t="s">
         <v>62</v>
       </c>
       <c r="E452" s="0" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="F452" s="0" t="s">
         <v>326</v>
@@ -42128,7 +42121,7 @@
         <v>326</v>
       </c>
       <c r="H452" s="0" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="J452" s="11">
         <v>46365.125</v>
@@ -42199,7 +42192,7 @@
         <v>644</v>
       </c>
       <c r="C453" s="0" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="D453" s="0" t="s">
         <v>769</v>
@@ -42214,7 +42207,7 @@
         <v>212</v>
       </c>
       <c r="H453" s="0" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="J453" s="11">
         <v>46365.125</v>
@@ -42285,13 +42278,13 @@
         <v>34</v>
       </c>
       <c r="C454" s="0" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="D454" s="0" t="s">
         <v>79</v>
       </c>
       <c r="E454" s="0" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="F454" s="0" t="s">
         <v>87</v>
@@ -42368,7 +42361,7 @@
         <v>34</v>
       </c>
       <c r="C455" s="0" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="D455" s="0" t="s">
         <v>36</v>
@@ -42451,13 +42444,13 @@
         <v>807</v>
       </c>
       <c r="C456" s="0" t="s">
+        <v>993</v>
+      </c>
+      <c r="D456" s="0" t="s">
         <v>994</v>
       </c>
-      <c r="D456" s="0" t="s">
-        <v>995</v>
-      </c>
       <c r="E456" s="0" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="F456" s="0" t="s">
         <v>203</v>
@@ -42525,7 +42518,7 @@
         <v>34</v>
       </c>
       <c r="C457" s="0" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="D457" s="0" t="s">
         <v>125</v>
@@ -42540,7 +42533,7 @@
         <v>76</v>
       </c>
       <c r="H457" s="0" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="J457" s="11">
         <v>46387.125</v>
@@ -42611,7 +42604,7 @@
         <v>34</v>
       </c>
       <c r="C458" s="0" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="D458" s="0" t="s">
         <v>125</v>
@@ -42626,7 +42619,7 @@
         <v>76</v>
       </c>
       <c r="H458" s="0" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="J458" s="11">
         <v>46326.125</v>
@@ -42697,7 +42690,7 @@
         <v>34</v>
       </c>
       <c r="C459" s="0" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
       <c r="D459" s="0" t="s">
         <v>50</v>
@@ -42712,7 +42705,7 @@
         <v>325</v>
       </c>
       <c r="H459" s="0" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="J459" s="11">
         <v>46326.125</v>
@@ -42783,13 +42776,13 @@
         <v>34</v>
       </c>
       <c r="C460" s="0" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="D460" s="0" t="s">
         <v>50</v>
       </c>
       <c r="E460" s="0" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="F460" s="0" t="s">
         <v>133</v>
@@ -42869,13 +42862,13 @@
         <v>34</v>
       </c>
       <c r="C461" s="0" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="D461" s="0" t="s">
         <v>182</v>
       </c>
       <c r="E461" s="0" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="F461" s="0" t="s">
         <v>151</v>
@@ -42884,7 +42877,7 @@
         <v>151</v>
       </c>
       <c r="H461" s="0" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="J461" s="11">
         <v>46310.125</v>
@@ -42955,13 +42948,13 @@
         <v>60</v>
       </c>
       <c r="C462" s="0" t="s">
+        <v>1004</v>
+      </c>
+      <c r="D462" s="0" t="s">
         <v>1005</v>
       </c>
-      <c r="D462" s="0" t="s">
+      <c r="E462" s="0" t="s">
         <v>1006</v>
-      </c>
-      <c r="E462" s="0" t="s">
-        <v>1007</v>
       </c>
       <c r="F462" s="0" t="s">
         <v>417</v>
@@ -42970,7 +42963,7 @@
         <v>417</v>
       </c>
       <c r="H462" s="0" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="J462" s="11">
         <v>46310.125</v>
@@ -43038,7 +43031,7 @@
         <v>60</v>
       </c>
       <c r="C463" s="0" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="D463" s="0" t="s">
         <v>79</v>
@@ -43053,7 +43046,7 @@
         <v>331</v>
       </c>
       <c r="H463" s="0" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="J463" s="11">
         <v>46406.125</v>
@@ -43124,13 +43117,13 @@
         <v>60</v>
       </c>
       <c r="C464" s="0" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="D464" s="0" t="s">
         <v>79</v>
       </c>
       <c r="E464" s="0" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="F464" s="0" t="s">
         <v>81</v>
@@ -43139,7 +43132,7 @@
         <v>231</v>
       </c>
       <c r="H464" s="0" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="J464" s="11">
         <v>46407.125</v>
@@ -43210,7 +43203,7 @@
         <v>60</v>
       </c>
       <c r="C465" s="0" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="D465" s="0" t="s">
         <v>249</v>
@@ -43225,7 +43218,7 @@
         <v>136</v>
       </c>
       <c r="H465" s="0" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="J465" s="11">
         <v>46407.125</v>
@@ -43296,7 +43289,7 @@
         <v>60</v>
       </c>
       <c r="C466" s="0" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
       <c r="D466" s="0" t="s">
         <v>249</v>
@@ -43311,7 +43304,7 @@
         <v>136</v>
       </c>
       <c r="H466" s="0" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="J466" s="11">
         <v>46407.125</v>
@@ -43382,7 +43375,7 @@
         <v>60</v>
       </c>
       <c r="C467" s="0" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="D467" s="0" t="s">
         <v>769</v>
@@ -43397,7 +43390,7 @@
         <v>53</v>
       </c>
       <c r="H467" s="0" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="J467" s="11">
         <v>46406.125</v>
@@ -43468,7 +43461,7 @@
         <v>60</v>
       </c>
       <c r="C468" s="0" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
       <c r="D468" s="0" t="s">
         <v>259</v>
@@ -43483,7 +43476,7 @@
         <v>76</v>
       </c>
       <c r="H468" s="0" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="J468" s="11">
         <v>46373.125</v>
@@ -43554,7 +43547,7 @@
         <v>48</v>
       </c>
       <c r="C469" s="0" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="D469" s="0" t="s">
         <v>50</v>
@@ -43640,13 +43633,13 @@
         <v>226</v>
       </c>
       <c r="C470" s="0" t="s">
+        <v>1019</v>
+      </c>
+      <c r="D470" s="0" t="s">
         <v>1020</v>
       </c>
-      <c r="D470" s="0" t="s">
+      <c r="E470" s="0" t="s">
         <v>1021</v>
-      </c>
-      <c r="E470" s="0" t="s">
-        <v>1022</v>
       </c>
       <c r="F470" s="0" t="s">
         <v>144</v>
@@ -43655,7 +43648,7 @@
         <v>144</v>
       </c>
       <c r="H470" s="0" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="J470" s="11">
         <v>46398.125</v>
@@ -43723,13 +43716,13 @@
         <v>807</v>
       </c>
       <c r="C471" s="0" t="s">
+        <v>1023</v>
+      </c>
+      <c r="D471" s="0" t="s">
         <v>1024</v>
       </c>
-      <c r="D471" s="0" t="s">
+      <c r="E471" s="0" t="s">
         <v>1025</v>
-      </c>
-      <c r="E471" s="0" t="s">
-        <v>1026</v>
       </c>
       <c r="F471" s="0" t="s">
         <v>203</v>
@@ -43768,7 +43761,7 @@
         <v>44</v>
       </c>
       <c r="AC471" s="0" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="AD471" s="11">
         <v>46219.55652277778</v>
@@ -43800,7 +43793,7 @@
         <v>48</v>
       </c>
       <c r="C472" s="0" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="D472" s="0" t="s">
         <v>381</v>
@@ -43815,7 +43808,7 @@
         <v>338</v>
       </c>
       <c r="H472" s="0" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="J472" s="11">
         <v>46402.125</v>
@@ -43886,7 +43879,7 @@
         <v>60</v>
       </c>
       <c r="C473" s="0" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="D473" s="0" t="s">
         <v>50</v>
@@ -43901,7 +43894,7 @@
         <v>81</v>
       </c>
       <c r="H473" s="0" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="J473" s="11">
         <v>46346.125</v>
@@ -43972,13 +43965,13 @@
         <v>60</v>
       </c>
       <c r="C474" s="0" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="D474" s="0" t="s">
         <v>249</v>
       </c>
       <c r="E474" s="0" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="F474" s="0" t="s">
         <v>338</v>
@@ -43987,7 +43980,7 @@
         <v>52</v>
       </c>
       <c r="H474" s="0" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="J474" s="11">
         <v>46346.125</v>
@@ -44058,7 +44051,7 @@
         <v>60</v>
       </c>
       <c r="C475" s="0" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="D475" s="0" t="s">
         <v>249</v>
@@ -44073,7 +44066,7 @@
         <v>211</v>
       </c>
       <c r="H475" s="0" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="J475" s="11">
         <v>46310.125</v>
@@ -44144,7 +44137,7 @@
         <v>60</v>
       </c>
       <c r="C476" s="0" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="D476" s="0" t="s">
         <v>50</v>
@@ -44159,7 +44152,7 @@
         <v>152</v>
       </c>
       <c r="H476" s="0" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="J476" s="11">
         <v>46407.125</v>
@@ -44230,7 +44223,7 @@
         <v>60</v>
       </c>
       <c r="C477" s="0" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="D477" s="0" t="s">
         <v>259</v>
@@ -44245,7 +44238,7 @@
         <v>231</v>
       </c>
       <c r="H477" s="0" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="J477" s="11">
         <v>46407.125</v>
@@ -44316,7 +44309,7 @@
         <v>60</v>
       </c>
       <c r="C478" s="0" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
       <c r="D478" s="0" t="s">
         <v>259</v>
@@ -44331,7 +44324,7 @@
         <v>231</v>
       </c>
       <c r="H478" s="0" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="J478" s="11">
         <v>46407.125</v>
@@ -44402,7 +44395,7 @@
         <v>622</v>
       </c>
       <c r="C479" s="0" t="s">
-        <v>1040</v>
+        <v>1039</v>
       </c>
       <c r="D479" s="0" t="s">
         <v>218</v>
@@ -44482,13 +44475,13 @@
         <v>622</v>
       </c>
       <c r="C480" s="0" t="s">
+        <v>1040</v>
+      </c>
+      <c r="D480" s="0" t="s">
         <v>1041</v>
       </c>
-      <c r="D480" s="0" t="s">
-        <v>1042</v>
-      </c>
       <c r="E480" s="0" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="F480" s="0" t="s">
         <v>438</v>
@@ -44562,13 +44555,13 @@
         <v>48</v>
       </c>
       <c r="C481" s="0" t="s">
+        <v>1042</v>
+      </c>
+      <c r="D481" s="0" t="s">
         <v>1043</v>
       </c>
-      <c r="D481" s="0" t="s">
-        <v>1044</v>
-      </c>
       <c r="E481" s="0" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
       <c r="F481" s="0" t="s">
         <v>100</v>
@@ -44648,13 +44641,13 @@
         <v>34</v>
       </c>
       <c r="C482" s="0" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="D482" s="0" t="s">
         <v>79</v>
       </c>
       <c r="E482" s="0" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
       <c r="F482" s="0" t="s">
         <v>38</v>
@@ -44663,7 +44656,7 @@
         <v>38</v>
       </c>
       <c r="H482" s="0" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="J482" s="11">
         <v>46310.125</v>
@@ -44734,13 +44727,13 @@
         <v>48</v>
       </c>
       <c r="C483" s="0" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D483" s="0" t="s">
         <v>1048</v>
       </c>
-      <c r="D483" s="0" t="s">
-        <v>1049</v>
-      </c>
       <c r="E483" s="0" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="F483" s="0" t="s">
         <v>139</v>
@@ -44817,7 +44810,7 @@
         <v>48</v>
       </c>
       <c r="C484" s="0" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="D484" s="0" t="s">
         <v>344</v>
@@ -44900,7 +44893,7 @@
         <v>48</v>
       </c>
       <c r="C485" s="0" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="D485" s="0" t="s">
         <v>344</v>
@@ -44983,7 +44976,7 @@
         <v>34</v>
       </c>
       <c r="C486" s="0" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="D486" s="0" t="s">
         <v>249</v>
@@ -44998,7 +44991,7 @@
         <v>38</v>
       </c>
       <c r="H486" s="0" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="J486" s="11">
         <v>46362.125</v>
@@ -45069,7 +45062,7 @@
         <v>34</v>
       </c>
       <c r="C487" s="0" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
       <c r="D487" s="0" t="s">
         <v>249</v>
@@ -45084,7 +45077,7 @@
         <v>38</v>
       </c>
       <c r="H487" s="0" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="J487" s="11">
         <v>46362.125</v>
@@ -45155,7 +45148,7 @@
         <v>48</v>
       </c>
       <c r="C488" s="0" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="D488" s="0" t="s">
         <v>365</v>
@@ -45238,13 +45231,13 @@
         <v>48</v>
       </c>
       <c r="C489" s="0" t="s">
+        <v>1054</v>
+      </c>
+      <c r="D489" s="0" t="s">
         <v>1055</v>
       </c>
-      <c r="D489" s="0" t="s">
-        <v>1056</v>
-      </c>
       <c r="E489" s="0" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="F489" s="0" t="s">
         <v>257</v>
@@ -45321,13 +45314,13 @@
         <v>48</v>
       </c>
       <c r="C490" s="0" t="s">
+        <v>1056</v>
+      </c>
+      <c r="D490" s="0" t="s">
         <v>1057</v>
       </c>
-      <c r="D490" s="0" t="s">
-        <v>1058</v>
-      </c>
       <c r="E490" s="0" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="F490" s="0" t="s">
         <v>133</v>
@@ -45404,13 +45397,13 @@
         <v>48</v>
       </c>
       <c r="C491" s="0" t="s">
+        <v>1058</v>
+      </c>
+      <c r="D491" s="0" t="s">
         <v>1059</v>
       </c>
-      <c r="D491" s="0" t="s">
-        <v>1060</v>
-      </c>
       <c r="E491" s="0" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="F491" s="0" t="s">
         <v>293</v>
@@ -45487,13 +45480,13 @@
         <v>60</v>
       </c>
       <c r="C492" s="0" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="D492" s="0" t="s">
         <v>525</v>
       </c>
       <c r="E492" s="0" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="F492" s="0" t="s">
         <v>107</v>
@@ -45573,13 +45566,13 @@
         <v>644</v>
       </c>
       <c r="C493" s="0" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="D493" s="0" t="s">
         <v>74</v>
       </c>
       <c r="E493" s="0" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
       <c r="F493" s="0" t="s">
         <v>292</v>
@@ -45588,7 +45581,7 @@
         <v>292</v>
       </c>
       <c r="H493" s="0" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="J493" s="11">
         <v>46372.125</v>
@@ -45659,19 +45652,19 @@
         <v>34</v>
       </c>
       <c r="C494" s="0" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="D494" s="0" t="s">
         <v>587</v>
       </c>
       <c r="E494" s="0" t="s">
+        <v>1065</v>
+      </c>
+      <c r="F494" s="0" t="s">
+        <v>863</v>
+      </c>
+      <c r="G494" s="0" t="s">
         <v>1066</v>
-      </c>
-      <c r="F494" s="0" t="s">
-        <v>864</v>
-      </c>
-      <c r="G494" s="0" t="s">
-        <v>1067</v>
       </c>
       <c r="H494" s="0" t="s">
         <v>204</v>
@@ -45745,19 +45738,19 @@
         <v>34</v>
       </c>
       <c r="C495" s="0" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="D495" s="0" t="s">
         <v>587</v>
       </c>
       <c r="E495" s="0" t="s">
+        <v>1065</v>
+      </c>
+      <c r="F495" s="0" t="s">
+        <v>863</v>
+      </c>
+      <c r="G495" s="0" t="s">
         <v>1066</v>
-      </c>
-      <c r="F495" s="0" t="s">
-        <v>864</v>
-      </c>
-      <c r="G495" s="0" t="s">
-        <v>1067</v>
       </c>
       <c r="H495" s="0" t="s">
         <v>204</v>
@@ -45831,7 +45824,7 @@
         <v>226</v>
       </c>
       <c r="C496" s="0" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="D496" s="0" t="s">
         <v>525</v>
@@ -45911,13 +45904,13 @@
         <v>807</v>
       </c>
       <c r="C497" s="0" t="s">
+        <v>1069</v>
+      </c>
+      <c r="D497" s="0" t="s">
         <v>1070</v>
       </c>
-      <c r="D497" s="0" t="s">
-        <v>1071</v>
-      </c>
       <c r="E497" s="0" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="F497" s="0" t="s">
         <v>293</v>
@@ -45982,16 +45975,16 @@
         <v>814</v>
       </c>
       <c r="B498" s="0" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="C498" s="0" t="s">
+        <v>1071</v>
+      </c>
+      <c r="D498" s="0" t="s">
+        <v>937</v>
+      </c>
+      <c r="E498" s="0" t="s">
         <v>1072</v>
-      </c>
-      <c r="D498" s="0" t="s">
-        <v>938</v>
-      </c>
-      <c r="E498" s="0" t="s">
-        <v>1073</v>
       </c>
       <c r="F498" s="0" t="s">
         <v>170</v>
@@ -46004,7 +45997,7 @@
         <v>70</v>
       </c>
       <c r="L498" s="0" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
       <c r="M498" s="0" t="s">
         <v>39</v>
@@ -46028,7 +46021,7 @@
         <v>43</v>
       </c>
       <c r="AC498" s="0" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="AD498" s="11">
         <v>46303.38590450231</v>
@@ -46049,16 +46042,16 @@
         <v>814</v>
       </c>
       <c r="B499" s="0" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="C499" s="0" t="s">
+        <v>1074</v>
+      </c>
+      <c r="D499" s="0" t="s">
         <v>1075</v>
       </c>
-      <c r="D499" s="0" t="s">
-        <v>1076</v>
-      </c>
       <c r="E499" s="0" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
       <c r="F499" s="0" t="s">
         <v>171</v>
@@ -46071,7 +46064,7 @@
         <v>70</v>
       </c>
       <c r="L499" s="0" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="M499" s="0" t="s">
         <v>39</v>
@@ -46095,7 +46088,7 @@
         <v>43</v>
       </c>
       <c r="AC499" s="0" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="AD499" s="11">
         <v>46303.38891412037</v>
@@ -46158,28 +46151,28 @@
         <v>15</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>14</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="E1" s="10" t="s">
         <v>32</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>22</v>
       </c>
       <c r="H1" s="10" t="s">
+        <v>1080</v>
+      </c>
+      <c r="I1" s="10" t="s">
         <v>1081</v>
-      </c>
-      <c r="I1" s="10" t="s">
-        <v>1082</v>
       </c>
       <c r="J1" s="10" t="s">
         <v>10</v>
@@ -46187,10 +46180,10 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>807</v>
@@ -46208,10 +46201,10 @@
         <v>46483.125</v>
       </c>
       <c r="H2" s="0" t="s">
+        <v>1083</v>
+      </c>
+      <c r="I2" s="0" t="s">
         <v>1084</v>
-      </c>
-      <c r="I2" s="0" t="s">
-        <v>1085</v>
       </c>
       <c r="J2" s="0" t="s">
         <v>807</v>
@@ -46219,10 +46212,10 @@
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="C3" s="0" t="s">
         <v>807</v>
@@ -46234,16 +46227,16 @@
         <v>46303</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="G3" s="11">
         <v>46483.125</v>
       </c>
       <c r="H3" s="0" t="s">
+        <v>1083</v>
+      </c>
+      <c r="I3" s="0" t="s">
         <v>1084</v>
-      </c>
-      <c r="I3" s="0" t="s">
-        <v>1085</v>
       </c>
       <c r="J3" s="0" t="s">
         <v>807</v>
@@ -46251,10 +46244,10 @@
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
       <c r="C4" s="0" t="s">
         <v>644</v>
@@ -46272,10 +46265,10 @@
         <v>46480.125</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="J4" s="0" t="s">
         <v>648</v>
@@ -46283,10 +46276,10 @@
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
       <c r="C5" s="0" t="s">
         <v>226</v>
@@ -46304,10 +46297,10 @@
         <v>46476.125</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
       <c r="I5" s="0" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="J5" s="0" t="s">
         <v>226</v>
@@ -46315,10 +46308,10 @@
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
       <c r="C6" s="0" t="s">
         <v>226</v>
@@ -46330,16 +46323,16 @@
         <v>46296</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="G6" s="11">
         <v>46476.125</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
       <c r="I6" s="0" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="J6" s="0" t="s">
         <v>226</v>
@@ -46347,10 +46340,10 @@
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="C7" s="0" t="s">
         <v>34</v>
@@ -46368,10 +46361,10 @@
         <v>46474.125</v>
       </c>
       <c r="H7" s="0" t="s">
+        <v>1091</v>
+      </c>
+      <c r="I7" s="0" t="s">
         <v>1092</v>
-      </c>
-      <c r="I7" s="0" t="s">
-        <v>1093</v>
       </c>
       <c r="J7" s="0" t="s">
         <v>205</v>
@@ -46379,10 +46372,10 @@
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="C8" s="0" t="s">
         <v>34</v>
@@ -46400,10 +46393,10 @@
         <v>46474.125</v>
       </c>
       <c r="H8" s="0" t="s">
+        <v>1091</v>
+      </c>
+      <c r="I8" s="0" t="s">
         <v>1092</v>
-      </c>
-      <c r="I8" s="0" t="s">
-        <v>1093</v>
       </c>
       <c r="J8" s="0" t="s">
         <v>205</v>
@@ -46411,10 +46404,10 @@
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
       <c r="C9" s="0" t="s">
         <v>644</v>
@@ -46432,10 +46425,10 @@
         <v>46474.125</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="I9" s="0" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="J9" s="0" t="s">
         <v>648</v>
@@ -46443,10 +46436,10 @@
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
       <c r="C10" s="0" t="s">
         <v>644</v>
@@ -46458,16 +46451,16 @@
         <v>46294</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="G10" s="11">
         <v>46474.125</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="I10" s="0" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="J10" s="0" t="s">
         <v>648</v>
@@ -46478,7 +46471,7 @@
         <v>842</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
       <c r="C11" s="0" t="s">
         <v>644</v>
@@ -46496,10 +46489,10 @@
         <v>46474.125</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="I11" s="0" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="J11" s="0" t="s">
         <v>648</v>
@@ -46510,7 +46503,7 @@
         <v>842</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
       <c r="C12" s="0" t="s">
         <v>644</v>
@@ -46522,16 +46515,16 @@
         <v>46294</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="G12" s="11">
         <v>46474.125</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="I12" s="0" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="J12" s="0" t="s">
         <v>648</v>
@@ -46539,10 +46532,10 @@
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
       <c r="C13" s="0" t="s">
         <v>60</v>
@@ -46554,16 +46547,16 @@
         <v>46289</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="G13" s="11">
         <v>46469.125</v>
       </c>
       <c r="H13" s="0" t="s">
+        <v>1097</v>
+      </c>
+      <c r="I13" s="0" t="s">
         <v>1098</v>
-      </c>
-      <c r="I13" s="0" t="s">
-        <v>1099</v>
       </c>
       <c r="J13" s="0" t="s">
         <v>66</v>
@@ -46571,10 +46564,10 @@
     </row>
     <row r="14">
       <c r="A14" s="0" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
       <c r="C14" s="0" t="s">
         <v>60</v>
@@ -46592,10 +46585,10 @@
         <v>46469.125</v>
       </c>
       <c r="H14" s="0" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="I14" s="0" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="J14" s="0" t="s">
         <v>66</v>
@@ -46603,10 +46596,10 @@
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>1101</v>
+        <v>1100</v>
       </c>
       <c r="C15" s="0" t="s">
         <v>644</v>
@@ -46624,10 +46617,10 @@
         <v>46455.125</v>
       </c>
       <c r="H15" s="0" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="I15" s="0" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="J15" s="0" t="s">
         <v>648</v>
@@ -46635,10 +46628,10 @@
     </row>
     <row r="16">
       <c r="A16" s="0" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>1101</v>
+        <v>1100</v>
       </c>
       <c r="C16" s="0" t="s">
         <v>644</v>
@@ -46650,16 +46643,16 @@
         <v>46275</v>
       </c>
       <c r="F16" s="0" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="G16" s="11">
         <v>46455.125</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="I16" s="0" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="J16" s="0" t="s">
         <v>648</v>
@@ -46667,13 +46660,13 @@
     </row>
     <row r="17">
       <c r="A17" s="0" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="D17" s="0" t="s">
         <v>30</v>
@@ -46688,24 +46681,24 @@
         <v>46449.125</v>
       </c>
       <c r="H17" s="0" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="I17" s="0" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="J17" s="0" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="D18" s="0" t="s">
         <v>29</v>
@@ -46714,30 +46707,30 @@
         <v>46269</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="G18" s="11">
         <v>46449.125</v>
       </c>
       <c r="H18" s="0" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="I18" s="0" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="J18" s="0" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="D19" s="0" t="s">
         <v>30</v>
@@ -46752,13 +46745,13 @@
         <v>46268</v>
       </c>
       <c r="H19" s="0" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="I19" s="0" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="J19" s="0" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
     </row>
     <row r="20">
@@ -46766,7 +46759,7 @@
         <v>551</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
       <c r="C20" s="0" t="s">
         <v>34</v>
@@ -46778,19 +46771,19 @@
         <v>46267</v>
       </c>
       <c r="F20" s="0" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="G20" s="11">
         <v>46447.125</v>
       </c>
       <c r="H20" s="0" t="s">
+        <v>1097</v>
+      </c>
+      <c r="I20" s="0" t="s">
         <v>1098</v>
       </c>
-      <c r="I20" s="0" t="s">
-        <v>1099</v>
-      </c>
       <c r="J20" s="0" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="21">
@@ -46798,7 +46791,7 @@
         <v>551</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
       <c r="C21" s="0" t="s">
         <v>34</v>
@@ -46816,21 +46809,21 @@
         <v>46447.125</v>
       </c>
       <c r="H21" s="0" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="I21" s="0" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="J21" s="0" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
       <c r="C22" s="0" t="s">
         <v>60</v>
@@ -46848,10 +46841,10 @@
         <v>46446.125</v>
       </c>
       <c r="H22" s="0" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="I22" s="0" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="J22" s="0" t="s">
         <v>610</v>
@@ -46859,10 +46852,10 @@
     </row>
     <row r="23">
       <c r="A23" s="0" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
       <c r="C23" s="0" t="s">
         <v>60</v>
@@ -46880,10 +46873,10 @@
         <v>46446.125</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="I23" s="0" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="J23" s="0" t="s">
         <v>610</v>
@@ -46894,7 +46887,7 @@
         <v>553</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="C24" s="0" t="s">
         <v>48</v>
@@ -46906,27 +46899,27 @@
         <v>46261</v>
       </c>
       <c r="F24" s="0" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="G24" s="11">
         <v>46441.125</v>
       </c>
       <c r="H24" s="0" t="s">
+        <v>1107</v>
+      </c>
+      <c r="I24" s="0" t="s">
+        <v>1098</v>
+      </c>
+      <c r="J24" s="0" t="s">
         <v>1108</v>
-      </c>
-      <c r="I24" s="0" t="s">
-        <v>1099</v>
-      </c>
-      <c r="J24" s="0" t="s">
-        <v>1109</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
       <c r="C25" s="0" t="s">
         <v>34</v>
@@ -46938,16 +46931,16 @@
         <v>46260</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="G25" s="11">
         <v>46440.125</v>
       </c>
       <c r="H25" s="0" t="s">
+        <v>1097</v>
+      </c>
+      <c r="I25" s="0" t="s">
         <v>1098</v>
-      </c>
-      <c r="I25" s="0" t="s">
-        <v>1099</v>
       </c>
       <c r="J25" s="0" t="s">
         <v>205</v>
@@ -46955,10 +46948,10 @@
     </row>
     <row r="26">
       <c r="A26" s="0" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="C26" s="0" t="s">
         <v>60</v>
@@ -46976,10 +46969,10 @@
         <v>46440.125</v>
       </c>
       <c r="H26" s="0" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="I26" s="0" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="J26" s="0" t="s">
         <v>66</v>
@@ -46987,10 +46980,10 @@
     </row>
     <row r="27">
       <c r="A27" s="0" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="C27" s="0" t="s">
         <v>34</v>
@@ -47008,10 +47001,10 @@
         <v>46439.125</v>
       </c>
       <c r="H27" s="0" t="s">
+        <v>1091</v>
+      </c>
+      <c r="I27" s="0" t="s">
         <v>1092</v>
-      </c>
-      <c r="I27" s="0" t="s">
-        <v>1093</v>
       </c>
       <c r="J27" s="0" t="s">
         <v>205</v>
@@ -47022,7 +47015,7 @@
         <v>657</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="C28" s="0" t="s">
         <v>34</v>
@@ -47040,10 +47033,10 @@
         <v>46439.125</v>
       </c>
       <c r="H28" s="0" t="s">
+        <v>1091</v>
+      </c>
+      <c r="I28" s="0" t="s">
         <v>1092</v>
-      </c>
-      <c r="I28" s="0" t="s">
-        <v>1093</v>
       </c>
       <c r="J28" s="0" t="s">
         <v>205</v>
@@ -47051,10 +47044,10 @@
     </row>
     <row r="29">
       <c r="A29" s="0" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
       <c r="C29" s="0" t="s">
         <v>34</v>
@@ -47072,10 +47065,10 @@
         <v>46439.125</v>
       </c>
       <c r="H29" s="0" t="s">
+        <v>1091</v>
+      </c>
+      <c r="I29" s="0" t="s">
         <v>1092</v>
-      </c>
-      <c r="I29" s="0" t="s">
-        <v>1093</v>
       </c>
       <c r="J29" s="0" t="s">
         <v>205</v>
@@ -47086,7 +47079,7 @@
         <v>653</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="C30" s="0" t="s">
         <v>60</v>
@@ -47104,10 +47097,10 @@
         <v>46439.125</v>
       </c>
       <c r="H30" s="0" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="I30" s="0" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="J30" s="0" t="s">
         <v>610</v>
@@ -47118,7 +47111,7 @@
         <v>342</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="C31" s="0" t="s">
         <v>60</v>
@@ -47136,10 +47129,10 @@
         <v>46439.125</v>
       </c>
       <c r="H31" s="0" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="I31" s="0" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="J31" s="0" t="s">
         <v>66</v>
@@ -47150,7 +47143,7 @@
         <v>472</v>
       </c>
       <c r="B32" s="0" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
       <c r="C32" s="0" t="s">
         <v>60</v>
@@ -47162,16 +47155,16 @@
         <v>46255</v>
       </c>
       <c r="F32" s="0" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="G32" s="11">
         <v>46435.125</v>
       </c>
       <c r="H32" s="0" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="I32" s="0" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
       <c r="J32" s="0" t="s">
         <v>66</v>
@@ -47182,7 +47175,7 @@
         <v>472</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
       <c r="C33" s="0" t="s">
         <v>60</v>
@@ -47200,10 +47193,10 @@
         <v>46435.125</v>
       </c>
       <c r="H33" s="0" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="I33" s="0" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="J33" s="0" t="s">
         <v>66</v>
@@ -47214,7 +47207,7 @@
         <v>651</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
       <c r="C34" s="0" t="s">
         <v>60</v>
@@ -47232,10 +47225,10 @@
         <v>46432.125</v>
       </c>
       <c r="H34" s="0" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="I34" s="0" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="J34" s="0" t="s">
         <v>610</v>
@@ -47246,7 +47239,7 @@
         <v>608</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
       <c r="C35" s="0" t="s">
         <v>60</v>
@@ -47264,10 +47257,10 @@
         <v>46432.125</v>
       </c>
       <c r="H35" s="0" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="I35" s="0" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="J35" s="0" t="s">
         <v>610</v>
@@ -47278,7 +47271,7 @@
         <v>607</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
       <c r="C36" s="0" t="s">
         <v>34</v>
@@ -47296,10 +47289,10 @@
         <v>46432.125</v>
       </c>
       <c r="H36" s="0" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="I36" s="0" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="J36" s="0" t="s">
         <v>45</v>
@@ -47307,10 +47300,10 @@
     </row>
     <row r="37">
       <c r="A37" s="0" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="C37" s="0" t="s">
         <v>34</v>
@@ -47328,10 +47321,10 @@
         <v>46432.125</v>
       </c>
       <c r="H37" s="0" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="I37" s="0" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="J37" s="0" t="s">
         <v>45</v>
@@ -47342,7 +47335,7 @@
         <v>607</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
       <c r="C38" s="0" t="s">
         <v>34</v>
@@ -47354,16 +47347,16 @@
         <v>46252</v>
       </c>
       <c r="F38" s="0" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="G38" s="11">
         <v>46432.125</v>
       </c>
       <c r="H38" s="0" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="I38" s="0" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
       <c r="J38" s="0" t="s">
         <v>45</v>
@@ -47371,10 +47364,10 @@
     </row>
     <row r="39">
       <c r="A39" s="0" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="C39" s="0" t="s">
         <v>48</v>
@@ -47386,16 +47379,16 @@
         <v>46251</v>
       </c>
       <c r="F39" s="0" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="G39" s="11">
         <v>46431.125</v>
       </c>
       <c r="H39" s="0" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="I39" s="0" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
       <c r="J39" s="0" t="s">
         <v>56</v>
@@ -47403,10 +47396,10 @@
     </row>
     <row r="40">
       <c r="A40" s="0" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="C40" s="0" t="s">
         <v>48</v>
@@ -47424,10 +47417,10 @@
         <v>46431.125</v>
       </c>
       <c r="H40" s="0" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="I40" s="0" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="J40" s="0" t="s">
         <v>56</v>
@@ -47435,10 +47428,10 @@
     </row>
     <row r="41">
       <c r="A41" s="0" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="C41" s="0" t="s">
         <v>48</v>
@@ -47456,10 +47449,10 @@
         <v>46431.125</v>
       </c>
       <c r="H41" s="0" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="I41" s="0" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="J41" s="0" t="s">
         <v>56</v>

</xml_diff>

<commit_message>
Atualiza dados — extração 15/10/2026 09:34 (via painel)
</commit_message>
<xml_diff>
--- a/dados/prontuario-equipamentos_1.xlsx
+++ b/dados/prontuario-equipamentos_1.xlsx
@@ -3570,7 +3570,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3">
-        <v>46310.34958142361</v>
+        <v>46310.39970675926</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -8562,7 +8562,7 @@
         <v>39</v>
       </c>
       <c r="J59" s="11">
-        <v>46310.125</v>
+        <v>46399.125</v>
       </c>
       <c r="K59" s="0" t="s">
         <v>55</v>
@@ -8577,7 +8577,7 @@
         <v>42</v>
       </c>
       <c r="O59" s="11">
-        <v>46310.125</v>
+        <v>46675.125</v>
       </c>
       <c r="Q59" s="0" t="s">
         <v>42</v>
@@ -35146,7 +35146,7 @@
         <v>832</v>
       </c>
       <c r="J370" s="11">
-        <v>46310.125</v>
+        <v>46392.125</v>
       </c>
       <c r="K370" s="0" t="s">
         <v>55</v>
@@ -35161,7 +35161,7 @@
         <v>42</v>
       </c>
       <c r="O370" s="11">
-        <v>46310.125</v>
+        <v>46675.125</v>
       </c>
       <c r="Q370" s="0" t="s">
         <v>42</v>

</xml_diff>

<commit_message>
Atualiza dados — extração 16/10/2026 15:01 (via painel)
</commit_message>
<xml_diff>
--- a/dados/prontuario-equipamentos_1.xlsx
+++ b/dados/prontuario-equipamentos_1.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1114" uniqueCount="1114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1115" uniqueCount="1115">
   <si>
     <t>Geração:</t>
   </si>
@@ -3246,22 +3246,25 @@
     <t>Perfil Responsável</t>
   </si>
   <si>
+    <t>Volkswagen / VW/19.330 CTC 4X2</t>
+  </si>
+  <si>
+    <t>MACAE BRUNE GOMES MELO</t>
+  </si>
+  <si>
+    <t>Transportador Fixo</t>
+  </si>
+  <si>
     <t>M.BENZ/ATEGO 2426 / M.BENZ/ATEGO 2426</t>
   </si>
   <si>
     <t>WANDERSON DE CARVALHO ROCHA</t>
   </si>
   <si>
-    <t>Transportador Fixo</t>
-  </si>
-  <si>
     <t>Checklist de Qualidade Tomate</t>
   </si>
   <si>
     <t>IVECO / IVECO/STRALIS 600S44T</t>
-  </si>
-  <si>
-    <t>MACAE BRUNE GOMES MELO</t>
   </si>
   <si>
     <t>M.BENZ / L 1113</t>
@@ -3546,7 +3549,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3">
-        <v>46311.34984981482</v>
+        <v>46311.62612400463</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -28850,13 +28853,13 @@
         <v>716</v>
       </c>
       <c r="J298" s="11">
-        <v>46338.125</v>
+        <v>46372.125</v>
       </c>
       <c r="K298" s="0" t="s">
-        <v>76</v>
+        <v>56</v>
       </c>
       <c r="L298" s="0" t="s">
-        <v>207</v>
+        <v>39</v>
       </c>
       <c r="M298" s="0" t="s">
         <v>39</v>
@@ -28871,7 +28874,7 @@
         <v>43</v>
       </c>
       <c r="R298" s="11">
-        <v>46338.125</v>
+        <v>46493.125</v>
       </c>
       <c r="T298" s="0" t="s">
         <v>44</v>
@@ -34048,7 +34051,7 @@
         <v>210</v>
       </c>
       <c r="J359" s="11">
-        <v>46341.125</v>
+        <v>46372.125</v>
       </c>
       <c r="K359" s="0" t="s">
         <v>56</v>
@@ -34063,13 +34066,13 @@
         <v>43</v>
       </c>
       <c r="O359" s="11">
-        <v>46341.125</v>
+        <v>46706.125</v>
       </c>
       <c r="Q359" s="0" t="s">
         <v>43</v>
       </c>
       <c r="R359" s="11">
-        <v>46382.125</v>
+        <v>46493.125</v>
       </c>
       <c r="T359" s="0" t="s">
         <v>44</v>
@@ -35484,7 +35487,7 @@
         <v>76</v>
       </c>
       <c r="L376" s="0" t="s">
-        <v>650</v>
+        <v>77</v>
       </c>
       <c r="M376" s="0" t="s">
         <v>39</v>
@@ -35499,7 +35502,7 @@
         <v>43</v>
       </c>
       <c r="R376" s="11">
-        <v>46338.125</v>
+        <v>46493.125</v>
       </c>
       <c r="T376" s="0" t="s">
         <v>44</v>
@@ -35563,12 +35566,14 @@
       <c r="H377" s="0" t="s">
         <v>716</v>
       </c>
-      <c r="J377" s="11"/>
+      <c r="J377" s="11">
+        <v>46326.125</v>
+      </c>
       <c r="K377" s="0" t="s">
-        <v>40</v>
+        <v>76</v>
       </c>
       <c r="L377" s="0" t="s">
-        <v>682</v>
+        <v>77</v>
       </c>
       <c r="M377" s="0" t="s">
         <v>39</v>
@@ -35583,7 +35588,7 @@
         <v>43</v>
       </c>
       <c r="R377" s="11">
-        <v>46382.125</v>
+        <v>46493.125</v>
       </c>
       <c r="T377" s="0" t="s">
         <v>44</v>
@@ -35613,13 +35618,13 @@
         <v>44</v>
       </c>
       <c r="AH377" s="0" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="AI377" s="3">
-        <v>46129.41428105324</v>
+        <v>46311.44135987268</v>
       </c>
       <c r="AJ377" s="3">
-        <v>46309</v>
+        <v>46491.125</v>
       </c>
     </row>
     <row r="378">
@@ -35737,10 +35742,10 @@
         <v>46341.125</v>
       </c>
       <c r="K379" s="0" t="s">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="L379" s="0" t="s">
-        <v>39</v>
+        <v>77</v>
       </c>
       <c r="M379" s="0" t="s">
         <v>39</v>
@@ -35755,7 +35760,7 @@
         <v>43</v>
       </c>
       <c r="R379" s="11">
-        <v>46360.125</v>
+        <v>46493.125</v>
       </c>
       <c r="T379" s="0" t="s">
         <v>44</v>
@@ -45836,7 +45841,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="16384" width="9.140625" customWidth="1"/>
@@ -45876,25 +45881,25 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>1065</v>
+        <v>841</v>
       </c>
       <c r="B2" s="0" t="s">
         <v>1077</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>804</v>
+        <v>641</v>
       </c>
       <c r="D2" s="0" t="s">
         <v>30</v>
       </c>
       <c r="E2" s="11">
-        <v>46303</v>
+        <v>46311</v>
       </c>
       <c r="F2" s="0" t="s">
         <v>30</v>
       </c>
       <c r="G2" s="11">
-        <v>46483.125</v>
+        <v>46491.125</v>
       </c>
       <c r="H2" s="0" t="s">
         <v>1078</v>
@@ -45903,7 +45908,7 @@
         <v>1079</v>
       </c>
       <c r="J2" s="0" t="s">
-        <v>804</v>
+        <v>645</v>
       </c>
     </row>
     <row r="3">
@@ -45911,25 +45916,25 @@
         <v>1065</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>1077</v>
+        <v>1080</v>
       </c>
       <c r="C3" s="0" t="s">
         <v>804</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E3" s="11">
         <v>46303</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>1080</v>
+        <v>30</v>
       </c>
       <c r="G3" s="11">
         <v>46483.125</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>1078</v>
+        <v>1081</v>
       </c>
       <c r="I3" s="0" t="s">
         <v>1079</v>
@@ -45940,66 +45945,66 @@
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>877</v>
+        <v>1065</v>
       </c>
       <c r="B4" s="0" t="s">
+        <v>1080</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>804</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="11">
+        <v>46303</v>
+      </c>
+      <c r="F4" s="0" t="s">
+        <v>1082</v>
+      </c>
+      <c r="G4" s="11">
+        <v>46483.125</v>
+      </c>
+      <c r="H4" s="0" t="s">
         <v>1081</v>
-      </c>
-      <c r="C4" s="0" t="s">
-        <v>641</v>
-      </c>
-      <c r="D4" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="E4" s="11">
-        <v>46300</v>
-      </c>
-      <c r="F4" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="G4" s="11">
-        <v>46480.125</v>
-      </c>
-      <c r="H4" s="0" t="s">
-        <v>1082</v>
       </c>
       <c r="I4" s="0" t="s">
         <v>1079</v>
       </c>
       <c r="J4" s="0" t="s">
-        <v>645</v>
+        <v>804</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>1064</v>
+        <v>877</v>
       </c>
       <c r="B5" s="0" t="s">
         <v>1083</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>224</v>
+        <v>641</v>
       </c>
       <c r="D5" s="0" t="s">
         <v>30</v>
       </c>
       <c r="E5" s="11">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="F5" s="0" t="s">
         <v>30</v>
       </c>
       <c r="G5" s="11">
-        <v>46476.125</v>
+        <v>46480.125</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>1084</v>
+        <v>1078</v>
       </c>
       <c r="I5" s="0" t="s">
         <v>1079</v>
       </c>
       <c r="J5" s="0" t="s">
-        <v>224</v>
+        <v>645</v>
       </c>
     </row>
     <row r="6">
@@ -46007,25 +46012,25 @@
         <v>1064</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>1083</v>
+        <v>1084</v>
       </c>
       <c r="C6" s="0" t="s">
         <v>224</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E6" s="11">
         <v>46296</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>1080</v>
+        <v>30</v>
       </c>
       <c r="G6" s="11">
         <v>46476.125</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>1084</v>
+        <v>1085</v>
       </c>
       <c r="I6" s="0" t="s">
         <v>1079</v>
@@ -46036,42 +46041,42 @@
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>1060</v>
+        <v>1064</v>
       </c>
       <c r="B7" s="0" t="s">
+        <v>1084</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>224</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" s="11">
+        <v>46296</v>
+      </c>
+      <c r="F7" s="0" t="s">
+        <v>1082</v>
+      </c>
+      <c r="G7" s="11">
+        <v>46476.125</v>
+      </c>
+      <c r="H7" s="0" t="s">
         <v>1085</v>
       </c>
-      <c r="C7" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="D7" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="E7" s="11">
-        <v>46294</v>
-      </c>
-      <c r="F7" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="G7" s="11">
-        <v>46474.125</v>
-      </c>
-      <c r="H7" s="0" t="s">
-        <v>1086</v>
-      </c>
       <c r="I7" s="0" t="s">
-        <v>1087</v>
+        <v>1079</v>
       </c>
       <c r="J7" s="0" t="s">
-        <v>203</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>1063</v>
+        <v>1060</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>1085</v>
+        <v>1086</v>
       </c>
       <c r="C8" s="0" t="s">
         <v>34</v>
@@ -46089,10 +46094,10 @@
         <v>46474.125</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>1086</v>
+        <v>1087</v>
       </c>
       <c r="I8" s="0" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="J8" s="0" t="s">
         <v>203</v>
@@ -46100,13 +46105,13 @@
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>876</v>
+        <v>1063</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>1088</v>
+        <v>1086</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>641</v>
+        <v>34</v>
       </c>
       <c r="D9" s="0" t="s">
         <v>30</v>
@@ -46121,13 +46126,13 @@
         <v>46474.125</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>1082</v>
+        <v>1087</v>
       </c>
       <c r="I9" s="0" t="s">
-        <v>1079</v>
+        <v>1088</v>
       </c>
       <c r="J9" s="0" t="s">
-        <v>645</v>
+        <v>203</v>
       </c>
     </row>
     <row r="10">
@@ -46135,25 +46140,25 @@
         <v>876</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>1088</v>
+        <v>1089</v>
       </c>
       <c r="C10" s="0" t="s">
         <v>641</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E10" s="11">
         <v>46294</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>1080</v>
+        <v>30</v>
       </c>
       <c r="G10" s="11">
         <v>46474.125</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>1082</v>
+        <v>1078</v>
       </c>
       <c r="I10" s="0" t="s">
         <v>1079</v>
@@ -46164,7 +46169,7 @@
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>839</v>
+        <v>876</v>
       </c>
       <c r="B11" s="0" t="s">
         <v>1089</v>
@@ -46173,19 +46178,19 @@
         <v>641</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E11" s="11">
         <v>46294</v>
       </c>
       <c r="F11" s="0" t="s">
-        <v>30</v>
+        <v>1082</v>
       </c>
       <c r="G11" s="11">
         <v>46474.125</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>1082</v>
+        <v>1078</v>
       </c>
       <c r="I11" s="0" t="s">
         <v>1079</v>
@@ -46199,25 +46204,25 @@
         <v>839</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>1089</v>
+        <v>1090</v>
       </c>
       <c r="C12" s="0" t="s">
         <v>641</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E12" s="11">
         <v>46294</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>1080</v>
+        <v>30</v>
       </c>
       <c r="G12" s="11">
         <v>46474.125</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>1082</v>
+        <v>1078</v>
       </c>
       <c r="I12" s="0" t="s">
         <v>1079</v>
@@ -46228,34 +46233,34 @@
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
-        <v>972</v>
+        <v>839</v>
       </c>
       <c r="B13" s="0" t="s">
         <v>1090</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>61</v>
+        <v>641</v>
       </c>
       <c r="D13" s="0" t="s">
         <v>29</v>
       </c>
       <c r="E13" s="11">
-        <v>46289</v>
+        <v>46294</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>1091</v>
+        <v>1082</v>
       </c>
       <c r="G13" s="11">
-        <v>46469.125</v>
+        <v>46474.125</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>1092</v>
+        <v>1078</v>
       </c>
       <c r="I13" s="0" t="s">
-        <v>1093</v>
+        <v>1079</v>
       </c>
       <c r="J13" s="0" t="s">
-        <v>67</v>
+        <v>645</v>
       </c>
     </row>
     <row r="14">
@@ -46263,28 +46268,28 @@
         <v>972</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>1090</v>
+        <v>1091</v>
       </c>
       <c r="C14" s="0" t="s">
         <v>61</v>
       </c>
       <c r="D14" s="0" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E14" s="11">
         <v>46289</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>30</v>
+        <v>1092</v>
       </c>
       <c r="G14" s="11">
         <v>46469.125</v>
       </c>
       <c r="H14" s="0" t="s">
+        <v>1093</v>
+      </c>
+      <c r="I14" s="0" t="s">
         <v>1094</v>
-      </c>
-      <c r="I14" s="0" t="s">
-        <v>1087</v>
       </c>
       <c r="J14" s="0" t="s">
         <v>67</v>
@@ -46292,34 +46297,34 @@
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>1058</v>
+        <v>972</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>1095</v>
+        <v>1091</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>641</v>
+        <v>61</v>
       </c>
       <c r="D15" s="0" t="s">
         <v>30</v>
       </c>
       <c r="E15" s="11">
-        <v>46275</v>
+        <v>46289</v>
       </c>
       <c r="F15" s="0" t="s">
         <v>30</v>
       </c>
       <c r="G15" s="11">
-        <v>46455.125</v>
+        <v>46469.125</v>
       </c>
       <c r="H15" s="0" t="s">
-        <v>1082</v>
+        <v>1095</v>
       </c>
       <c r="I15" s="0" t="s">
-        <v>1079</v>
+        <v>1088</v>
       </c>
       <c r="J15" s="0" t="s">
-        <v>645</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16">
@@ -46327,25 +46332,25 @@
         <v>1058</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="C16" s="0" t="s">
         <v>641</v>
       </c>
       <c r="D16" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E16" s="11">
         <v>46275</v>
       </c>
       <c r="F16" s="0" t="s">
-        <v>1080</v>
+        <v>30</v>
       </c>
       <c r="G16" s="11">
         <v>46455.125</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>1082</v>
+        <v>1078</v>
       </c>
       <c r="I16" s="0" t="s">
         <v>1079</v>
@@ -46356,34 +46361,34 @@
     </row>
     <row r="17">
       <c r="A17" s="0" t="s">
-        <v>848</v>
+        <v>1058</v>
       </c>
       <c r="B17" s="0" t="s">
         <v>1096</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>847</v>
+        <v>641</v>
       </c>
       <c r="D17" s="0" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E17" s="11">
-        <v>46269</v>
+        <v>46275</v>
       </c>
       <c r="F17" s="0" t="s">
-        <v>30</v>
+        <v>1082</v>
       </c>
       <c r="G17" s="11">
-        <v>46449.125</v>
+        <v>46455.125</v>
       </c>
       <c r="H17" s="0" t="s">
-        <v>1097</v>
+        <v>1078</v>
       </c>
       <c r="I17" s="0" t="s">
         <v>1079</v>
       </c>
       <c r="J17" s="0" t="s">
-        <v>849</v>
+        <v>645</v>
       </c>
     </row>
     <row r="18">
@@ -46391,25 +46396,25 @@
         <v>848</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="C18" s="0" t="s">
         <v>847</v>
       </c>
       <c r="D18" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E18" s="11">
         <v>46269</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>1080</v>
+        <v>30</v>
       </c>
       <c r="G18" s="11">
         <v>46449.125</v>
       </c>
       <c r="H18" s="0" t="s">
-        <v>1097</v>
+        <v>1098</v>
       </c>
       <c r="I18" s="0" t="s">
         <v>1079</v>
@@ -46423,25 +46428,25 @@
         <v>848</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="C19" s="0" t="s">
         <v>847</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E19" s="11">
         <v>46269</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>30</v>
+        <v>1082</v>
       </c>
       <c r="G19" s="11">
-        <v>46268</v>
+        <v>46449.125</v>
       </c>
       <c r="H19" s="0" t="s">
-        <v>1097</v>
+        <v>1098</v>
       </c>
       <c r="I19" s="0" t="s">
         <v>1079</v>
@@ -46452,34 +46457,34 @@
     </row>
     <row r="20">
       <c r="A20" s="0" t="s">
-        <v>548</v>
+        <v>848</v>
       </c>
       <c r="B20" s="0" t="s">
+        <v>1097</v>
+      </c>
+      <c r="C20" s="0" t="s">
+        <v>847</v>
+      </c>
+      <c r="D20" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="E20" s="11">
+        <v>46269</v>
+      </c>
+      <c r="F20" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="G20" s="11">
+        <v>46268</v>
+      </c>
+      <c r="H20" s="0" t="s">
         <v>1098</v>
       </c>
-      <c r="C20" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="D20" s="0" t="s">
-        <v>29</v>
-      </c>
-      <c r="E20" s="11">
-        <v>46267</v>
-      </c>
-      <c r="F20" s="0" t="s">
-        <v>1091</v>
-      </c>
-      <c r="G20" s="11">
-        <v>46447.125</v>
-      </c>
-      <c r="H20" s="0" t="s">
-        <v>1092</v>
-      </c>
       <c r="I20" s="0" t="s">
-        <v>1093</v>
+        <v>1079</v>
       </c>
       <c r="J20" s="0" t="s">
-        <v>1099</v>
+        <v>849</v>
       </c>
     </row>
     <row r="21">
@@ -46487,71 +46492,71 @@
         <v>548</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>1098</v>
+        <v>1099</v>
       </c>
       <c r="C21" s="0" t="s">
         <v>34</v>
       </c>
       <c r="D21" s="0" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E21" s="11">
         <v>46267</v>
       </c>
       <c r="F21" s="0" t="s">
-        <v>30</v>
+        <v>1092</v>
       </c>
       <c r="G21" s="11">
         <v>46447.125</v>
       </c>
       <c r="H21" s="0" t="s">
+        <v>1093</v>
+      </c>
+      <c r="I21" s="0" t="s">
         <v>1094</v>
       </c>
-      <c r="I21" s="0" t="s">
-        <v>1087</v>
-      </c>
       <c r="J21" s="0" t="s">
-        <v>1099</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="s">
-        <v>866</v>
+        <v>548</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>61</v>
+        <v>34</v>
       </c>
       <c r="D22" s="0" t="s">
         <v>30</v>
       </c>
       <c r="E22" s="11">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="F22" s="0" t="s">
         <v>30</v>
       </c>
       <c r="G22" s="11">
-        <v>46446.125</v>
+        <v>46447.125</v>
       </c>
       <c r="H22" s="0" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="I22" s="0" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="J22" s="0" t="s">
-        <v>607</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="s">
-        <v>869</v>
+        <v>866</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="C23" s="0" t="s">
         <v>61</v>
@@ -46569,10 +46574,10 @@
         <v>46446.125</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="I23" s="0" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="J23" s="0" t="s">
         <v>607</v>
@@ -46580,138 +46585,138 @@
     </row>
     <row r="24">
       <c r="A24" s="0" t="s">
-        <v>550</v>
+        <v>869</v>
       </c>
       <c r="B24" s="0" t="s">
         <v>1101</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="D24" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E24" s="11">
-        <v>46261</v>
+        <v>46266</v>
       </c>
       <c r="F24" s="0" t="s">
-        <v>1091</v>
+        <v>30</v>
       </c>
       <c r="G24" s="11">
-        <v>46441.125</v>
+        <v>46446.125</v>
       </c>
       <c r="H24" s="0" t="s">
-        <v>1102</v>
+        <v>1095</v>
       </c>
       <c r="I24" s="0" t="s">
-        <v>1093</v>
+        <v>1088</v>
       </c>
       <c r="J24" s="0" t="s">
-        <v>1103</v>
+        <v>607</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="s">
-        <v>865</v>
+        <v>550</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>1104</v>
+        <v>1102</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="D25" s="0" t="s">
         <v>29</v>
       </c>
       <c r="E25" s="11">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="G25" s="11">
-        <v>46440.125</v>
+        <v>46441.125</v>
       </c>
       <c r="H25" s="0" t="s">
-        <v>1092</v>
+        <v>1103</v>
       </c>
       <c r="I25" s="0" t="s">
-        <v>1093</v>
+        <v>1094</v>
       </c>
       <c r="J25" s="0" t="s">
-        <v>203</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="s">
-        <v>1056</v>
+        <v>865</v>
       </c>
       <c r="B26" s="0" t="s">
         <v>1105</v>
       </c>
       <c r="C26" s="0" t="s">
-        <v>61</v>
+        <v>34</v>
       </c>
       <c r="D26" s="0" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E26" s="11">
         <v>46260</v>
       </c>
       <c r="F26" s="0" t="s">
-        <v>30</v>
+        <v>1092</v>
       </c>
       <c r="G26" s="11">
         <v>46440.125</v>
       </c>
       <c r="H26" s="0" t="s">
+        <v>1093</v>
+      </c>
+      <c r="I26" s="0" t="s">
         <v>1094</v>
       </c>
-      <c r="I26" s="0" t="s">
-        <v>1087</v>
-      </c>
       <c r="J26" s="0" t="s">
-        <v>67</v>
+        <v>203</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="0" t="s">
-        <v>864</v>
+        <v>1056</v>
       </c>
       <c r="B27" s="0" t="s">
         <v>1106</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>34</v>
+        <v>61</v>
       </c>
       <c r="D27" s="0" t="s">
         <v>30</v>
       </c>
       <c r="E27" s="11">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="F27" s="0" t="s">
         <v>30</v>
       </c>
       <c r="G27" s="11">
-        <v>46439.125</v>
+        <v>46440.125</v>
       </c>
       <c r="H27" s="0" t="s">
-        <v>1086</v>
+        <v>1095</v>
       </c>
       <c r="I27" s="0" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="J27" s="0" t="s">
-        <v>203</v>
+        <v>67</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="s">
-        <v>655</v>
+        <v>864</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>1106</v>
+        <v>1107</v>
       </c>
       <c r="C28" s="0" t="s">
         <v>34</v>
@@ -46729,10 +46734,10 @@
         <v>46439.125</v>
       </c>
       <c r="H28" s="0" t="s">
-        <v>1086</v>
+        <v>1087</v>
       </c>
       <c r="I28" s="0" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="J28" s="0" t="s">
         <v>203</v>
@@ -46740,10 +46745,10 @@
     </row>
     <row r="29">
       <c r="A29" s="0" t="s">
-        <v>865</v>
+        <v>655</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>1104</v>
+        <v>1107</v>
       </c>
       <c r="C29" s="0" t="s">
         <v>34</v>
@@ -46761,10 +46766,10 @@
         <v>46439.125</v>
       </c>
       <c r="H29" s="0" t="s">
-        <v>1086</v>
+        <v>1087</v>
       </c>
       <c r="I29" s="0" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="J29" s="0" t="s">
         <v>203</v>
@@ -46772,13 +46777,13 @@
     </row>
     <row r="30">
       <c r="A30" s="0" t="s">
-        <v>651</v>
+        <v>865</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>1107</v>
+        <v>1105</v>
       </c>
       <c r="C30" s="0" t="s">
-        <v>61</v>
+        <v>34</v>
       </c>
       <c r="D30" s="0" t="s">
         <v>30</v>
@@ -46793,18 +46798,18 @@
         <v>46439.125</v>
       </c>
       <c r="H30" s="0" t="s">
-        <v>1094</v>
+        <v>1087</v>
       </c>
       <c r="I30" s="0" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="J30" s="0" t="s">
-        <v>607</v>
+        <v>203</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="0" t="s">
-        <v>340</v>
+        <v>651</v>
       </c>
       <c r="B31" s="0" t="s">
         <v>1108</v>
@@ -46825,18 +46830,18 @@
         <v>46439.125</v>
       </c>
       <c r="H31" s="0" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="I31" s="0" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="J31" s="0" t="s">
-        <v>67</v>
+        <v>607</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="0" t="s">
-        <v>470</v>
+        <v>340</v>
       </c>
       <c r="B32" s="0" t="s">
         <v>1109</v>
@@ -46845,22 +46850,22 @@
         <v>61</v>
       </c>
       <c r="D32" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E32" s="11">
-        <v>46255</v>
+        <v>46259</v>
       </c>
       <c r="F32" s="0" t="s">
-        <v>1091</v>
+        <v>30</v>
       </c>
       <c r="G32" s="11">
-        <v>46435.125</v>
+        <v>46439.125</v>
       </c>
       <c r="H32" s="0" t="s">
-        <v>1102</v>
+        <v>1095</v>
       </c>
       <c r="I32" s="0" t="s">
-        <v>1093</v>
+        <v>1088</v>
       </c>
       <c r="J32" s="0" t="s">
         <v>67</v>
@@ -46871,28 +46876,28 @@
         <v>470</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>1109</v>
+        <v>1110</v>
       </c>
       <c r="C33" s="0" t="s">
         <v>61</v>
       </c>
       <c r="D33" s="0" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E33" s="11">
         <v>46255</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>30</v>
+        <v>1092</v>
       </c>
       <c r="G33" s="11">
         <v>46435.125</v>
       </c>
       <c r="H33" s="0" t="s">
+        <v>1103</v>
+      </c>
+      <c r="I33" s="0" t="s">
         <v>1094</v>
-      </c>
-      <c r="I33" s="0" t="s">
-        <v>1087</v>
       </c>
       <c r="J33" s="0" t="s">
         <v>67</v>
@@ -46900,7 +46905,7 @@
     </row>
     <row r="34">
       <c r="A34" s="0" t="s">
-        <v>648</v>
+        <v>470</v>
       </c>
       <c r="B34" s="0" t="s">
         <v>1110</v>
@@ -46912,27 +46917,27 @@
         <v>30</v>
       </c>
       <c r="E34" s="11">
-        <v>46252</v>
+        <v>46255</v>
       </c>
       <c r="F34" s="0" t="s">
         <v>30</v>
       </c>
       <c r="G34" s="11">
-        <v>46432.125</v>
+        <v>46435.125</v>
       </c>
       <c r="H34" s="0" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="I34" s="0" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="J34" s="0" t="s">
-        <v>607</v>
+        <v>67</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="0" t="s">
-        <v>605</v>
+        <v>648</v>
       </c>
       <c r="B35" s="0" t="s">
         <v>1111</v>
@@ -46953,10 +46958,10 @@
         <v>46432.125</v>
       </c>
       <c r="H35" s="0" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="I35" s="0" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="J35" s="0" t="s">
         <v>607</v>
@@ -46964,13 +46969,13 @@
     </row>
     <row r="36">
       <c r="A36" s="0" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="B36" s="0" t="s">
         <v>1112</v>
       </c>
       <c r="C36" s="0" t="s">
-        <v>34</v>
+        <v>61</v>
       </c>
       <c r="D36" s="0" t="s">
         <v>30</v>
@@ -46985,18 +46990,18 @@
         <v>46432.125</v>
       </c>
       <c r="H36" s="0" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="I36" s="0" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="J36" s="0" t="s">
-        <v>46</v>
+        <v>607</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="0" t="s">
-        <v>995</v>
+        <v>604</v>
       </c>
       <c r="B37" s="0" t="s">
         <v>1113</v>
@@ -47017,10 +47022,10 @@
         <v>46432.125</v>
       </c>
       <c r="H37" s="0" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="I37" s="0" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="J37" s="0" t="s">
         <v>46</v>
@@ -47028,33 +47033,65 @@
     </row>
     <row r="38">
       <c r="A38" s="0" t="s">
-        <v>604</v>
+        <v>995</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>1112</v>
+        <v>1114</v>
       </c>
       <c r="C38" s="0" t="s">
         <v>34</v>
       </c>
       <c r="D38" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E38" s="11">
         <v>46252</v>
       </c>
       <c r="F38" s="0" t="s">
-        <v>1091</v>
+        <v>30</v>
       </c>
       <c r="G38" s="11">
         <v>46432.125</v>
       </c>
       <c r="H38" s="0" t="s">
-        <v>1102</v>
+        <v>1095</v>
       </c>
       <c r="I38" s="0" t="s">
-        <v>1093</v>
+        <v>1088</v>
       </c>
       <c r="J38" s="0" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="s">
+        <v>604</v>
+      </c>
+      <c r="B39" s="0" t="s">
+        <v>1113</v>
+      </c>
+      <c r="C39" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="D39" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="E39" s="11">
+        <v>46252</v>
+      </c>
+      <c r="F39" s="0" t="s">
+        <v>1092</v>
+      </c>
+      <c r="G39" s="11">
+        <v>46432.125</v>
+      </c>
+      <c r="H39" s="0" t="s">
+        <v>1103</v>
+      </c>
+      <c r="I39" s="0" t="s">
+        <v>1094</v>
+      </c>
+      <c r="J39" s="0" t="s">
         <v>46</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dados — extração 19/10/2026 14:55 (via painel)
</commit_message>
<xml_diff>
--- a/dados/prontuario-equipamentos_1.xlsx
+++ b/dados/prontuario-equipamentos_1.xlsx
@@ -2634,9 +2634,6 @@
     <t>EGI3E88</t>
   </si>
   <si>
-    <t>Inspeção Checklist de Qualidade pendente / Documento ConsultaCRLV vencendo</t>
-  </si>
-  <si>
     <t>Copel Industria e Comercio de Reciclaveis LTDA</t>
   </si>
   <si>
@@ -3255,6 +3252,18 @@
     <t>Perfil Responsável</t>
   </si>
   <si>
+    <t>SR / IMPERIAL GR000227T0 1</t>
+  </si>
+  <si>
+    <t>Checklist de Qualidade Safra</t>
+  </si>
+  <si>
+    <t>MARCONI BELO SOBRINHO</t>
+  </si>
+  <si>
+    <t>Gestor Heinz</t>
+  </si>
+  <si>
     <t>Volkswagen / VW/19.330 CTC 4X2</t>
   </si>
   <si>
@@ -3300,15 +3309,9 @@
     <t>M. BENZ / L 2013</t>
   </si>
   <si>
-    <t>Checklist de Qualidade Safra</t>
-  </si>
-  <si>
     <t>MARCIO ADRINO GONCALVES</t>
   </si>
   <si>
-    <t>Gestor Heinz</t>
-  </si>
-  <si>
     <t>Denisclea Silva</t>
   </si>
   <si>
@@ -3325,9 +3328,6 @@
   </si>
   <si>
     <t>MILHO | GNOVA TRANSPORTES LTDA;TOMATE | GNOVA TRANSPORTES LTDA</t>
-  </si>
-  <si>
-    <t>SR / IMPERIAL GR000227T0 1</t>
   </si>
   <si>
     <t>SR/IMPERIAL GR000227T0 1 / SR/IMPERIAL GR000227T0 1</t>
@@ -3549,7 +3549,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3">
-        <v>46314.33859302083</v>
+        <v>46314.62248803241</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -36620,12 +36620,14 @@
       <c r="G390" s="0" t="s">
         <v>200</v>
       </c>
-      <c r="J390" s="11"/>
+      <c r="J390" s="11">
+        <v>46326.125</v>
+      </c>
       <c r="K390" s="0" t="s">
-        <v>40</v>
+        <v>114</v>
       </c>
       <c r="L390" s="0" t="s">
-        <v>873</v>
+        <v>206</v>
       </c>
       <c r="M390" s="0" t="s">
         <v>39</v>
@@ -36661,10 +36663,14 @@
         <v>46076.369408252314</v>
       </c>
       <c r="AE390" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="AF390" s="3"/>
-      <c r="AG390" s="3"/>
+        <v>43</v>
+      </c>
+      <c r="AF390" s="3">
+        <v>46314.364552743056</v>
+      </c>
+      <c r="AG390" s="3">
+        <v>46494.125</v>
+      </c>
       <c r="AH390" s="0" t="s">
         <v>43</v>
       </c>
@@ -36680,22 +36686,22 @@
         <v>860</v>
       </c>
       <c r="B391" s="0" t="s">
+        <v>873</v>
+      </c>
+      <c r="C391" s="0" t="s">
         <v>874</v>
-      </c>
-      <c r="C391" s="0" t="s">
-        <v>875</v>
       </c>
       <c r="D391" s="0" t="s">
         <v>587</v>
       </c>
       <c r="E391" s="0" t="s">
+        <v>875</v>
+      </c>
+      <c r="F391" s="0" t="s">
         <v>876</v>
       </c>
-      <c r="F391" s="0" t="s">
-        <v>877</v>
-      </c>
       <c r="G391" s="0" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="J391" s="11">
         <v>46401.125</v>
@@ -36728,7 +36734,7 @@
         <v>45</v>
       </c>
       <c r="AC391" s="0" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="AD391" s="11">
         <v>46104.56253545139</v>
@@ -36760,7 +36766,7 @@
         <v>643</v>
       </c>
       <c r="C392" s="0" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="D392" s="0" t="s">
         <v>109</v>
@@ -36846,7 +36852,7 @@
         <v>643</v>
       </c>
       <c r="C393" s="0" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="D393" s="0" t="s">
         <v>63</v>
@@ -36932,13 +36938,13 @@
         <v>61</v>
       </c>
       <c r="C394" s="0" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="D394" s="0" t="s">
         <v>63</v>
       </c>
       <c r="E394" s="0" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="F394" s="0" t="s">
         <v>60</v>
@@ -36951,7 +36957,7 @@
         <v>40</v>
       </c>
       <c r="L394" s="0" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="M394" s="0" t="s">
         <v>39</v>
@@ -37013,7 +37019,7 @@
         <v>643</v>
       </c>
       <c r="C395" s="0" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="D395" s="0" t="s">
         <v>109</v>
@@ -37035,7 +37041,7 @@
         <v>40</v>
       </c>
       <c r="L395" s="0" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="M395" s="0" t="s">
         <v>39</v>
@@ -37097,7 +37103,7 @@
         <v>34</v>
       </c>
       <c r="C396" s="0" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="D396" s="0" t="s">
         <v>198</v>
@@ -37183,13 +37189,13 @@
         <v>49</v>
       </c>
       <c r="C397" s="0" t="s">
+        <v>886</v>
+      </c>
+      <c r="D397" s="0" t="s">
         <v>887</v>
       </c>
-      <c r="D397" s="0" t="s">
-        <v>888</v>
-      </c>
       <c r="E397" s="0" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="F397" s="0" t="s">
         <v>244</v>
@@ -37198,7 +37204,7 @@
         <v>244</v>
       </c>
       <c r="H397" s="0" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="J397" s="11">
         <v>46413.125</v>
@@ -37269,13 +37275,13 @@
         <v>49</v>
       </c>
       <c r="C398" s="0" t="s">
+        <v>889</v>
+      </c>
+      <c r="D398" s="0" t="s">
         <v>890</v>
       </c>
-      <c r="D398" s="0" t="s">
-        <v>891</v>
-      </c>
       <c r="E398" s="0" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="F398" s="0" t="s">
         <v>53</v>
@@ -37284,7 +37290,7 @@
         <v>54</v>
       </c>
       <c r="H398" s="0" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="J398" s="11">
         <v>46357.125</v>
@@ -37355,7 +37361,7 @@
         <v>34</v>
       </c>
       <c r="C399" s="0" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="D399" s="0" t="s">
         <v>162</v>
@@ -37370,7 +37376,7 @@
         <v>54</v>
       </c>
       <c r="H399" s="0" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="J399" s="11">
         <v>46361.125</v>
@@ -37441,7 +37447,7 @@
         <v>34</v>
       </c>
       <c r="C400" s="0" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="D400" s="0" t="s">
         <v>51</v>
@@ -37456,7 +37462,7 @@
         <v>150</v>
       </c>
       <c r="H400" s="0" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="J400" s="11">
         <v>46365.125</v>
@@ -37527,7 +37533,7 @@
         <v>34</v>
       </c>
       <c r="C401" s="0" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="D401" s="0" t="s">
         <v>51</v>
@@ -37542,7 +37548,7 @@
         <v>134</v>
       </c>
       <c r="H401" s="0" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="J401" s="11">
         <v>46365.125</v>
@@ -37613,7 +37619,7 @@
         <v>34</v>
       </c>
       <c r="C402" s="0" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="D402" s="0" t="s">
         <v>36</v>
@@ -37628,7 +37634,7 @@
         <v>134</v>
       </c>
       <c r="H402" s="0" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="J402" s="11"/>
       <c r="K402" s="0" t="s">
@@ -37697,13 +37703,13 @@
         <v>49</v>
       </c>
       <c r="C403" s="0" t="s">
+        <v>898</v>
+      </c>
+      <c r="D403" s="0" t="s">
         <v>899</v>
       </c>
-      <c r="D403" s="0" t="s">
-        <v>900</v>
-      </c>
       <c r="E403" s="0" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="F403" s="0" t="s">
         <v>54</v>
@@ -37712,7 +37718,7 @@
         <v>54</v>
       </c>
       <c r="H403" s="0" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="J403" s="11">
         <v>46365.125</v>
@@ -37783,7 +37789,7 @@
         <v>49</v>
       </c>
       <c r="C404" s="0" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="D404" s="0" t="s">
         <v>322</v>
@@ -37798,7 +37804,7 @@
         <v>134</v>
       </c>
       <c r="H404" s="0" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="J404" s="11">
         <v>46362.125</v>
@@ -37869,13 +37875,13 @@
         <v>34</v>
       </c>
       <c r="C405" s="0" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="D405" s="0" t="s">
         <v>77</v>
       </c>
       <c r="E405" s="0" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="F405" s="0" t="s">
         <v>65</v>
@@ -37955,7 +37961,7 @@
         <v>34</v>
       </c>
       <c r="C406" s="0" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="D406" s="0" t="s">
         <v>36</v>
@@ -38041,7 +38047,7 @@
         <v>34</v>
       </c>
       <c r="C407" s="0" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="D407" s="0" t="s">
         <v>36</v>
@@ -38127,13 +38133,13 @@
         <v>34</v>
       </c>
       <c r="C408" s="0" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="D408" s="0" t="s">
         <v>77</v>
       </c>
       <c r="E408" s="0" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="F408" s="0" t="s">
         <v>439</v>
@@ -38142,7 +38148,7 @@
         <v>439</v>
       </c>
       <c r="H408" s="0" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="J408" s="11"/>
       <c r="K408" s="0" t="s">
@@ -38211,13 +38217,13 @@
         <v>34</v>
       </c>
       <c r="C409" s="0" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="D409" s="0" t="s">
         <v>72</v>
       </c>
       <c r="E409" s="0" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="F409" s="0" t="s">
         <v>134</v>
@@ -38226,7 +38232,7 @@
         <v>134</v>
       </c>
       <c r="H409" s="0" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="J409" s="11"/>
       <c r="K409" s="0" t="s">
@@ -38295,7 +38301,7 @@
         <v>34</v>
       </c>
       <c r="C410" s="0" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="D410" s="0" t="s">
         <v>72</v>
@@ -38382,7 +38388,7 @@
         <v>34</v>
       </c>
       <c r="C411" s="0" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="D411" s="0" t="s">
         <v>51</v>
@@ -38397,7 +38403,7 @@
         <v>339</v>
       </c>
       <c r="H411" s="0" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="J411" s="11">
         <v>46356.125</v>
@@ -38471,13 +38477,13 @@
         <v>34</v>
       </c>
       <c r="C412" s="0" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="D412" s="0" t="s">
         <v>140</v>
       </c>
       <c r="E412" s="0" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="F412" s="0" t="s">
         <v>142</v>
@@ -38486,7 +38492,7 @@
         <v>142</v>
       </c>
       <c r="H412" s="0" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="J412" s="11"/>
       <c r="K412" s="0" t="s">
@@ -38558,13 +38564,13 @@
         <v>34</v>
       </c>
       <c r="C413" s="0" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="D413" s="0" t="s">
         <v>162</v>
       </c>
       <c r="E413" s="0" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="F413" s="0" t="s">
         <v>93</v>
@@ -38573,7 +38579,7 @@
         <v>93</v>
       </c>
       <c r="H413" s="0" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="J413" s="11"/>
       <c r="K413" s="0" t="s">
@@ -38645,7 +38651,7 @@
         <v>34</v>
       </c>
       <c r="C414" s="0" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="D414" s="0" t="s">
         <v>123</v>
@@ -38660,7 +38666,7 @@
         <v>60</v>
       </c>
       <c r="H414" s="0" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="J414" s="11"/>
       <c r="K414" s="0" t="s">
@@ -38729,7 +38735,7 @@
         <v>34</v>
       </c>
       <c r="C415" s="0" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="D415" s="0" t="s">
         <v>123</v>
@@ -38744,7 +38750,7 @@
         <v>60</v>
       </c>
       <c r="H415" s="0" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="J415" s="11"/>
       <c r="K415" s="0" t="s">
@@ -38813,13 +38819,13 @@
         <v>49</v>
       </c>
       <c r="C416" s="0" t="s">
+        <v>922</v>
+      </c>
+      <c r="D416" s="0" t="s">
         <v>923</v>
       </c>
-      <c r="D416" s="0" t="s">
-        <v>924</v>
-      </c>
       <c r="E416" s="0" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="F416" s="0" t="s">
         <v>200</v>
@@ -38896,7 +38902,7 @@
         <v>34</v>
       </c>
       <c r="C417" s="0" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="D417" s="0" t="s">
         <v>63</v>
@@ -38982,7 +38988,7 @@
         <v>34</v>
       </c>
       <c r="C418" s="0" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="D418" s="0" t="s">
         <v>36</v>
@@ -38997,14 +39003,14 @@
         <v>38</v>
       </c>
       <c r="H418" s="0" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="J418" s="11"/>
       <c r="K418" s="0" t="s">
         <v>40</v>
       </c>
       <c r="L418" s="0" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="M418" s="0" t="s">
         <v>39</v>
@@ -39069,7 +39075,7 @@
         <v>34</v>
       </c>
       <c r="C419" s="0" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="D419" s="0" t="s">
         <v>36</v>
@@ -39084,14 +39090,14 @@
         <v>38</v>
       </c>
       <c r="H419" s="0" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="J419" s="11"/>
       <c r="K419" s="0" t="s">
         <v>40</v>
       </c>
       <c r="L419" s="0" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="M419" s="0" t="s">
         <v>39</v>
@@ -39156,13 +39162,13 @@
         <v>49</v>
       </c>
       <c r="C420" s="0" t="s">
+        <v>929</v>
+      </c>
+      <c r="D420" s="0" t="s">
         <v>930</v>
       </c>
-      <c r="D420" s="0" t="s">
-        <v>931</v>
-      </c>
       <c r="E420" s="0" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="F420" s="0" t="s">
         <v>65</v>
@@ -39239,7 +39245,7 @@
         <v>49</v>
       </c>
       <c r="C421" s="0" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="D421" s="0" t="s">
         <v>322</v>
@@ -39322,13 +39328,13 @@
         <v>34</v>
       </c>
       <c r="C422" s="0" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="D422" s="0" t="s">
         <v>315</v>
       </c>
       <c r="E422" s="0" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="F422" s="0" t="s">
         <v>93</v>
@@ -39337,14 +39343,14 @@
         <v>38</v>
       </c>
       <c r="H422" s="0" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="J422" s="11"/>
       <c r="K422" s="0" t="s">
         <v>40</v>
       </c>
       <c r="L422" s="0" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="M422" s="0" t="s">
         <v>39</v>
@@ -39409,7 +39415,7 @@
         <v>49</v>
       </c>
       <c r="C423" s="0" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="D423" s="0" t="s">
         <v>388</v>
@@ -39492,13 +39498,13 @@
         <v>49</v>
       </c>
       <c r="C424" s="0" t="s">
+        <v>936</v>
+      </c>
+      <c r="D424" s="0" t="s">
         <v>937</v>
       </c>
-      <c r="D424" s="0" t="s">
-        <v>938</v>
-      </c>
       <c r="E424" s="0" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="F424" s="0" t="s">
         <v>150</v>
@@ -39575,7 +39581,7 @@
         <v>61</v>
       </c>
       <c r="C425" s="0" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="D425" s="0" t="s">
         <v>51</v>
@@ -39590,7 +39596,7 @@
         <v>168</v>
       </c>
       <c r="H425" s="0" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="J425" s="11"/>
       <c r="K425" s="0" t="s">
@@ -39659,13 +39665,13 @@
         <v>61</v>
       </c>
       <c r="C426" s="0" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="D426" s="0" t="s">
         <v>77</v>
       </c>
       <c r="E426" s="0" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="F426" s="0" t="s">
         <v>332</v>
@@ -39674,7 +39680,7 @@
         <v>332</v>
       </c>
       <c r="H426" s="0" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="J426" s="11">
         <v>46373.125</v>
@@ -39745,7 +39751,7 @@
         <v>61</v>
       </c>
       <c r="C427" s="0" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="D427" s="0" t="s">
         <v>77</v>
@@ -39760,7 +39766,7 @@
         <v>524</v>
       </c>
       <c r="H427" s="0" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="J427" s="11"/>
       <c r="K427" s="0" t="s">
@@ -39832,13 +39838,13 @@
         <v>61</v>
       </c>
       <c r="C428" s="0" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="D428" s="0" t="s">
         <v>162</v>
       </c>
       <c r="E428" s="0" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="F428" s="0" t="s">
         <v>169</v>
@@ -39921,7 +39927,7 @@
         <v>61</v>
       </c>
       <c r="C429" s="0" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="D429" s="0" t="s">
         <v>77</v>
@@ -39936,7 +39942,7 @@
         <v>54</v>
       </c>
       <c r="H429" s="0" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="J429" s="11">
         <v>46373.125</v>
@@ -40007,13 +40013,13 @@
         <v>61</v>
       </c>
       <c r="C430" s="0" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="D430" s="0" t="s">
         <v>162</v>
       </c>
       <c r="E430" s="0" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="F430" s="0" t="s">
         <v>258</v>
@@ -40022,7 +40028,7 @@
         <v>258</v>
       </c>
       <c r="H430" s="0" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="J430" s="11"/>
       <c r="K430" s="0" t="s">
@@ -40091,7 +40097,7 @@
         <v>61</v>
       </c>
       <c r="C431" s="0" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="D431" s="0" t="s">
         <v>51</v>
@@ -40106,7 +40112,7 @@
         <v>150</v>
       </c>
       <c r="H431" s="0" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="J431" s="11">
         <v>46373.125</v>
@@ -40177,13 +40183,13 @@
         <v>61</v>
       </c>
       <c r="C432" s="0" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="D432" s="0" t="s">
         <v>731</v>
       </c>
       <c r="E432" s="0" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="F432" s="0" t="s">
         <v>209</v>
@@ -40261,7 +40267,7 @@
         <v>61</v>
       </c>
       <c r="C433" s="0" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="D433" s="0" t="s">
         <v>250</v>
@@ -40276,7 +40282,7 @@
         <v>327</v>
       </c>
       <c r="H433" s="0" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="J433" s="11"/>
       <c r="K433" s="0" t="s">
@@ -40345,7 +40351,7 @@
         <v>61</v>
       </c>
       <c r="C434" s="0" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="D434" s="0" t="s">
         <v>260</v>
@@ -40360,7 +40366,7 @@
         <v>93</v>
       </c>
       <c r="H434" s="0" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="J434" s="11"/>
       <c r="K434" s="0" t="s">
@@ -40429,13 +40435,13 @@
         <v>61</v>
       </c>
       <c r="C435" s="0" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="D435" s="0" t="s">
         <v>260</v>
       </c>
       <c r="E435" s="0" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="F435" s="0" t="s">
         <v>168</v>
@@ -40444,7 +40450,7 @@
         <v>168</v>
       </c>
       <c r="H435" s="0" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="J435" s="11"/>
       <c r="K435" s="0" t="s">
@@ -40516,7 +40522,7 @@
         <v>61</v>
       </c>
       <c r="C436" s="0" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="D436" s="0" t="s">
         <v>250</v>
@@ -40603,13 +40609,13 @@
         <v>61</v>
       </c>
       <c r="C437" s="0" t="s">
+        <v>961</v>
+      </c>
+      <c r="D437" s="0" t="s">
         <v>962</v>
       </c>
-      <c r="D437" s="0" t="s">
+      <c r="E437" s="0" t="s">
         <v>963</v>
-      </c>
-      <c r="E437" s="0" t="s">
-        <v>964</v>
       </c>
       <c r="F437" s="0" t="s">
         <v>294</v>
@@ -40689,7 +40695,7 @@
         <v>61</v>
       </c>
       <c r="C438" s="0" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="D438" s="0" t="s">
         <v>260</v>
@@ -40776,7 +40782,7 @@
         <v>61</v>
       </c>
       <c r="C439" s="0" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="D439" s="0" t="s">
         <v>412</v>
@@ -40791,7 +40797,7 @@
         <v>169</v>
       </c>
       <c r="H439" s="0" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="J439" s="11">
         <v>46373.125</v>
@@ -40862,7 +40868,7 @@
         <v>61</v>
       </c>
       <c r="C440" s="0" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
       <c r="D440" s="0" t="s">
         <v>260</v>
@@ -40946,7 +40952,7 @@
         <v>61</v>
       </c>
       <c r="C441" s="0" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="D441" s="0" t="s">
         <v>260</v>
@@ -41030,7 +41036,7 @@
         <v>61</v>
       </c>
       <c r="C442" s="0" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="D442" s="0" t="s">
         <v>412</v>
@@ -41045,7 +41051,7 @@
         <v>327</v>
       </c>
       <c r="H442" s="0" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="J442" s="11">
         <v>46373.125</v>
@@ -41116,7 +41122,7 @@
         <v>61</v>
       </c>
       <c r="C443" s="0" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="D443" s="0" t="s">
         <v>260</v>
@@ -41131,7 +41137,7 @@
         <v>74</v>
       </c>
       <c r="H443" s="0" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="J443" s="11"/>
       <c r="K443" s="0" t="s">
@@ -41200,7 +41206,7 @@
         <v>61</v>
       </c>
       <c r="C444" s="0" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="D444" s="0" t="s">
         <v>260</v>
@@ -41287,7 +41293,7 @@
         <v>61</v>
       </c>
       <c r="C445" s="0" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="D445" s="0" t="s">
         <v>412</v>
@@ -41302,7 +41308,7 @@
         <v>169</v>
       </c>
       <c r="H445" s="0" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="J445" s="11">
         <v>46373.125</v>
@@ -41373,7 +41379,7 @@
         <v>61</v>
       </c>
       <c r="C446" s="0" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="D446" s="0" t="s">
         <v>260</v>
@@ -41457,7 +41463,7 @@
         <v>61</v>
       </c>
       <c r="C447" s="0" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="D447" s="0" t="s">
         <v>162</v>
@@ -41472,7 +41478,7 @@
         <v>176</v>
       </c>
       <c r="H447" s="0" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="J447" s="11"/>
       <c r="K447" s="0" t="s">
@@ -41541,13 +41547,13 @@
         <v>61</v>
       </c>
       <c r="C448" s="0" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="D448" s="0" t="s">
         <v>162</v>
       </c>
       <c r="E448" s="0" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="F448" s="0" t="s">
         <v>502</v>
@@ -41556,7 +41562,7 @@
         <v>502</v>
       </c>
       <c r="H448" s="0" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="J448" s="11">
         <v>46373.125</v>
@@ -41627,7 +41633,7 @@
         <v>61</v>
       </c>
       <c r="C449" s="0" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="D449" s="0" t="s">
         <v>162</v>
@@ -41642,7 +41648,7 @@
         <v>518</v>
       </c>
       <c r="H449" s="0" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="J449" s="11"/>
       <c r="K449" s="0" t="s">
@@ -41711,13 +41717,13 @@
         <v>61</v>
       </c>
       <c r="C450" s="0" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="D450" s="0" t="s">
         <v>162</v>
       </c>
       <c r="E450" s="0" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="F450" s="0" t="s">
         <v>332</v>
@@ -41726,7 +41732,7 @@
         <v>332</v>
       </c>
       <c r="H450" s="0" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="J450" s="11"/>
       <c r="K450" s="0" t="s">
@@ -41798,7 +41804,7 @@
         <v>61</v>
       </c>
       <c r="C451" s="0" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="D451" s="0" t="s">
         <v>162</v>
@@ -41813,7 +41819,7 @@
         <v>332</v>
       </c>
       <c r="H451" s="0" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="J451" s="11"/>
       <c r="K451" s="0" t="s">
@@ -41879,22 +41885,22 @@
         <v>860</v>
       </c>
       <c r="B452" s="0" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="C452" s="0" t="s">
+        <v>986</v>
+      </c>
+      <c r="D452" s="0" t="s">
         <v>987</v>
       </c>
-      <c r="D452" s="0" t="s">
-        <v>988</v>
-      </c>
       <c r="E452" s="0" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="F452" s="0" t="s">
         <v>300</v>
       </c>
       <c r="G452" s="0" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="J452" s="11">
         <v>46383.125</v>
@@ -41927,7 +41933,7 @@
         <v>45</v>
       </c>
       <c r="AC452" s="0" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="AD452" s="11">
         <v>46203.65469700231</v>
@@ -41959,7 +41965,7 @@
         <v>643</v>
       </c>
       <c r="C453" s="0" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="D453" s="0" t="s">
         <v>63</v>
@@ -42045,7 +42051,7 @@
         <v>643</v>
       </c>
       <c r="C454" s="0" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="D454" s="0" t="s">
         <v>770</v>
@@ -42131,13 +42137,13 @@
         <v>34</v>
       </c>
       <c r="C455" s="0" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="D455" s="0" t="s">
         <v>77</v>
       </c>
       <c r="E455" s="0" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="F455" s="0" t="s">
         <v>85</v>
@@ -42214,7 +42220,7 @@
         <v>34</v>
       </c>
       <c r="C456" s="0" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="D456" s="0" t="s">
         <v>36</v>
@@ -42297,7 +42303,7 @@
         <v>34</v>
       </c>
       <c r="C457" s="0" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="D457" s="0" t="s">
         <v>123</v>
@@ -42312,7 +42318,7 @@
         <v>74</v>
       </c>
       <c r="H457" s="0" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="J457" s="11">
         <v>46387.125</v>
@@ -42383,7 +42389,7 @@
         <v>34</v>
       </c>
       <c r="C458" s="0" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="D458" s="0" t="s">
         <v>123</v>
@@ -42398,7 +42404,7 @@
         <v>74</v>
       </c>
       <c r="H458" s="0" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="J458" s="11">
         <v>46326.125</v>
@@ -42469,7 +42475,7 @@
         <v>34</v>
       </c>
       <c r="C459" s="0" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="D459" s="0" t="s">
         <v>51</v>
@@ -42484,7 +42490,7 @@
         <v>326</v>
       </c>
       <c r="H459" s="0" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="J459" s="11">
         <v>46326.125</v>
@@ -42555,13 +42561,13 @@
         <v>34</v>
       </c>
       <c r="C460" s="0" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="D460" s="0" t="s">
         <v>51</v>
       </c>
       <c r="E460" s="0" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
       <c r="F460" s="0" t="s">
         <v>131</v>
@@ -42639,13 +42645,13 @@
         <v>34</v>
       </c>
       <c r="C461" s="0" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="D461" s="0" t="s">
         <v>179</v>
       </c>
       <c r="E461" s="0" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="F461" s="0" t="s">
         <v>149</v>
@@ -42654,7 +42660,7 @@
         <v>149</v>
       </c>
       <c r="H461" s="0" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="J461" s="11"/>
       <c r="K461" s="0" t="s">
@@ -42723,13 +42729,13 @@
         <v>61</v>
       </c>
       <c r="C462" s="0" t="s">
+        <v>1002</v>
+      </c>
+      <c r="D462" s="0" t="s">
         <v>1003</v>
       </c>
-      <c r="D462" s="0" t="s">
+      <c r="E462" s="0" t="s">
         <v>1004</v>
-      </c>
-      <c r="E462" s="0" t="s">
-        <v>1005</v>
       </c>
       <c r="F462" s="0" t="s">
         <v>418</v>
@@ -42738,7 +42744,7 @@
         <v>418</v>
       </c>
       <c r="H462" s="0" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="J462" s="11"/>
       <c r="K462" s="0" t="s">
@@ -42804,7 +42810,7 @@
         <v>61</v>
       </c>
       <c r="C463" s="0" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="D463" s="0" t="s">
         <v>77</v>
@@ -42819,7 +42825,7 @@
         <v>332</v>
       </c>
       <c r="H463" s="0" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="J463" s="11">
         <v>46406.125</v>
@@ -42890,13 +42896,13 @@
         <v>61</v>
       </c>
       <c r="C464" s="0" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="D464" s="0" t="s">
         <v>77</v>
       </c>
       <c r="E464" s="0" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="F464" s="0" t="s">
         <v>79</v>
@@ -42905,7 +42911,7 @@
         <v>232</v>
       </c>
       <c r="H464" s="0" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="J464" s="11">
         <v>46407.125</v>
@@ -42976,7 +42982,7 @@
         <v>61</v>
       </c>
       <c r="C465" s="0" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="D465" s="0" t="s">
         <v>250</v>
@@ -42991,7 +42997,7 @@
         <v>134</v>
       </c>
       <c r="H465" s="0" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="J465" s="11">
         <v>46407.125</v>
@@ -43062,7 +43068,7 @@
         <v>61</v>
       </c>
       <c r="C466" s="0" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="D466" s="0" t="s">
         <v>250</v>
@@ -43077,7 +43083,7 @@
         <v>134</v>
       </c>
       <c r="H466" s="0" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="J466" s="11">
         <v>46407.125</v>
@@ -43148,7 +43154,7 @@
         <v>61</v>
       </c>
       <c r="C467" s="0" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="D467" s="0" t="s">
         <v>770</v>
@@ -43163,7 +43169,7 @@
         <v>54</v>
       </c>
       <c r="H467" s="0" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="J467" s="11">
         <v>46406.125</v>
@@ -43234,7 +43240,7 @@
         <v>61</v>
       </c>
       <c r="C468" s="0" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
       <c r="D468" s="0" t="s">
         <v>260</v>
@@ -43249,7 +43255,7 @@
         <v>74</v>
       </c>
       <c r="H468" s="0" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="J468" s="11">
         <v>46373.125</v>
@@ -43320,7 +43326,7 @@
         <v>49</v>
       </c>
       <c r="C469" s="0" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
       <c r="D469" s="0" t="s">
         <v>51</v>
@@ -43406,13 +43412,13 @@
         <v>227</v>
       </c>
       <c r="C470" s="0" t="s">
+        <v>1017</v>
+      </c>
+      <c r="D470" s="0" t="s">
         <v>1018</v>
       </c>
-      <c r="D470" s="0" t="s">
+      <c r="E470" s="0" t="s">
         <v>1019</v>
-      </c>
-      <c r="E470" s="0" t="s">
-        <v>1020</v>
       </c>
       <c r="F470" s="0" t="s">
         <v>142</v>
@@ -43421,7 +43427,7 @@
         <v>142</v>
       </c>
       <c r="H470" s="0" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="J470" s="11">
         <v>46398.125</v>
@@ -43489,13 +43495,13 @@
         <v>807</v>
       </c>
       <c r="C471" s="0" t="s">
+        <v>1021</v>
+      </c>
+      <c r="D471" s="0" t="s">
         <v>1022</v>
       </c>
-      <c r="D471" s="0" t="s">
+      <c r="E471" s="0" t="s">
         <v>1023</v>
-      </c>
-      <c r="E471" s="0" t="s">
-        <v>1024</v>
       </c>
       <c r="F471" s="0" t="s">
         <v>200</v>
@@ -43534,7 +43540,7 @@
         <v>45</v>
       </c>
       <c r="AC471" s="0" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
       <c r="AD471" s="11">
         <v>46219.55652277778</v>
@@ -43566,7 +43572,7 @@
         <v>49</v>
       </c>
       <c r="C472" s="0" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="D472" s="0" t="s">
         <v>382</v>
@@ -43581,7 +43587,7 @@
         <v>339</v>
       </c>
       <c r="H472" s="0" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="J472" s="11">
         <v>46402.125</v>
@@ -43652,7 +43658,7 @@
         <v>61</v>
       </c>
       <c r="C473" s="0" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="D473" s="0" t="s">
         <v>51</v>
@@ -43667,7 +43673,7 @@
         <v>79</v>
       </c>
       <c r="H473" s="0" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="J473" s="11">
         <v>46346.125</v>
@@ -43738,13 +43744,13 @@
         <v>61</v>
       </c>
       <c r="C474" s="0" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="D474" s="0" t="s">
         <v>250</v>
       </c>
       <c r="E474" s="0" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="F474" s="0" t="s">
         <v>339</v>
@@ -43753,7 +43759,7 @@
         <v>53</v>
       </c>
       <c r="H474" s="0" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="J474" s="11">
         <v>46346.125</v>
@@ -43824,7 +43830,7 @@
         <v>61</v>
       </c>
       <c r="C475" s="0" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="D475" s="0" t="s">
         <v>250</v>
@@ -43839,7 +43845,7 @@
         <v>208</v>
       </c>
       <c r="H475" s="0" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="J475" s="11"/>
       <c r="K475" s="0" t="s">
@@ -43908,7 +43914,7 @@
         <v>61</v>
       </c>
       <c r="C476" s="0" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="D476" s="0" t="s">
         <v>51</v>
@@ -43923,7 +43929,7 @@
         <v>150</v>
       </c>
       <c r="H476" s="0" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="J476" s="11">
         <v>46407.125</v>
@@ -43994,7 +44000,7 @@
         <v>61</v>
       </c>
       <c r="C477" s="0" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="D477" s="0" t="s">
         <v>260</v>
@@ -44009,7 +44015,7 @@
         <v>232</v>
       </c>
       <c r="H477" s="0" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="J477" s="11">
         <v>46407.125</v>
@@ -44080,7 +44086,7 @@
         <v>61</v>
       </c>
       <c r="C478" s="0" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="D478" s="0" t="s">
         <v>260</v>
@@ -44095,7 +44101,7 @@
         <v>232</v>
       </c>
       <c r="H478" s="0" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="J478" s="11">
         <v>46407.125</v>
@@ -44166,7 +44172,7 @@
         <v>621</v>
       </c>
       <c r="C479" s="0" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="D479" s="0" t="s">
         <v>212</v>
@@ -44246,13 +44252,13 @@
         <v>621</v>
       </c>
       <c r="C480" s="0" t="s">
+        <v>1038</v>
+      </c>
+      <c r="D480" s="0" t="s">
         <v>1039</v>
       </c>
-      <c r="D480" s="0" t="s">
-        <v>1040</v>
-      </c>
       <c r="E480" s="0" t="s">
-        <v>1040</v>
+        <v>1039</v>
       </c>
       <c r="F480" s="0" t="s">
         <v>439</v>
@@ -44326,13 +44332,13 @@
         <v>49</v>
       </c>
       <c r="C481" s="0" t="s">
+        <v>1040</v>
+      </c>
+      <c r="D481" s="0" t="s">
         <v>1041</v>
       </c>
-      <c r="D481" s="0" t="s">
-        <v>1042</v>
-      </c>
       <c r="E481" s="0" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="F481" s="0" t="s">
         <v>98</v>
@@ -44412,13 +44418,13 @@
         <v>34</v>
       </c>
       <c r="C482" s="0" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="D482" s="0" t="s">
         <v>77</v>
       </c>
       <c r="E482" s="0" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
       <c r="F482" s="0" t="s">
         <v>38</v>
@@ -44427,7 +44433,7 @@
         <v>38</v>
       </c>
       <c r="H482" s="0" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="J482" s="11"/>
       <c r="K482" s="0" t="s">
@@ -44496,13 +44502,13 @@
         <v>49</v>
       </c>
       <c r="C483" s="0" t="s">
+        <v>1045</v>
+      </c>
+      <c r="D483" s="0" t="s">
         <v>1046</v>
       </c>
-      <c r="D483" s="0" t="s">
-        <v>1047</v>
-      </c>
       <c r="E483" s="0" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="F483" s="0" t="s">
         <v>137</v>
@@ -44579,7 +44585,7 @@
         <v>49</v>
       </c>
       <c r="C484" s="0" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="D484" s="0" t="s">
         <v>345</v>
@@ -44662,7 +44668,7 @@
         <v>49</v>
       </c>
       <c r="C485" s="0" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="D485" s="0" t="s">
         <v>345</v>
@@ -44745,7 +44751,7 @@
         <v>34</v>
       </c>
       <c r="C486" s="0" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="D486" s="0" t="s">
         <v>250</v>
@@ -44760,7 +44766,7 @@
         <v>38</v>
       </c>
       <c r="H486" s="0" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="J486" s="11">
         <v>46362.125</v>
@@ -44831,7 +44837,7 @@
         <v>34</v>
       </c>
       <c r="C487" s="0" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="D487" s="0" t="s">
         <v>250</v>
@@ -44846,7 +44852,7 @@
         <v>38</v>
       </c>
       <c r="H487" s="0" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="J487" s="11">
         <v>46362.125</v>
@@ -44917,7 +44923,7 @@
         <v>49</v>
       </c>
       <c r="C488" s="0" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="D488" s="0" t="s">
         <v>366</v>
@@ -45000,13 +45006,13 @@
         <v>49</v>
       </c>
       <c r="C489" s="0" t="s">
+        <v>1052</v>
+      </c>
+      <c r="D489" s="0" t="s">
         <v>1053</v>
       </c>
-      <c r="D489" s="0" t="s">
-        <v>1054</v>
-      </c>
       <c r="E489" s="0" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="F489" s="0" t="s">
         <v>258</v>
@@ -45083,13 +45089,13 @@
         <v>49</v>
       </c>
       <c r="C490" s="0" t="s">
+        <v>1054</v>
+      </c>
+      <c r="D490" s="0" t="s">
         <v>1055</v>
       </c>
-      <c r="D490" s="0" t="s">
-        <v>1056</v>
-      </c>
       <c r="E490" s="0" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="F490" s="0" t="s">
         <v>131</v>
@@ -45166,13 +45172,13 @@
         <v>49</v>
       </c>
       <c r="C491" s="0" t="s">
+        <v>1056</v>
+      </c>
+      <c r="D491" s="0" t="s">
         <v>1057</v>
       </c>
-      <c r="D491" s="0" t="s">
-        <v>1058</v>
-      </c>
       <c r="E491" s="0" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="F491" s="0" t="s">
         <v>294</v>
@@ -45249,13 +45255,13 @@
         <v>61</v>
       </c>
       <c r="C492" s="0" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="D492" s="0" t="s">
         <v>526</v>
       </c>
       <c r="E492" s="0" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="F492" s="0" t="s">
         <v>105</v>
@@ -45333,13 +45339,13 @@
         <v>643</v>
       </c>
       <c r="C493" s="0" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="D493" s="0" t="s">
         <v>72</v>
       </c>
       <c r="E493" s="0" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="F493" s="0" t="s">
         <v>293</v>
@@ -45419,19 +45425,19 @@
         <v>34</v>
       </c>
       <c r="C494" s="0" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="D494" s="0" t="s">
         <v>587</v>
       </c>
       <c r="E494" s="0" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
       <c r="F494" s="0" t="s">
         <v>863</v>
       </c>
       <c r="G494" s="0" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="H494" s="0" t="s">
         <v>201</v>
@@ -45505,19 +45511,19 @@
         <v>34</v>
       </c>
       <c r="C495" s="0" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="D495" s="0" t="s">
         <v>587</v>
       </c>
       <c r="E495" s="0" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
       <c r="F495" s="0" t="s">
         <v>863</v>
       </c>
       <c r="G495" s="0" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="H495" s="0" t="s">
         <v>201</v>
@@ -45591,7 +45597,7 @@
         <v>227</v>
       </c>
       <c r="C496" s="0" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="D496" s="0" t="s">
         <v>526</v>
@@ -45671,13 +45677,13 @@
         <v>807</v>
       </c>
       <c r="C497" s="0" t="s">
+        <v>1067</v>
+      </c>
+      <c r="D497" s="0" t="s">
         <v>1068</v>
       </c>
-      <c r="D497" s="0" t="s">
-        <v>1069</v>
-      </c>
       <c r="E497" s="0" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="F497" s="0" t="s">
         <v>294</v>
@@ -45745,13 +45751,13 @@
         <v>850</v>
       </c>
       <c r="C498" s="0" t="s">
+        <v>1069</v>
+      </c>
+      <c r="D498" s="0" t="s">
+        <v>937</v>
+      </c>
+      <c r="E498" s="0" t="s">
         <v>1070</v>
-      </c>
-      <c r="D498" s="0" t="s">
-        <v>938</v>
-      </c>
-      <c r="E498" s="0" t="s">
-        <v>1071</v>
       </c>
       <c r="F498" s="0" t="s">
         <v>168</v>
@@ -45764,7 +45770,7 @@
         <v>40</v>
       </c>
       <c r="L498" s="0" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
       <c r="M498" s="0" t="s">
         <v>39</v>
@@ -45812,13 +45818,13 @@
         <v>850</v>
       </c>
       <c r="C499" s="0" t="s">
+        <v>1072</v>
+      </c>
+      <c r="D499" s="0" t="s">
         <v>1073</v>
       </c>
-      <c r="D499" s="0" t="s">
-        <v>1074</v>
-      </c>
       <c r="E499" s="0" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
       <c r="F499" s="0" t="s">
         <v>169</v>
@@ -45831,7 +45837,7 @@
         <v>40</v>
       </c>
       <c r="L499" s="0" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
       <c r="M499" s="0" t="s">
         <v>39</v>
@@ -45907,7 +45913,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="16384" width="9.140625" customWidth="1"/>
@@ -45918,28 +45924,28 @@
         <v>15</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>14</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
       <c r="E1" s="10" t="s">
         <v>32</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>22</v>
       </c>
       <c r="H1" s="10" t="s">
+        <v>1077</v>
+      </c>
+      <c r="I1" s="10" t="s">
         <v>1078</v>
-      </c>
-      <c r="I1" s="10" t="s">
-        <v>1079</v>
       </c>
       <c r="J1" s="10" t="s">
         <v>10</v>
@@ -45947,25 +45953,25 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>844</v>
+        <v>872</v>
       </c>
       <c r="B2" s="0" t="s">
+        <v>1079</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" s="11">
+        <v>46314</v>
+      </c>
+      <c r="F2" s="0" t="s">
         <v>1080</v>
       </c>
-      <c r="C2" s="0" t="s">
-        <v>643</v>
-      </c>
-      <c r="D2" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="E2" s="11">
-        <v>46311</v>
-      </c>
-      <c r="F2" s="0" t="s">
-        <v>30</v>
-      </c>
       <c r="G2" s="11">
-        <v>46491.125</v>
+        <v>46494.125</v>
       </c>
       <c r="H2" s="0" t="s">
         <v>1081</v>
@@ -45974,68 +45980,68 @@
         <v>1082</v>
       </c>
       <c r="J2" s="0" t="s">
-        <v>647</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>1068</v>
+        <v>844</v>
       </c>
       <c r="B3" s="0" t="s">
         <v>1083</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>807</v>
+        <v>643</v>
       </c>
       <c r="D3" s="0" t="s">
         <v>30</v>
       </c>
       <c r="E3" s="11">
-        <v>46303</v>
+        <v>46311</v>
       </c>
       <c r="F3" s="0" t="s">
         <v>30</v>
       </c>
       <c r="G3" s="11">
-        <v>46483.125</v>
+        <v>46491.125</v>
       </c>
       <c r="H3" s="0" t="s">
         <v>1084</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>1082</v>
+        <v>1085</v>
       </c>
       <c r="J3" s="0" t="s">
-        <v>807</v>
+        <v>647</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>1083</v>
+        <v>1086</v>
       </c>
       <c r="C4" s="0" t="s">
         <v>807</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E4" s="11">
         <v>46303</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>1085</v>
+        <v>30</v>
       </c>
       <c r="G4" s="11">
         <v>46483.125</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>1084</v>
+        <v>1087</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>1082</v>
+        <v>1085</v>
       </c>
       <c r="J4" s="0" t="s">
         <v>807</v>
@@ -46043,95 +46049,95 @@
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>880</v>
+        <v>1067</v>
       </c>
       <c r="B5" s="0" t="s">
         <v>1086</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>643</v>
+        <v>807</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E5" s="11">
-        <v>46300</v>
+        <v>46303</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>30</v>
+        <v>1088</v>
       </c>
       <c r="G5" s="11">
-        <v>46480.125</v>
+        <v>46483.125</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>1081</v>
+        <v>1087</v>
       </c>
       <c r="I5" s="0" t="s">
-        <v>1082</v>
+        <v>1085</v>
       </c>
       <c r="J5" s="0" t="s">
-        <v>647</v>
+        <v>807</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>1067</v>
+        <v>879</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>1087</v>
+        <v>1089</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>227</v>
+        <v>643</v>
       </c>
       <c r="D6" s="0" t="s">
         <v>30</v>
       </c>
       <c r="E6" s="11">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="F6" s="0" t="s">
         <v>30</v>
       </c>
       <c r="G6" s="11">
-        <v>46476.125</v>
+        <v>46480.125</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>1088</v>
+        <v>1084</v>
       </c>
       <c r="I6" s="0" t="s">
-        <v>1082</v>
+        <v>1085</v>
       </c>
       <c r="J6" s="0" t="s">
-        <v>227</v>
+        <v>647</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>1087</v>
+        <v>1090</v>
       </c>
       <c r="C7" s="0" t="s">
         <v>227</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E7" s="11">
         <v>46296</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>1085</v>
+        <v>30</v>
       </c>
       <c r="G7" s="11">
         <v>46476.125</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>1088</v>
+        <v>1091</v>
       </c>
       <c r="I7" s="0" t="s">
-        <v>1082</v>
+        <v>1085</v>
       </c>
       <c r="J7" s="0" t="s">
         <v>227</v>
@@ -46139,42 +46145,42 @@
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>1063</v>
+        <v>1066</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>1089</v>
+        <v>1090</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>34</v>
+        <v>227</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E8" s="11">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>30</v>
+        <v>1088</v>
       </c>
       <c r="G8" s="11">
-        <v>46474.125</v>
+        <v>46476.125</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>1090</v>
+        <v>1091</v>
       </c>
       <c r="I8" s="0" t="s">
-        <v>1091</v>
+        <v>1085</v>
       </c>
       <c r="J8" s="0" t="s">
-        <v>202</v>
+        <v>227</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>1066</v>
+        <v>1062</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>1089</v>
+        <v>1092</v>
       </c>
       <c r="C9" s="0" t="s">
         <v>34</v>
@@ -46192,10 +46198,10 @@
         <v>46474.125</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>1090</v>
+        <v>1093</v>
       </c>
       <c r="I9" s="0" t="s">
-        <v>1091</v>
+        <v>1094</v>
       </c>
       <c r="J9" s="0" t="s">
         <v>202</v>
@@ -46203,13 +46209,13 @@
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>879</v>
+        <v>1065</v>
       </c>
       <c r="B10" s="0" t="s">
         <v>1092</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>643</v>
+        <v>34</v>
       </c>
       <c r="D10" s="0" t="s">
         <v>30</v>
@@ -46224,42 +46230,42 @@
         <v>46474.125</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>1081</v>
+        <v>1093</v>
       </c>
       <c r="I10" s="0" t="s">
-        <v>1082</v>
+        <v>1094</v>
       </c>
       <c r="J10" s="0" t="s">
-        <v>647</v>
+        <v>202</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>1092</v>
+        <v>1095</v>
       </c>
       <c r="C11" s="0" t="s">
         <v>643</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E11" s="11">
         <v>46294</v>
       </c>
       <c r="F11" s="0" t="s">
-        <v>1085</v>
+        <v>30</v>
       </c>
       <c r="G11" s="11">
         <v>46474.125</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>1081</v>
+        <v>1084</v>
       </c>
       <c r="I11" s="0" t="s">
-        <v>1082</v>
+        <v>1085</v>
       </c>
       <c r="J11" s="0" t="s">
         <v>647</v>
@@ -46267,31 +46273,31 @@
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>842</v>
+        <v>878</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>1093</v>
+        <v>1095</v>
       </c>
       <c r="C12" s="0" t="s">
         <v>643</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E12" s="11">
         <v>46294</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>30</v>
+        <v>1088</v>
       </c>
       <c r="G12" s="11">
         <v>46474.125</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>1081</v>
+        <v>1084</v>
       </c>
       <c r="I12" s="0" t="s">
-        <v>1082</v>
+        <v>1085</v>
       </c>
       <c r="J12" s="0" t="s">
         <v>647</v>
@@ -46302,28 +46308,28 @@
         <v>842</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>1093</v>
+        <v>1096</v>
       </c>
       <c r="C13" s="0" t="s">
         <v>643</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E13" s="11">
         <v>46294</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>1085</v>
+        <v>30</v>
       </c>
       <c r="G13" s="11">
         <v>46474.125</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>1081</v>
+        <v>1084</v>
       </c>
       <c r="I13" s="0" t="s">
-        <v>1082</v>
+        <v>1085</v>
       </c>
       <c r="J13" s="0" t="s">
         <v>647</v>
@@ -46331,54 +46337,54 @@
     </row>
     <row r="14">
       <c r="A14" s="0" t="s">
-        <v>975</v>
+        <v>842</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>1094</v>
+        <v>1096</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>61</v>
+        <v>643</v>
       </c>
       <c r="D14" s="0" t="s">
         <v>29</v>
       </c>
       <c r="E14" s="11">
-        <v>46289</v>
+        <v>46294</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>1095</v>
+        <v>1088</v>
       </c>
       <c r="G14" s="11">
-        <v>46469.125</v>
+        <v>46474.125</v>
       </c>
       <c r="H14" s="0" t="s">
-        <v>1096</v>
+        <v>1084</v>
       </c>
       <c r="I14" s="0" t="s">
-        <v>1097</v>
+        <v>1085</v>
       </c>
       <c r="J14" s="0" t="s">
-        <v>67</v>
+        <v>647</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>1094</v>
+        <v>1097</v>
       </c>
       <c r="C15" s="0" t="s">
         <v>61</v>
       </c>
       <c r="D15" s="0" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E15" s="11">
         <v>46289</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>30</v>
+        <v>1080</v>
       </c>
       <c r="G15" s="11">
         <v>46469.125</v>
@@ -46387,7 +46393,7 @@
         <v>1098</v>
       </c>
       <c r="I15" s="0" t="s">
-        <v>1091</v>
+        <v>1082</v>
       </c>
       <c r="J15" s="0" t="s">
         <v>67</v>
@@ -46395,63 +46401,63 @@
     </row>
     <row r="16">
       <c r="A16" s="0" t="s">
-        <v>1061</v>
+        <v>974</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>1099</v>
+        <v>1097</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>643</v>
+        <v>61</v>
       </c>
       <c r="D16" s="0" t="s">
         <v>30</v>
       </c>
       <c r="E16" s="11">
-        <v>46275</v>
+        <v>46289</v>
       </c>
       <c r="F16" s="0" t="s">
         <v>30</v>
       </c>
       <c r="G16" s="11">
-        <v>46455.125</v>
+        <v>46469.125</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>1081</v>
+        <v>1099</v>
       </c>
       <c r="I16" s="0" t="s">
-        <v>1082</v>
+        <v>1094</v>
       </c>
       <c r="J16" s="0" t="s">
-        <v>647</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>1099</v>
+        <v>1100</v>
       </c>
       <c r="C17" s="0" t="s">
         <v>643</v>
       </c>
       <c r="D17" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E17" s="11">
         <v>46275</v>
       </c>
       <c r="F17" s="0" t="s">
-        <v>1085</v>
+        <v>30</v>
       </c>
       <c r="G17" s="11">
         <v>46455.125</v>
       </c>
       <c r="H17" s="0" t="s">
-        <v>1081</v>
+        <v>1084</v>
       </c>
       <c r="I17" s="0" t="s">
-        <v>1082</v>
+        <v>1085</v>
       </c>
       <c r="J17" s="0" t="s">
         <v>647</v>
@@ -46459,34 +46465,34 @@
     </row>
     <row r="18">
       <c r="A18" s="0" t="s">
-        <v>851</v>
+        <v>1060</v>
       </c>
       <c r="B18" s="0" t="s">
         <v>1100</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>850</v>
+        <v>643</v>
       </c>
       <c r="D18" s="0" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E18" s="11">
-        <v>46269</v>
+        <v>46275</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>30</v>
+        <v>1088</v>
       </c>
       <c r="G18" s="11">
-        <v>46449.125</v>
+        <v>46455.125</v>
       </c>
       <c r="H18" s="0" t="s">
-        <v>1101</v>
+        <v>1084</v>
       </c>
       <c r="I18" s="0" t="s">
-        <v>1082</v>
+        <v>1085</v>
       </c>
       <c r="J18" s="0" t="s">
-        <v>852</v>
+        <v>647</v>
       </c>
     </row>
     <row r="19">
@@ -46494,28 +46500,28 @@
         <v>851</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="C19" s="0" t="s">
         <v>850</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E19" s="11">
         <v>46269</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>1085</v>
+        <v>30</v>
       </c>
       <c r="G19" s="11">
         <v>46449.125</v>
       </c>
       <c r="H19" s="0" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="I19" s="0" t="s">
-        <v>1082</v>
+        <v>1085</v>
       </c>
       <c r="J19" s="0" t="s">
         <v>852</v>
@@ -46526,28 +46532,28 @@
         <v>851</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="C20" s="0" t="s">
         <v>850</v>
       </c>
       <c r="D20" s="0" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E20" s="11">
         <v>46269</v>
       </c>
       <c r="F20" s="0" t="s">
-        <v>30</v>
+        <v>1088</v>
       </c>
       <c r="G20" s="11">
-        <v>46268</v>
+        <v>46449.125</v>
       </c>
       <c r="H20" s="0" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="I20" s="0" t="s">
-        <v>1082</v>
+        <v>1085</v>
       </c>
       <c r="J20" s="0" t="s">
         <v>852</v>
@@ -46555,34 +46561,34 @@
     </row>
     <row r="21">
       <c r="A21" s="0" t="s">
-        <v>551</v>
+        <v>851</v>
       </c>
       <c r="B21" s="0" t="s">
+        <v>1101</v>
+      </c>
+      <c r="C21" s="0" t="s">
+        <v>850</v>
+      </c>
+      <c r="D21" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="E21" s="11">
+        <v>46269</v>
+      </c>
+      <c r="F21" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="G21" s="11">
+        <v>46268</v>
+      </c>
+      <c r="H21" s="0" t="s">
         <v>1102</v>
       </c>
-      <c r="C21" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="D21" s="0" t="s">
-        <v>29</v>
-      </c>
-      <c r="E21" s="11">
-        <v>46267</v>
-      </c>
-      <c r="F21" s="0" t="s">
-        <v>1095</v>
-      </c>
-      <c r="G21" s="11">
-        <v>46447.125</v>
-      </c>
-      <c r="H21" s="0" t="s">
-        <v>1096</v>
-      </c>
       <c r="I21" s="0" t="s">
-        <v>1097</v>
+        <v>1085</v>
       </c>
       <c r="J21" s="0" t="s">
-        <v>1103</v>
+        <v>852</v>
       </c>
     </row>
     <row r="22">
@@ -46590,19 +46596,19 @@
         <v>551</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="C22" s="0" t="s">
         <v>34</v>
       </c>
       <c r="D22" s="0" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E22" s="11">
         <v>46267</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>30</v>
+        <v>1080</v>
       </c>
       <c r="G22" s="11">
         <v>46447.125</v>
@@ -46611,50 +46617,50 @@
         <v>1098</v>
       </c>
       <c r="I22" s="0" t="s">
-        <v>1091</v>
+        <v>1082</v>
       </c>
       <c r="J22" s="0" t="s">
-        <v>1103</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="s">
-        <v>869</v>
+        <v>551</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>61</v>
+        <v>34</v>
       </c>
       <c r="D23" s="0" t="s">
         <v>30</v>
       </c>
       <c r="E23" s="11">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="F23" s="0" t="s">
         <v>30</v>
       </c>
       <c r="G23" s="11">
-        <v>46446.125</v>
+        <v>46447.125</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>1098</v>
+        <v>1099</v>
       </c>
       <c r="I23" s="0" t="s">
-        <v>1091</v>
+        <v>1094</v>
       </c>
       <c r="J23" s="0" t="s">
-        <v>215</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="s">
-        <v>872</v>
+        <v>869</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>1104</v>
+        <v>1079</v>
       </c>
       <c r="C24" s="0" t="s">
         <v>61</v>
@@ -46672,10 +46678,10 @@
         <v>46446.125</v>
       </c>
       <c r="H24" s="0" t="s">
-        <v>1098</v>
+        <v>1099</v>
       </c>
       <c r="I24" s="0" t="s">
-        <v>1091</v>
+        <v>1094</v>
       </c>
       <c r="J24" s="0" t="s">
         <v>215</v>
@@ -46683,86 +46689,86 @@
     </row>
     <row r="25">
       <c r="A25" s="0" t="s">
-        <v>553</v>
+        <v>872</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>1105</v>
+        <v>1079</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="D25" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E25" s="11">
-        <v>46261</v>
+        <v>46266</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>1095</v>
+        <v>30</v>
       </c>
       <c r="G25" s="11">
-        <v>46441.125</v>
+        <v>46446.125</v>
       </c>
       <c r="H25" s="0" t="s">
-        <v>1106</v>
+        <v>1099</v>
       </c>
       <c r="I25" s="0" t="s">
-        <v>1097</v>
+        <v>1094</v>
       </c>
       <c r="J25" s="0" t="s">
-        <v>1107</v>
+        <v>215</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="s">
-        <v>868</v>
+        <v>553</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>1108</v>
+        <v>1105</v>
       </c>
       <c r="C26" s="0" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="D26" s="0" t="s">
         <v>29</v>
       </c>
       <c r="E26" s="11">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="F26" s="0" t="s">
-        <v>1095</v>
+        <v>1080</v>
       </c>
       <c r="G26" s="11">
-        <v>46440.125</v>
+        <v>46441.125</v>
       </c>
       <c r="H26" s="0" t="s">
-        <v>1096</v>
+        <v>1106</v>
       </c>
       <c r="I26" s="0" t="s">
-        <v>1097</v>
+        <v>1082</v>
       </c>
       <c r="J26" s="0" t="s">
-        <v>202</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="0" t="s">
-        <v>1059</v>
+        <v>868</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>61</v>
+        <v>34</v>
       </c>
       <c r="D27" s="0" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E27" s="11">
         <v>46260</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>30</v>
+        <v>1080</v>
       </c>
       <c r="G27" s="11">
         <v>46440.125</v>
@@ -46771,47 +46777,47 @@
         <v>1098</v>
       </c>
       <c r="I27" s="0" t="s">
-        <v>1091</v>
+        <v>1082</v>
       </c>
       <c r="J27" s="0" t="s">
-        <v>67</v>
+        <v>202</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="s">
-        <v>867</v>
+        <v>1058</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
       <c r="C28" s="0" t="s">
-        <v>34</v>
+        <v>61</v>
       </c>
       <c r="D28" s="0" t="s">
         <v>30</v>
       </c>
       <c r="E28" s="11">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="F28" s="0" t="s">
         <v>30</v>
       </c>
       <c r="G28" s="11">
-        <v>46439.125</v>
+        <v>46440.125</v>
       </c>
       <c r="H28" s="0" t="s">
-        <v>1090</v>
+        <v>1099</v>
       </c>
       <c r="I28" s="0" t="s">
-        <v>1091</v>
+        <v>1094</v>
       </c>
       <c r="J28" s="0" t="s">
-        <v>202</v>
+        <v>67</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="s">
-        <v>657</v>
+        <v>867</v>
       </c>
       <c r="B29" s="0" t="s">
         <v>1110</v>
@@ -46832,10 +46838,10 @@
         <v>46439.125</v>
       </c>
       <c r="H29" s="0" t="s">
-        <v>1090</v>
+        <v>1093</v>
       </c>
       <c r="I29" s="0" t="s">
-        <v>1091</v>
+        <v>1094</v>
       </c>
       <c r="J29" s="0" t="s">
         <v>202</v>
@@ -46843,10 +46849,10 @@
     </row>
     <row r="30">
       <c r="A30" s="0" t="s">
-        <v>868</v>
+        <v>657</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>1108</v>
+        <v>1110</v>
       </c>
       <c r="C30" s="0" t="s">
         <v>34</v>
@@ -46864,10 +46870,10 @@
         <v>46439.125</v>
       </c>
       <c r="H30" s="0" t="s">
-        <v>1090</v>
+        <v>1093</v>
       </c>
       <c r="I30" s="0" t="s">
-        <v>1091</v>
+        <v>1094</v>
       </c>
       <c r="J30" s="0" t="s">
         <v>202</v>
@@ -46875,13 +46881,13 @@
     </row>
     <row r="31">
       <c r="A31" s="0" t="s">
-        <v>653</v>
+        <v>868</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>1111</v>
+        <v>1108</v>
       </c>
       <c r="C31" s="0" t="s">
-        <v>61</v>
+        <v>34</v>
       </c>
       <c r="D31" s="0" t="s">
         <v>30</v>
@@ -46896,21 +46902,21 @@
         <v>46439.125</v>
       </c>
       <c r="H31" s="0" t="s">
-        <v>1098</v>
+        <v>1093</v>
       </c>
       <c r="I31" s="0" t="s">
-        <v>1091</v>
+        <v>1094</v>
       </c>
       <c r="J31" s="0" t="s">
-        <v>215</v>
+        <v>202</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="0" t="s">
-        <v>211</v>
+        <v>653</v>
       </c>
       <c r="B32" s="0" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="C32" s="0" t="s">
         <v>61</v>
@@ -46928,10 +46934,10 @@
         <v>46439.125</v>
       </c>
       <c r="H32" s="0" t="s">
-        <v>1098</v>
+        <v>1099</v>
       </c>
       <c r="I32" s="0" t="s">
-        <v>1091</v>
+        <v>1094</v>
       </c>
       <c r="J32" s="0" t="s">
         <v>215</v>
@@ -46939,10 +46945,10 @@
     </row>
     <row r="33">
       <c r="A33" s="0" t="s">
-        <v>343</v>
+        <v>211</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="C33" s="0" t="s">
         <v>61</v>
@@ -46960,42 +46966,42 @@
         <v>46439.125</v>
       </c>
       <c r="H33" s="0" t="s">
-        <v>1098</v>
+        <v>1099</v>
       </c>
       <c r="I33" s="0" t="s">
-        <v>1091</v>
+        <v>1094</v>
       </c>
       <c r="J33" s="0" t="s">
-        <v>67</v>
+        <v>215</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="0" t="s">
-        <v>473</v>
+        <v>343</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="C34" s="0" t="s">
         <v>61</v>
       </c>
       <c r="D34" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E34" s="11">
-        <v>46255</v>
+        <v>46259</v>
       </c>
       <c r="F34" s="0" t="s">
-        <v>1095</v>
+        <v>30</v>
       </c>
       <c r="G34" s="11">
-        <v>46435.125</v>
+        <v>46439.125</v>
       </c>
       <c r="H34" s="0" t="s">
-        <v>1106</v>
+        <v>1099</v>
       </c>
       <c r="I34" s="0" t="s">
-        <v>1097</v>
+        <v>1094</v>
       </c>
       <c r="J34" s="0" t="s">
         <v>67</v>
@@ -47012,24 +47018,56 @@
         <v>61</v>
       </c>
       <c r="D35" s="0" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E35" s="11">
         <v>46255</v>
       </c>
       <c r="F35" s="0" t="s">
-        <v>30</v>
+        <v>1080</v>
       </c>
       <c r="G35" s="11">
         <v>46435.125</v>
       </c>
       <c r="H35" s="0" t="s">
-        <v>1098</v>
+        <v>1106</v>
       </c>
       <c r="I35" s="0" t="s">
-        <v>1091</v>
+        <v>1082</v>
       </c>
       <c r="J35" s="0" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="s">
+        <v>473</v>
+      </c>
+      <c r="B36" s="0" t="s">
+        <v>1114</v>
+      </c>
+      <c r="C36" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="D36" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="E36" s="11">
+        <v>46255</v>
+      </c>
+      <c r="F36" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="G36" s="11">
+        <v>46435.125</v>
+      </c>
+      <c r="H36" s="0" t="s">
+        <v>1099</v>
+      </c>
+      <c r="I36" s="0" t="s">
+        <v>1094</v>
+      </c>
+      <c r="J36" s="0" t="s">
         <v>67</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dados — extração 23/10/2026 15:56 (via painel)
</commit_message>
<xml_diff>
--- a/dados/prontuario-equipamentos_1.xlsx
+++ b/dados/prontuario-equipamentos_1.xlsx
@@ -3504,7 +3504,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3">
-        <v>46318.37395836806</v>
+        <v>46318.66441013889</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -34568,13 +34568,13 @@
         <v>698</v>
       </c>
       <c r="J366" s="11">
-        <v>46326.125</v>
+        <v>46372.125</v>
       </c>
       <c r="K366" s="0" t="s">
-        <v>114</v>
+        <v>56</v>
       </c>
       <c r="L366" s="0" t="s">
-        <v>710</v>
+        <v>39</v>
       </c>
       <c r="M366" s="0" t="s">
         <v>39</v>
@@ -34583,7 +34583,7 @@
         <v>43</v>
       </c>
       <c r="O366" s="11">
-        <v>46326.125</v>
+        <v>46691.125</v>
       </c>
       <c r="Q366" s="0" t="s">
         <v>43</v>
@@ -34654,13 +34654,13 @@
         <v>698</v>
       </c>
       <c r="J367" s="11">
-        <v>46326.125</v>
+        <v>46372.125</v>
       </c>
       <c r="K367" s="0" t="s">
-        <v>114</v>
+        <v>56</v>
       </c>
       <c r="L367" s="0" t="s">
-        <v>710</v>
+        <v>39</v>
       </c>
       <c r="M367" s="0" t="s">
         <v>39</v>
@@ -34669,7 +34669,7 @@
         <v>43</v>
       </c>
       <c r="O367" s="11">
-        <v>46326.125</v>
+        <v>46691.125</v>
       </c>
       <c r="Q367" s="0" t="s">
         <v>43</v>
@@ -34826,13 +34826,13 @@
         <v>830</v>
       </c>
       <c r="J369" s="11">
-        <v>46341.125</v>
+        <v>46356.125</v>
       </c>
       <c r="K369" s="0" t="s">
-        <v>114</v>
+        <v>56</v>
       </c>
       <c r="L369" s="0" t="s">
-        <v>710</v>
+        <v>39</v>
       </c>
       <c r="M369" s="0" t="s">
         <v>39</v>
@@ -34841,7 +34841,7 @@
         <v>43</v>
       </c>
       <c r="O369" s="11">
-        <v>46341.125</v>
+        <v>46706.125</v>
       </c>
       <c r="Q369" s="0" t="s">
         <v>43</v>

</xml_diff>

<commit_message>
Atualiza dados — extração 26/10/2026 15:04 (via painel)
</commit_message>
<xml_diff>
--- a/dados/prontuario-equipamentos_1.xlsx
+++ b/dados/prontuario-equipamentos_1.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1092" uniqueCount="1092">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1089" uniqueCount="1089">
   <si>
     <t>Geração:</t>
   </si>
@@ -3280,15 +3280,6 @@
   </si>
   <si>
     <t>MILHO | GNOVA TRANSPORTES LTDA;TOMATE | GNOVA TRANSPORTES LTDA</t>
-  </si>
-  <si>
-    <t>SR/IMPERIAL GR000227T0 1 / SR/IMPERIAL GR000227T0 1</t>
-  </si>
-  <si>
-    <t>Weverson Cavalcante Da Silva</t>
-  </si>
-  <si>
-    <t>MILHO | ITUM ARMAZENS GERAIS E SERVIÇOS LTDA;TOMATE | ITUM ARMAZENS GERAIS E SERVIÇOS LTDA</t>
   </si>
 </sst>
 </file>
@@ -3480,7 +3471,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3">
-        <v>46321.38724898148</v>
+        <v>46321.62844402778</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -44890,7 +44881,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="16384" width="9.140625" customWidth="1"/>
@@ -45824,38 +45815,6 @@
         <v>214</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="0" t="s">
-        <v>536</v>
-      </c>
-      <c r="B30" s="0" t="s">
-        <v>1089</v>
-      </c>
-      <c r="C30" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="D30" s="0" t="s">
-        <v>29</v>
-      </c>
-      <c r="E30" s="11">
-        <v>46261</v>
-      </c>
-      <c r="F30" s="0" t="s">
-        <v>1063</v>
-      </c>
-      <c r="G30" s="11">
-        <v>46441.125</v>
-      </c>
-      <c r="H30" s="0" t="s">
-        <v>1090</v>
-      </c>
-      <c r="I30" s="0" t="s">
-        <v>1065</v>
-      </c>
-      <c r="J30" s="0" t="s">
-        <v>1091</v>
-      </c>
-    </row>
   </sheetData>
   <headerFooter/>
 </worksheet>

</xml_diff>

<commit_message>
Atualiza dados — extração 27/10/2026 09:02 (via painel)
</commit_message>
<xml_diff>
--- a/dados/prontuario-equipamentos_1.xlsx
+++ b/dados/prontuario-equipamentos_1.xlsx
@@ -3471,7 +3471,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3">
-        <v>46321.62844402778</v>
+        <v>46322.37704277778</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -24473,10 +24473,10 @@
         <v>46351.125</v>
       </c>
       <c r="K247" s="0" t="s">
-        <v>56</v>
+        <v>114</v>
       </c>
       <c r="L247" s="0" t="s">
-        <v>39</v>
+        <v>206</v>
       </c>
       <c r="M247" s="0" t="s">
         <v>39</v>

</xml_diff>

<commit_message>
Atualiza dados — extração 30/10/2026 08:27 (via painel)
</commit_message>
<xml_diff>
--- a/dados/prontuario-equipamentos_1.xlsx
+++ b/dados/prontuario-equipamentos_1.xlsx
@@ -375,157 +375,157 @@
     <t>HRO6A06</t>
   </si>
   <si>
+    <t>SAFRA CARRETA</t>
+  </si>
+  <si>
+    <t>HDI7046</t>
+  </si>
+  <si>
+    <t>SR/GUERRA</t>
+  </si>
+  <si>
+    <t>AG GR</t>
+  </si>
+  <si>
+    <t>2006</t>
+  </si>
+  <si>
+    <t>059472922</t>
+  </si>
+  <si>
+    <t>JHX7603</t>
+  </si>
+  <si>
+    <t>STRALIS 570S41T</t>
+  </si>
+  <si>
+    <t>KIT8J31</t>
+  </si>
+  <si>
+    <t>FH 400 6X2T</t>
+  </si>
+  <si>
+    <t>2007</t>
+  </si>
+  <si>
+    <t>054682677</t>
+  </si>
+  <si>
+    <t>OMP3E05</t>
+  </si>
+  <si>
+    <t>2013</t>
+  </si>
+  <si>
+    <t>059315199</t>
+  </si>
+  <si>
+    <t>KDO7124</t>
+  </si>
+  <si>
+    <t>1999</t>
+  </si>
+  <si>
+    <t>SAFRA CARRETA ARRENDADO</t>
+  </si>
+  <si>
+    <t>BWZ6507</t>
+  </si>
+  <si>
+    <t>REB/RANDON</t>
+  </si>
+  <si>
+    <t>SR GR TR</t>
+  </si>
+  <si>
+    <t>1994</t>
+  </si>
+  <si>
+    <t>059765333</t>
+  </si>
+  <si>
+    <t>JLG6E58</t>
+  </si>
+  <si>
+    <t>NL12 360 4X2</t>
+  </si>
+  <si>
+    <t>048941358</t>
+  </si>
+  <si>
+    <t>LVD0G76</t>
+  </si>
+  <si>
+    <t>R124 LA6X2NA 400</t>
+  </si>
+  <si>
+    <t>2004</t>
+  </si>
+  <si>
+    <t>2005</t>
+  </si>
+  <si>
+    <t>059510688</t>
+  </si>
+  <si>
+    <t>SAFRA CAVALO ARRENDADO</t>
+  </si>
+  <si>
+    <t>BRF1J56</t>
+  </si>
+  <si>
+    <t>R113 H 4X2 360</t>
+  </si>
+  <si>
+    <t>1993</t>
+  </si>
+  <si>
+    <t>059297444</t>
+  </si>
+  <si>
+    <t>BWM2D91</t>
+  </si>
+  <si>
+    <t>REB/FACCHINI</t>
+  </si>
+  <si>
+    <t>SRF GR</t>
+  </si>
+  <si>
+    <t>049357788</t>
+  </si>
+  <si>
+    <t>HOA0E87</t>
+  </si>
+  <si>
+    <t>M. BENZ</t>
+  </si>
+  <si>
+    <t>AXOR 2035 S</t>
+  </si>
+  <si>
+    <t>IMI4C27</t>
+  </si>
+  <si>
+    <t>FH12 380 4X2T</t>
+  </si>
+  <si>
+    <t>058966088</t>
+  </si>
+  <si>
+    <t>JMU5F59</t>
+  </si>
+  <si>
+    <t>2000</t>
+  </si>
+  <si>
+    <t>2001</t>
+  </si>
+  <si>
+    <t>059703044</t>
+  </si>
+  <si>
     <t>Documento CRLV ausente ou vencido / Documento ConsultaCRLV vencendo</t>
-  </si>
-  <si>
-    <t>SAFRA CARRETA</t>
-  </si>
-  <si>
-    <t>HDI7046</t>
-  </si>
-  <si>
-    <t>SR/GUERRA</t>
-  </si>
-  <si>
-    <t>AG GR</t>
-  </si>
-  <si>
-    <t>2006</t>
-  </si>
-  <si>
-    <t>059472922</t>
-  </si>
-  <si>
-    <t>JHX7603</t>
-  </si>
-  <si>
-    <t>STRALIS 570S41T</t>
-  </si>
-  <si>
-    <t>KIT8J31</t>
-  </si>
-  <si>
-    <t>FH 400 6X2T</t>
-  </si>
-  <si>
-    <t>2007</t>
-  </si>
-  <si>
-    <t>054682677</t>
-  </si>
-  <si>
-    <t>OMP3E05</t>
-  </si>
-  <si>
-    <t>2013</t>
-  </si>
-  <si>
-    <t>059315199</t>
-  </si>
-  <si>
-    <t>KDO7124</t>
-  </si>
-  <si>
-    <t>1999</t>
-  </si>
-  <si>
-    <t>SAFRA CARRETA ARRENDADO</t>
-  </si>
-  <si>
-    <t>BWZ6507</t>
-  </si>
-  <si>
-    <t>REB/RANDON</t>
-  </si>
-  <si>
-    <t>SR GR TR</t>
-  </si>
-  <si>
-    <t>1994</t>
-  </si>
-  <si>
-    <t>059765333</t>
-  </si>
-  <si>
-    <t>JLG6E58</t>
-  </si>
-  <si>
-    <t>NL12 360 4X2</t>
-  </si>
-  <si>
-    <t>048941358</t>
-  </si>
-  <si>
-    <t>LVD0G76</t>
-  </si>
-  <si>
-    <t>R124 LA6X2NA 400</t>
-  </si>
-  <si>
-    <t>2004</t>
-  </si>
-  <si>
-    <t>2005</t>
-  </si>
-  <si>
-    <t>059510688</t>
-  </si>
-  <si>
-    <t>SAFRA CAVALO ARRENDADO</t>
-  </si>
-  <si>
-    <t>BRF1J56</t>
-  </si>
-  <si>
-    <t>R113 H 4X2 360</t>
-  </si>
-  <si>
-    <t>1993</t>
-  </si>
-  <si>
-    <t>059297444</t>
-  </si>
-  <si>
-    <t>BWM2D91</t>
-  </si>
-  <si>
-    <t>REB/FACCHINI</t>
-  </si>
-  <si>
-    <t>SRF GR</t>
-  </si>
-  <si>
-    <t>049357788</t>
-  </si>
-  <si>
-    <t>HOA0E87</t>
-  </si>
-  <si>
-    <t>M. BENZ</t>
-  </si>
-  <si>
-    <t>AXOR 2035 S</t>
-  </si>
-  <si>
-    <t>IMI4C27</t>
-  </si>
-  <si>
-    <t>FH12 380 4X2T</t>
-  </si>
-  <si>
-    <t>058966088</t>
-  </si>
-  <si>
-    <t>JMU5F59</t>
-  </si>
-  <si>
-    <t>2000</t>
-  </si>
-  <si>
-    <t>2001</t>
-  </si>
-  <si>
-    <t>059703044</t>
   </si>
   <si>
     <t>NFK8A40</t>
@@ -3471,7 +3471,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3">
-        <v>46324.64689034722</v>
+        <v>46325.35281707176</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -5874,7 +5874,7 @@
         <v>40</v>
       </c>
       <c r="L29" s="0" t="s">
-        <v>120</v>
+        <v>107</v>
       </c>
       <c r="M29" s="0" t="s">
         <v>39</v>
@@ -5886,7 +5886,7 @@
         <v>46310.125</v>
       </c>
       <c r="Q29" s="0" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R29" s="11">
         <v>46324.125</v>
@@ -5930,28 +5930,28 @@
     </row>
     <row r="30">
       <c r="A30" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B30" s="0" t="s">
         <v>34</v>
       </c>
       <c r="C30" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="D30" s="0" t="s">
         <v>122</v>
       </c>
-      <c r="D30" s="0" t="s">
+      <c r="E30" s="0" t="s">
         <v>123</v>
       </c>
-      <c r="E30" s="0" t="s">
+      <c r="F30" s="0" t="s">
         <v>124</v>
       </c>
-      <c r="F30" s="0" t="s">
+      <c r="G30" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="H30" s="0" t="s">
         <v>125</v>
-      </c>
-      <c r="G30" s="0" t="s">
-        <v>125</v>
-      </c>
-      <c r="H30" s="0" t="s">
-        <v>126</v>
       </c>
       <c r="J30" s="11"/>
       <c r="K30" s="0" t="s">
@@ -6020,13 +6020,13 @@
         <v>34</v>
       </c>
       <c r="C31" s="0" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D31" s="0" t="s">
         <v>63</v>
       </c>
       <c r="E31" s="0" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F31" s="0" t="s">
         <v>74</v>
@@ -6035,7 +6035,7 @@
         <v>74</v>
       </c>
       <c r="H31" s="0" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J31" s="11"/>
       <c r="K31" s="0" t="s">
@@ -6104,22 +6104,22 @@
         <v>49</v>
       </c>
       <c r="C32" s="0" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D32" s="0" t="s">
         <v>51</v>
       </c>
       <c r="E32" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="F32" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="G32" s="0" t="s">
         <v>130</v>
       </c>
-      <c r="F32" s="0" t="s">
-        <v>125</v>
-      </c>
-      <c r="G32" s="0" t="s">
+      <c r="H32" s="0" t="s">
         <v>131</v>
-      </c>
-      <c r="H32" s="0" t="s">
-        <v>132</v>
       </c>
       <c r="J32" s="11">
         <v>46391.125</v>
@@ -6184,13 +6184,13 @@
     </row>
     <row r="33">
       <c r="A33" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B33" s="0" t="s">
         <v>34</v>
       </c>
       <c r="C33" s="0" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D33" s="0" t="s">
         <v>36</v>
@@ -6202,10 +6202,10 @@
         <v>60</v>
       </c>
       <c r="G33" s="0" t="s">
+        <v>133</v>
+      </c>
+      <c r="H33" s="0" t="s">
         <v>134</v>
-      </c>
-      <c r="H33" s="0" t="s">
-        <v>135</v>
       </c>
       <c r="J33" s="11"/>
       <c r="K33" s="0" t="s">
@@ -6274,7 +6274,7 @@
         <v>34</v>
       </c>
       <c r="C34" s="0" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D34" s="0" t="s">
         <v>51</v>
@@ -6286,10 +6286,10 @@
         <v>85</v>
       </c>
       <c r="G34" s="0" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H34" s="0" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="J34" s="11"/>
       <c r="K34" s="0" t="s">
@@ -6352,28 +6352,28 @@
     </row>
     <row r="35">
       <c r="A35" s="0" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B35" s="0" t="s">
         <v>61</v>
       </c>
       <c r="C35" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="D35" s="0" t="s">
         <v>139</v>
       </c>
-      <c r="D35" s="0" t="s">
+      <c r="E35" s="0" t="s">
         <v>140</v>
       </c>
-      <c r="E35" s="0" t="s">
+      <c r="F35" s="0" t="s">
         <v>141</v>
       </c>
-      <c r="F35" s="0" t="s">
+      <c r="G35" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="H35" s="0" t="s">
         <v>142</v>
-      </c>
-      <c r="G35" s="0" t="s">
-        <v>142</v>
-      </c>
-      <c r="H35" s="0" t="s">
-        <v>143</v>
       </c>
       <c r="J35" s="11">
         <v>46367.125</v>
@@ -6447,22 +6447,22 @@
         <v>49</v>
       </c>
       <c r="C36" s="0" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D36" s="0" t="s">
         <v>51</v>
       </c>
       <c r="E36" s="0" t="s">
+        <v>144</v>
+      </c>
+      <c r="F36" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="G36" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="H36" s="0" t="s">
         <v>145</v>
-      </c>
-      <c r="F36" s="0" t="s">
-        <v>142</v>
-      </c>
-      <c r="G36" s="0" t="s">
-        <v>142</v>
-      </c>
-      <c r="H36" s="0" t="s">
-        <v>146</v>
       </c>
       <c r="J36" s="11">
         <v>46361.125</v>
@@ -6533,22 +6533,22 @@
         <v>49</v>
       </c>
       <c r="C37" s="0" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D37" s="0" t="s">
         <v>77</v>
       </c>
       <c r="E37" s="0" t="s">
+        <v>147</v>
+      </c>
+      <c r="F37" s="0" t="s">
         <v>148</v>
       </c>
-      <c r="F37" s="0" t="s">
+      <c r="G37" s="0" t="s">
         <v>149</v>
       </c>
-      <c r="G37" s="0" t="s">
+      <c r="H37" s="0" t="s">
         <v>150</v>
-      </c>
-      <c r="H37" s="0" t="s">
-        <v>151</v>
       </c>
       <c r="J37" s="11">
         <v>46374.125</v>
@@ -6613,28 +6613,28 @@
     </row>
     <row r="38">
       <c r="A38" s="0" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B38" s="0" t="s">
         <v>61</v>
       </c>
       <c r="C38" s="0" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D38" s="0" t="s">
         <v>77</v>
       </c>
       <c r="E38" s="0" t="s">
+        <v>153</v>
+      </c>
+      <c r="F38" s="0" t="s">
         <v>154</v>
       </c>
-      <c r="F38" s="0" t="s">
+      <c r="G38" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="H38" s="0" t="s">
         <v>155</v>
-      </c>
-      <c r="G38" s="0" t="s">
-        <v>155</v>
-      </c>
-      <c r="H38" s="0" t="s">
-        <v>156</v>
       </c>
       <c r="J38" s="11">
         <v>46356.125</v>
@@ -6702,28 +6702,28 @@
     </row>
     <row r="39">
       <c r="A39" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B39" s="0" t="s">
         <v>34</v>
       </c>
       <c r="C39" s="0" t="s">
+        <v>156</v>
+      </c>
+      <c r="D39" s="0" t="s">
         <v>157</v>
       </c>
-      <c r="D39" s="0" t="s">
+      <c r="E39" s="0" t="s">
         <v>158</v>
       </c>
-      <c r="E39" s="0" t="s">
+      <c r="F39" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="G39" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="H39" s="0" t="s">
         <v>159</v>
-      </c>
-      <c r="F39" s="0" t="s">
-        <v>155</v>
-      </c>
-      <c r="G39" s="0" t="s">
-        <v>155</v>
-      </c>
-      <c r="H39" s="0" t="s">
-        <v>160</v>
       </c>
       <c r="J39" s="11">
         <v>46390.125</v>
@@ -6794,13 +6794,13 @@
         <v>34</v>
       </c>
       <c r="C40" s="0" t="s">
+        <v>160</v>
+      </c>
+      <c r="D40" s="0" t="s">
         <v>161</v>
       </c>
-      <c r="D40" s="0" t="s">
+      <c r="E40" s="0" t="s">
         <v>162</v>
-      </c>
-      <c r="E40" s="0" t="s">
-        <v>163</v>
       </c>
       <c r="F40" s="0" t="s">
         <v>74</v>
@@ -6809,7 +6809,7 @@
         <v>65</v>
       </c>
       <c r="H40" s="0" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J40" s="11"/>
       <c r="K40" s="0" t="s">
@@ -6872,28 +6872,28 @@
     </row>
     <row r="41">
       <c r="A41" s="0" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B41" s="0" t="s">
         <v>61</v>
       </c>
       <c r="C41" s="0" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D41" s="0" t="s">
         <v>51</v>
       </c>
       <c r="E41" s="0" t="s">
+        <v>164</v>
+      </c>
+      <c r="F41" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="G41" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="H41" s="0" t="s">
         <v>165</v>
-      </c>
-      <c r="F41" s="0" t="s">
-        <v>150</v>
-      </c>
-      <c r="G41" s="0" t="s">
-        <v>150</v>
-      </c>
-      <c r="H41" s="0" t="s">
-        <v>166</v>
       </c>
       <c r="J41" s="11"/>
       <c r="K41" s="0" t="s">
@@ -6959,35 +6959,35 @@
     </row>
     <row r="42">
       <c r="A42" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B42" s="0" t="s">
         <v>34</v>
       </c>
       <c r="C42" s="0" t="s">
+        <v>166</v>
+      </c>
+      <c r="D42" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="E42" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="F42" s="0" t="s">
         <v>167</v>
       </c>
-      <c r="D42" s="0" t="s">
-        <v>123</v>
-      </c>
-      <c r="E42" s="0" t="s">
-        <v>124</v>
-      </c>
-      <c r="F42" s="0" t="s">
+      <c r="G42" s="0" t="s">
         <v>168</v>
       </c>
-      <c r="G42" s="0" t="s">
+      <c r="H42" s="0" t="s">
         <v>169</v>
-      </c>
-      <c r="H42" s="0" t="s">
-        <v>170</v>
       </c>
       <c r="J42" s="11"/>
       <c r="K42" s="0" t="s">
         <v>40</v>
       </c>
       <c r="L42" s="0" t="s">
-        <v>120</v>
+        <v>170</v>
       </c>
       <c r="M42" s="0" t="s">
         <v>39</v>
@@ -7052,26 +7052,26 @@
         <v>171</v>
       </c>
       <c r="D43" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E43" s="0" t="s">
         <v>172</v>
       </c>
       <c r="F43" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G43" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H43" s="0" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="J43" s="11"/>
       <c r="K43" s="0" t="s">
         <v>40</v>
       </c>
       <c r="L43" s="0" t="s">
-        <v>120</v>
+        <v>170</v>
       </c>
       <c r="M43" s="0" t="s">
         <v>39</v>
@@ -7136,7 +7136,7 @@
         <v>174</v>
       </c>
       <c r="D44" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E44" s="0" t="s">
         <v>175</v>
@@ -7303,7 +7303,7 @@
         <v>182</v>
       </c>
       <c r="D46" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E46" s="0" t="s">
         <v>183</v>
@@ -7387,7 +7387,7 @@
         <v>186</v>
       </c>
       <c r="D47" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E47" s="0" t="s">
         <v>187</v>
@@ -7555,7 +7555,7 @@
         <v>194</v>
       </c>
       <c r="D49" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E49" s="0" t="s">
         <v>195</v>
@@ -7632,7 +7632,7 @@
     </row>
     <row r="50">
       <c r="A50" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B50" s="0" t="s">
         <v>34</v>
@@ -7718,7 +7718,7 @@
     </row>
     <row r="51">
       <c r="A51" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B51" s="0" t="s">
         <v>34</v>
@@ -7804,7 +7804,7 @@
     </row>
     <row r="52">
       <c r="A52" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B52" s="0" t="s">
         <v>34</v>
@@ -7974,7 +7974,7 @@
     </row>
     <row r="54">
       <c r="A54" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B54" s="0" t="s">
         <v>49</v>
@@ -7989,13 +7989,13 @@
         <v>72</v>
       </c>
       <c r="F54" s="0" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G54" s="0" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="H54" s="0" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="J54" s="11">
         <v>46374.125</v>
@@ -8060,7 +8060,7 @@
     </row>
     <row r="55">
       <c r="A55" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B55" s="0" t="s">
         <v>61</v>
@@ -8155,7 +8155,7 @@
         <v>215</v>
       </c>
       <c r="D56" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E56" s="0" t="s">
         <v>216</v>
@@ -8245,10 +8245,10 @@
         <v>219</v>
       </c>
       <c r="F57" s="0" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G57" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H57" s="0" t="s">
         <v>39</v>
@@ -8325,16 +8325,16 @@
         <v>220</v>
       </c>
       <c r="D58" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E58" s="0" t="s">
         <v>172</v>
       </c>
       <c r="F58" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G58" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H58" s="0" t="s">
         <v>221</v>
@@ -8402,7 +8402,7 @@
     </row>
     <row r="59">
       <c r="A59" s="0" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B59" s="0" t="s">
         <v>61</v>
@@ -8417,10 +8417,10 @@
         <v>223</v>
       </c>
       <c r="F59" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G59" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H59" s="0" t="s">
         <v>224</v>
@@ -8586,13 +8586,13 @@
         <v>51</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F61" s="0" t="s">
         <v>231</v>
       </c>
       <c r="G61" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H61" s="0" t="s">
         <v>232</v>
@@ -8660,7 +8660,7 @@
     </row>
     <row r="62">
       <c r="A62" s="0" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B62" s="0" t="s">
         <v>61</v>
@@ -8764,10 +8764,10 @@
         <v>237</v>
       </c>
       <c r="F63" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G63" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H63" s="0" t="s">
         <v>39</v>
@@ -9087,7 +9087,7 @@
     </row>
     <row r="67">
       <c r="A67" s="0" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B67" s="0" t="s">
         <v>61</v>
@@ -9176,7 +9176,7 @@
     </row>
     <row r="68">
       <c r="A68" s="0" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B68" s="0" t="s">
         <v>61</v>
@@ -9265,7 +9265,7 @@
     </row>
     <row r="69">
       <c r="A69" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B69" s="0" t="s">
         <v>61</v>
@@ -9280,10 +9280,10 @@
         <v>37</v>
       </c>
       <c r="F69" s="0" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G69" s="0" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H69" s="0" t="s">
         <v>254</v>
@@ -9435,7 +9435,7 @@
     </row>
     <row r="71">
       <c r="A71" s="0" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B71" s="0" t="s">
         <v>61</v>
@@ -9522,7 +9522,7 @@
     </row>
     <row r="72">
       <c r="A72" s="0" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B72" s="0" t="s">
         <v>61</v>
@@ -9537,10 +9537,10 @@
         <v>264</v>
       </c>
       <c r="F72" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G72" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H72" s="0" t="s">
         <v>261</v>
@@ -9609,7 +9609,7 @@
     </row>
     <row r="73">
       <c r="A73" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B73" s="0" t="s">
         <v>34</v>
@@ -9693,7 +9693,7 @@
     </row>
     <row r="74">
       <c r="A74" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B74" s="0" t="s">
         <v>34</v>
@@ -9789,13 +9789,13 @@
         <v>51</v>
       </c>
       <c r="E75" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="F75" s="0" t="s">
         <v>130</v>
       </c>
-      <c r="F75" s="0" t="s">
-        <v>131</v>
-      </c>
       <c r="G75" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H75" s="0" t="s">
         <v>266</v>
@@ -9876,10 +9876,10 @@
         <v>272</v>
       </c>
       <c r="F76" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G76" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H76" s="0" t="s">
         <v>273</v>
@@ -9962,10 +9962,10 @@
         <v>275</v>
       </c>
       <c r="F77" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G77" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H77" s="0" t="s">
         <v>273</v>
@@ -10045,13 +10045,13 @@
         <v>51</v>
       </c>
       <c r="E78" s="0" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F78" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G78" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H78" s="0" t="s">
         <v>273</v>
@@ -10119,7 +10119,7 @@
     </row>
     <row r="79">
       <c r="A79" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B79" s="0" t="s">
         <v>61</v>
@@ -10134,10 +10134,10 @@
         <v>272</v>
       </c>
       <c r="F79" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G79" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H79" s="0" t="s">
         <v>278</v>
@@ -10205,7 +10205,7 @@
     </row>
     <row r="80">
       <c r="A80" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B80" s="0" t="s">
         <v>61</v>
@@ -10220,10 +10220,10 @@
         <v>275</v>
       </c>
       <c r="F80" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G80" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H80" s="0" t="s">
         <v>278</v>
@@ -10291,7 +10291,7 @@
     </row>
     <row r="81">
       <c r="A81" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B81" s="0" t="s">
         <v>61</v>
@@ -10375,7 +10375,7 @@
     </row>
     <row r="82">
       <c r="A82" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B82" s="0" t="s">
         <v>61</v>
@@ -10715,7 +10715,7 @@
     </row>
     <row r="86">
       <c r="A86" s="0" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B86" s="0" t="s">
         <v>61</v>
@@ -10804,7 +10804,7 @@
     </row>
     <row r="87">
       <c r="A87" s="0" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B87" s="0" t="s">
         <v>61</v>
@@ -10893,7 +10893,7 @@
     </row>
     <row r="88">
       <c r="A88" s="0" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B88" s="0" t="s">
         <v>61</v>
@@ -11261,7 +11261,7 @@
         <v>200</v>
       </c>
       <c r="H92" s="0" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="J92" s="11">
         <v>46391.125</v>
@@ -11427,10 +11427,10 @@
         <v>304</v>
       </c>
       <c r="F94" s="0" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G94" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H94" s="0" t="s">
         <v>39</v>
@@ -11513,10 +11513,10 @@
         <v>304</v>
       </c>
       <c r="F95" s="0" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G95" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H95" s="0" t="s">
         <v>39</v>
@@ -11599,10 +11599,10 @@
         <v>307</v>
       </c>
       <c r="F96" s="0" t="s">
+        <v>148</v>
+      </c>
+      <c r="G96" s="0" t="s">
         <v>149</v>
-      </c>
-      <c r="G96" s="0" t="s">
-        <v>150</v>
       </c>
       <c r="H96" s="0" t="s">
         <v>39</v>
@@ -12029,10 +12029,10 @@
         <v>316</v>
       </c>
       <c r="F101" s="0" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G101" s="0" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H101" s="0" t="s">
         <v>317</v>
@@ -12199,10 +12199,10 @@
         <v>322</v>
       </c>
       <c r="F103" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G103" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H103" s="0" t="s">
         <v>39</v>
@@ -12283,10 +12283,10 @@
         <v>322</v>
       </c>
       <c r="F104" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G104" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H104" s="0" t="s">
         <v>39</v>
@@ -12696,7 +12696,7 @@
     </row>
     <row r="109">
       <c r="A109" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B109" s="0" t="s">
         <v>61</v>
@@ -12780,7 +12780,7 @@
     </row>
     <row r="110">
       <c r="A110" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B110" s="0" t="s">
         <v>61</v>
@@ -12948,7 +12948,7 @@
     </row>
     <row r="112">
       <c r="A112" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B112" s="0" t="s">
         <v>61</v>
@@ -13034,7 +13034,7 @@
     </row>
     <row r="113">
       <c r="A113" s="0" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B113" s="0" t="s">
         <v>61</v>
@@ -13055,7 +13055,7 @@
         <v>79</v>
       </c>
       <c r="H113" s="0" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J113" s="11">
         <v>46356.125</v>
@@ -13209,7 +13209,7 @@
     </row>
     <row r="115">
       <c r="A115" s="0" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B115" s="0" t="s">
         <v>34</v>
@@ -13224,10 +13224,10 @@
         <v>234</v>
       </c>
       <c r="F115" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G115" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H115" s="0" t="s">
         <v>344</v>
@@ -13311,7 +13311,7 @@
         <v>346</v>
       </c>
       <c r="F116" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G116" s="0" t="s">
         <v>93</v>
@@ -13820,13 +13820,13 @@
         <v>51</v>
       </c>
       <c r="E122" s="0" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F122" s="0" t="s">
         <v>231</v>
       </c>
       <c r="G122" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H122" s="0" t="s">
         <v>352</v>
@@ -13901,13 +13901,13 @@
         <v>355</v>
       </c>
       <c r="D123" s="0" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E123" s="0" t="s">
         <v>356</v>
       </c>
       <c r="F123" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G123" s="0" t="s">
         <v>79</v>
@@ -13985,13 +13985,13 @@
         <v>358</v>
       </c>
       <c r="D124" s="0" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E124" s="0" t="s">
         <v>356</v>
       </c>
       <c r="F124" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G124" s="0" t="s">
         <v>79</v>
@@ -14077,10 +14077,10 @@
         <v>360</v>
       </c>
       <c r="F125" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G125" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H125" s="0" t="s">
         <v>357</v>
@@ -14333,10 +14333,10 @@
         <v>366</v>
       </c>
       <c r="F128" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G128" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H128" s="0" t="s">
         <v>39</v>
@@ -14662,7 +14662,7 @@
     </row>
     <row r="132">
       <c r="A132" s="0" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B132" s="0" t="s">
         <v>61</v>
@@ -14683,7 +14683,7 @@
         <v>38</v>
       </c>
       <c r="H132" s="0" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J132" s="11">
         <v>46356.125</v>
@@ -14769,7 +14769,7 @@
         <v>231</v>
       </c>
       <c r="G133" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H133" s="0" t="s">
         <v>39</v>
@@ -14852,10 +14852,10 @@
         <v>304</v>
       </c>
       <c r="F134" s="0" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G134" s="0" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H134" s="0" t="s">
         <v>39</v>
@@ -14938,10 +14938,10 @@
         <v>304</v>
       </c>
       <c r="F135" s="0" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G135" s="0" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H135" s="0" t="s">
         <v>39</v>
@@ -15107,7 +15107,7 @@
         <v>51</v>
       </c>
       <c r="E137" s="0" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F137" s="0" t="s">
         <v>79</v>
@@ -15196,10 +15196,10 @@
         <v>339</v>
       </c>
       <c r="F138" s="0" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G138" s="0" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="H138" s="0" t="s">
         <v>39</v>
@@ -16050,10 +16050,10 @@
         <v>396</v>
       </c>
       <c r="F148" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G148" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H148" s="0" t="s">
         <v>39</v>
@@ -16298,7 +16298,7 @@
         <v>401</v>
       </c>
       <c r="D151" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E151" s="0" t="s">
         <v>216</v>
@@ -16388,10 +16388,10 @@
         <v>371</v>
       </c>
       <c r="F152" s="0" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G152" s="0" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H152" s="0" t="s">
         <v>39</v>
@@ -16715,7 +16715,7 @@
     </row>
     <row r="156">
       <c r="A156" s="0" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B156" s="0" t="s">
         <v>61</v>
@@ -16736,7 +16736,7 @@
         <v>192</v>
       </c>
       <c r="H156" s="0" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J156" s="11">
         <v>46367.125</v>
@@ -16819,10 +16819,10 @@
         <v>411</v>
       </c>
       <c r="F157" s="0" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G157" s="0" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H157" s="0" t="s">
         <v>39</v>
@@ -16985,10 +16985,10 @@
         <v>413</v>
       </c>
       <c r="D159" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="E159" s="0" t="s">
         <v>123</v>
-      </c>
-      <c r="E159" s="0" t="s">
-        <v>124</v>
       </c>
       <c r="F159" s="0" t="s">
         <v>74</v>
@@ -17161,10 +17161,10 @@
         <v>419</v>
       </c>
       <c r="F161" s="0" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G161" s="0" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H161" s="0" t="s">
         <v>39</v>
@@ -17247,10 +17247,10 @@
         <v>311</v>
       </c>
       <c r="F162" s="0" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G162" s="0" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H162" s="0" t="s">
         <v>39</v>
@@ -18191,7 +18191,7 @@
         <v>337</v>
       </c>
       <c r="F173" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G173" s="0" t="s">
         <v>93</v>
@@ -18449,10 +18449,10 @@
         <v>304</v>
       </c>
       <c r="F176" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G176" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H176" s="0" t="s">
         <v>39</v>
@@ -18710,10 +18710,10 @@
         <v>304</v>
       </c>
       <c r="F179" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G179" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H179" s="0" t="s">
         <v>39</v>
@@ -18951,7 +18951,7 @@
     </row>
     <row r="182">
       <c r="A182" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B182" s="0" t="s">
         <v>34</v>
@@ -18966,10 +18966,10 @@
         <v>452</v>
       </c>
       <c r="F182" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G182" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H182" s="0" t="s">
         <v>450</v>
@@ -19044,16 +19044,16 @@
         <v>453</v>
       </c>
       <c r="D183" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E183" s="0" t="s">
         <v>187</v>
       </c>
       <c r="F183" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G183" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H183" s="0" t="s">
         <v>454</v>
@@ -19121,7 +19121,7 @@
     </row>
     <row r="184">
       <c r="A184" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B184" s="0" t="s">
         <v>61</v>
@@ -19302,7 +19302,7 @@
         <v>460</v>
       </c>
       <c r="D186" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E186" s="0" t="s">
         <v>461</v>
@@ -19391,10 +19391,10 @@
         <v>464</v>
       </c>
       <c r="F187" s="0" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G187" s="0" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="H187" s="0" t="s">
         <v>465</v>
@@ -19460,7 +19460,7 @@
     </row>
     <row r="188">
       <c r="A188" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B188" s="0" t="s">
         <v>34</v>
@@ -19475,10 +19475,10 @@
         <v>467</v>
       </c>
       <c r="F188" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G188" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H188" s="0" t="s">
         <v>465</v>
@@ -19553,10 +19553,10 @@
         <v>468</v>
       </c>
       <c r="D189" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="E189" s="0" t="s">
         <v>123</v>
-      </c>
-      <c r="E189" s="0" t="s">
-        <v>124</v>
       </c>
       <c r="F189" s="0" t="s">
         <v>38</v>
@@ -19637,10 +19637,10 @@
         <v>469</v>
       </c>
       <c r="D190" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="E190" s="0" t="s">
         <v>123</v>
-      </c>
-      <c r="E190" s="0" t="s">
-        <v>124</v>
       </c>
       <c r="F190" s="0" t="s">
         <v>38</v>
@@ -19712,7 +19712,7 @@
     </row>
     <row r="191">
       <c r="A191" s="0" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B191" s="0" t="s">
         <v>61</v>
@@ -19799,7 +19799,7 @@
     </row>
     <row r="192">
       <c r="A192" s="0" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B192" s="0" t="s">
         <v>61</v>
@@ -19808,7 +19808,7 @@
         <v>472</v>
       </c>
       <c r="D192" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E192" s="0" t="s">
         <v>473</v>
@@ -19886,7 +19886,7 @@
     </row>
     <row r="193">
       <c r="A193" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B193" s="0" t="s">
         <v>61</v>
@@ -19985,10 +19985,10 @@
         <v>234</v>
       </c>
       <c r="F194" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G194" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H194" s="0" t="s">
         <v>476</v>
@@ -20063,7 +20063,7 @@
         <v>478</v>
       </c>
       <c r="D195" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E195" s="0" t="s">
         <v>183</v>
@@ -20233,7 +20233,7 @@
         <v>483</v>
       </c>
       <c r="D197" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E197" s="0" t="s">
         <v>175</v>
@@ -20319,16 +20319,16 @@
         <v>486</v>
       </c>
       <c r="D198" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E198" s="0" t="s">
         <v>487</v>
       </c>
       <c r="F198" s="0" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G198" s="0" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H198" s="0" t="s">
         <v>488</v>
@@ -20489,7 +20489,7 @@
         <v>492</v>
       </c>
       <c r="D200" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E200" s="0" t="s">
         <v>175</v>
@@ -20579,7 +20579,7 @@
         <v>496</v>
       </c>
       <c r="F201" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G201" s="0" t="s">
         <v>93</v>
@@ -20659,7 +20659,7 @@
         <v>498</v>
       </c>
       <c r="D202" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E202" s="0" t="s">
         <v>499</v>
@@ -20754,10 +20754,10 @@
         <v>503</v>
       </c>
       <c r="F203" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G203" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H203" s="0" t="s">
         <v>504</v>
@@ -20823,7 +20823,7 @@
     </row>
     <row r="204">
       <c r="A204" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B204" s="0" t="s">
         <v>34</v>
@@ -20832,16 +20832,16 @@
         <v>505</v>
       </c>
       <c r="D204" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="E204" s="0" t="s">
         <v>140</v>
-      </c>
-      <c r="E204" s="0" t="s">
-        <v>141</v>
       </c>
       <c r="F204" s="0" t="s">
         <v>506</v>
       </c>
       <c r="G204" s="0" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="H204" s="0" t="s">
         <v>504</v>
@@ -20924,10 +20924,10 @@
         <v>187</v>
       </c>
       <c r="F205" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G205" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H205" s="0" t="s">
         <v>509</v>
@@ -21008,10 +21008,10 @@
         <v>511</v>
       </c>
       <c r="F206" s="0" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G206" s="0" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H206" s="0" t="s">
         <v>512</v>
@@ -21163,7 +21163,7 @@
     </row>
     <row r="208">
       <c r="A208" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B208" s="0" t="s">
         <v>34</v>
@@ -21178,10 +21178,10 @@
         <v>516</v>
       </c>
       <c r="F208" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G208" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H208" s="0" t="s">
         <v>514</v>
@@ -21348,13 +21348,13 @@
         <v>521</v>
       </c>
       <c r="F210" s="0" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G210" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H210" s="0" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="J210" s="11">
         <v>46373.125</v>
@@ -21428,10 +21428,10 @@
         <v>522</v>
       </c>
       <c r="D211" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="E211" s="0" t="s">
         <v>123</v>
-      </c>
-      <c r="E211" s="0" t="s">
-        <v>124</v>
       </c>
       <c r="F211" s="0" t="s">
         <v>38</v>
@@ -21512,10 +21512,10 @@
         <v>524</v>
       </c>
       <c r="D212" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="E212" s="0" t="s">
         <v>123</v>
-      </c>
-      <c r="E212" s="0" t="s">
-        <v>124</v>
       </c>
       <c r="F212" s="0" t="s">
         <v>38</v>
@@ -21587,7 +21587,7 @@
     </row>
     <row r="213">
       <c r="A213" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B213" s="0" t="s">
         <v>34</v>
@@ -21596,10 +21596,10 @@
         <v>525</v>
       </c>
       <c r="D213" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="E213" s="0" t="s">
         <v>123</v>
-      </c>
-      <c r="E213" s="0" t="s">
-        <v>124</v>
       </c>
       <c r="F213" s="0" t="s">
         <v>526</v>
@@ -21755,7 +21755,7 @@
     </row>
     <row r="215">
       <c r="A215" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B215" s="0" t="s">
         <v>34</v>
@@ -21839,7 +21839,7 @@
     </row>
     <row r="216">
       <c r="A216" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B216" s="0" t="s">
         <v>34</v>
@@ -21848,13 +21848,13 @@
         <v>534</v>
       </c>
       <c r="D216" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="E216" s="0" t="s">
         <v>140</v>
       </c>
-      <c r="E216" s="0" t="s">
+      <c r="F216" s="0" t="s">
         <v>141</v>
-      </c>
-      <c r="F216" s="0" t="s">
-        <v>142</v>
       </c>
       <c r="G216" s="0" t="s">
         <v>332</v>
@@ -21944,7 +21944,7 @@
         <v>200</v>
       </c>
       <c r="H217" s="0" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="J217" s="11">
         <v>46384.125</v>
@@ -22273,13 +22273,13 @@
         <v>51</v>
       </c>
       <c r="E221" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="F221" s="0" t="s">
         <v>130</v>
       </c>
-      <c r="F221" s="0" t="s">
-        <v>131</v>
-      </c>
       <c r="G221" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H221" s="0" t="s">
         <v>543</v>
@@ -22347,7 +22347,7 @@
     </row>
     <row r="222">
       <c r="A222" s="0" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B222" s="0" t="s">
         <v>61</v>
@@ -22362,13 +22362,13 @@
         <v>545</v>
       </c>
       <c r="F222" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G222" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H222" s="0" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J222" s="11"/>
       <c r="K222" s="0" t="s">
@@ -22530,10 +22530,10 @@
         <v>550</v>
       </c>
       <c r="F224" s="0" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G224" s="0" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J224" s="11">
         <v>46419.125</v>
@@ -22598,7 +22598,7 @@
     </row>
     <row r="225">
       <c r="A225" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B225" s="0" t="s">
         <v>61</v>
@@ -22613,13 +22613,13 @@
         <v>228</v>
       </c>
       <c r="F225" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="G225" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="H225" s="0" t="s">
         <v>155</v>
-      </c>
-      <c r="G225" s="0" t="s">
-        <v>155</v>
-      </c>
-      <c r="H225" s="0" t="s">
-        <v>156</v>
       </c>
       <c r="J225" s="11"/>
       <c r="K225" s="0" t="s">
@@ -22783,10 +22783,10 @@
         <v>556</v>
       </c>
       <c r="F227" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G227" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H227" s="0" t="s">
         <v>557</v>
@@ -22869,10 +22869,10 @@
         <v>559</v>
       </c>
       <c r="F228" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G228" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H228" s="0" t="s">
         <v>557</v>
@@ -23041,10 +23041,10 @@
         <v>563</v>
       </c>
       <c r="F230" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G230" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J230" s="11">
         <v>46416.125</v>
@@ -23202,16 +23202,16 @@
         <v>568</v>
       </c>
       <c r="D232" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="E232" s="0" t="s">
         <v>123</v>
       </c>
-      <c r="E232" s="0" t="s">
+      <c r="F232" s="0" t="s">
         <v>124</v>
       </c>
-      <c r="F232" s="0" t="s">
-        <v>125</v>
-      </c>
       <c r="G232" s="0" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H232" s="0" t="s">
         <v>567</v>
@@ -23286,16 +23286,16 @@
         <v>569</v>
       </c>
       <c r="D233" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="E233" s="0" t="s">
         <v>123</v>
       </c>
-      <c r="E233" s="0" t="s">
+      <c r="F233" s="0" t="s">
         <v>124</v>
       </c>
-      <c r="F233" s="0" t="s">
-        <v>125</v>
-      </c>
       <c r="G233" s="0" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H233" s="0" t="s">
         <v>567</v>
@@ -23533,16 +23533,16 @@
         <v>576</v>
       </c>
       <c r="D236" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E236" s="0" t="s">
         <v>487</v>
       </c>
       <c r="F236" s="0" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G236" s="0" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H236" s="0" t="s">
         <v>577</v>
@@ -23693,7 +23693,7 @@
     </row>
     <row r="238">
       <c r="A238" s="0" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B238" s="0" t="s">
         <v>61</v>
@@ -23864,7 +23864,7 @@
     </row>
     <row r="240">
       <c r="A240" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B240" s="0" t="s">
         <v>34</v>
@@ -23879,10 +23879,10 @@
         <v>304</v>
       </c>
       <c r="F240" s="0" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G240" s="0" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H240" s="0" t="s">
         <v>535</v>
@@ -23948,7 +23948,7 @@
     </row>
     <row r="241">
       <c r="A241" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B241" s="0" t="s">
         <v>61</v>
@@ -24212,10 +24212,10 @@
         <v>259</v>
       </c>
       <c r="F244" s="0" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G244" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H244" s="0" t="s">
         <v>39</v>
@@ -24292,7 +24292,7 @@
         <v>51</v>
       </c>
       <c r="E245" s="0" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F245" s="0" t="s">
         <v>79</v>
@@ -24630,7 +24630,7 @@
         <v>60</v>
       </c>
       <c r="G249" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H249" s="0" t="s">
         <v>39</v>
@@ -24640,7 +24640,7 @@
         <v>40</v>
       </c>
       <c r="L249" s="0" t="s">
-        <v>120</v>
+        <v>170</v>
       </c>
       <c r="M249" s="0" t="s">
         <v>39</v>
@@ -24791,10 +24791,10 @@
         <v>613</v>
       </c>
       <c r="F251" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G251" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H251" s="0" t="s">
         <v>39</v>
@@ -24957,7 +24957,7 @@
         <v>618</v>
       </c>
       <c r="F253" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G253" s="0" t="s">
         <v>526</v>
@@ -25123,10 +25123,10 @@
         <v>624</v>
       </c>
       <c r="F255" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G255" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H255" s="0" t="s">
         <v>39</v>
@@ -25361,7 +25361,7 @@
     </row>
     <row r="258">
       <c r="A258" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B258" s="0" t="s">
         <v>61</v>
@@ -25695,7 +25695,7 @@
         <v>644</v>
       </c>
       <c r="F262" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G262" s="0" t="s">
         <v>645</v>
@@ -25773,10 +25773,10 @@
         <v>313</v>
       </c>
       <c r="F263" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G263" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H263" s="0" t="s">
         <v>648</v>
@@ -25859,7 +25859,7 @@
         <v>311</v>
       </c>
       <c r="F264" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G264" s="0" t="s">
         <v>650</v>
@@ -26025,7 +26025,7 @@
         <v>654</v>
       </c>
       <c r="D266" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E266" s="0" t="s">
         <v>187</v>
@@ -26112,10 +26112,10 @@
         <v>658</v>
       </c>
       <c r="F267" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G267" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H267" s="0" t="s">
         <v>659</v>
@@ -26192,7 +26192,7 @@
         <v>660</v>
       </c>
       <c r="D268" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E268" s="0" t="s">
         <v>661</v>
@@ -26704,10 +26704,10 @@
         <v>672</v>
       </c>
       <c r="D274" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="E274" s="0" t="s">
         <v>123</v>
-      </c>
-      <c r="E274" s="0" t="s">
-        <v>124</v>
       </c>
       <c r="F274" s="0" t="s">
         <v>38</v>
@@ -26788,10 +26788,10 @@
         <v>673</v>
       </c>
       <c r="D275" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="E275" s="0" t="s">
         <v>123</v>
-      </c>
-      <c r="E275" s="0" t="s">
-        <v>124</v>
       </c>
       <c r="F275" s="0" t="s">
         <v>38</v>
@@ -27049,7 +27049,7 @@
         <v>60</v>
       </c>
       <c r="G278" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H278" s="0" t="s">
         <v>384</v>
@@ -27130,10 +27130,10 @@
         <v>678</v>
       </c>
       <c r="F279" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G279" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H279" s="0" t="s">
         <v>679</v>
@@ -27201,7 +27201,7 @@
     </row>
     <row r="280">
       <c r="A280" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B280" s="0" t="s">
         <v>61</v>
@@ -27287,7 +27287,7 @@
     </row>
     <row r="281">
       <c r="A281" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B281" s="0" t="s">
         <v>61</v>
@@ -27388,10 +27388,10 @@
         <v>683</v>
       </c>
       <c r="F282" s="0" t="s">
+        <v>167</v>
+      </c>
+      <c r="G282" s="0" t="s">
         <v>168</v>
-      </c>
-      <c r="G282" s="0" t="s">
-        <v>169</v>
       </c>
       <c r="H282" s="0" t="s">
         <v>684</v>
@@ -27472,10 +27472,10 @@
         <v>84</v>
       </c>
       <c r="F283" s="0" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G283" s="0" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H283" s="0" t="s">
         <v>686</v>
@@ -27556,10 +27556,10 @@
         <v>688</v>
       </c>
       <c r="F284" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G284" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H284" s="0" t="s">
         <v>686</v>
@@ -27642,10 +27642,10 @@
         <v>688</v>
       </c>
       <c r="F285" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G285" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H285" s="0" t="s">
         <v>686</v>
@@ -27720,13 +27720,13 @@
         <v>690</v>
       </c>
       <c r="D286" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E286" s="0" t="s">
         <v>487</v>
       </c>
       <c r="F286" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G286" s="0" t="s">
         <v>93</v>
@@ -27812,7 +27812,7 @@
         <v>693</v>
       </c>
       <c r="F287" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G287" s="0" t="s">
         <v>526</v>
@@ -27883,7 +27883,7 @@
     </row>
     <row r="288">
       <c r="A288" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B288" s="0" t="s">
         <v>61</v>
@@ -28053,7 +28053,7 @@
     </row>
     <row r="290">
       <c r="A290" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B290" s="0" t="s">
         <v>61</v>
@@ -28139,7 +28139,7 @@
     </row>
     <row r="291">
       <c r="A291" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B291" s="0" t="s">
         <v>61</v>
@@ -28223,7 +28223,7 @@
     </row>
     <row r="292">
       <c r="A292" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B292" s="0" t="s">
         <v>61</v>
@@ -28309,7 +28309,7 @@
     </row>
     <row r="293">
       <c r="A293" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B293" s="0" t="s">
         <v>61</v>
@@ -28324,7 +28324,7 @@
         <v>73</v>
       </c>
       <c r="F293" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G293" s="0" t="s">
         <v>526</v>
@@ -28395,7 +28395,7 @@
     </row>
     <row r="294">
       <c r="A294" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B294" s="0" t="s">
         <v>61</v>
@@ -28481,7 +28481,7 @@
     </row>
     <row r="295">
       <c r="A295" s="0" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B295" s="0" t="s">
         <v>61</v>
@@ -28502,7 +28502,7 @@
         <v>93</v>
       </c>
       <c r="H295" s="0" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="J295" s="11"/>
       <c r="K295" s="0" t="s">
@@ -28568,7 +28568,7 @@
     </row>
     <row r="296">
       <c r="A296" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B296" s="0" t="s">
         <v>61</v>
@@ -28740,7 +28740,7 @@
     </row>
     <row r="298">
       <c r="A298" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B298" s="0" t="s">
         <v>61</v>
@@ -28826,7 +28826,7 @@
     </row>
     <row r="299">
       <c r="A299" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B299" s="0" t="s">
         <v>61</v>
@@ -28912,7 +28912,7 @@
     </row>
     <row r="300">
       <c r="A300" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B300" s="0" t="s">
         <v>61</v>
@@ -28998,7 +28998,7 @@
     </row>
     <row r="301">
       <c r="A301" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B301" s="0" t="s">
         <v>61</v>
@@ -29013,7 +29013,7 @@
         <v>87</v>
       </c>
       <c r="F301" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G301" s="0" t="s">
         <v>526</v>
@@ -29084,7 +29084,7 @@
     </row>
     <row r="302">
       <c r="A302" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B302" s="0" t="s">
         <v>61</v>
@@ -29170,7 +29170,7 @@
     </row>
     <row r="303">
       <c r="A303" s="0" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B303" s="0" t="s">
         <v>61</v>
@@ -29191,7 +29191,7 @@
         <v>93</v>
       </c>
       <c r="H303" s="0" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="J303" s="11"/>
       <c r="K303" s="0" t="s">
@@ -29269,13 +29269,13 @@
         <v>51</v>
       </c>
       <c r="E304" s="0" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F304" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G304" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H304" s="0" t="s">
         <v>719</v>
@@ -29427,7 +29427,7 @@
     </row>
     <row r="306">
       <c r="A306" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B306" s="0" t="s">
         <v>61</v>
@@ -29442,7 +29442,7 @@
         <v>228</v>
       </c>
       <c r="F306" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G306" s="0" t="s">
         <v>332</v>
@@ -29513,7 +29513,7 @@
     </row>
     <row r="307">
       <c r="A307" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B307" s="0" t="s">
         <v>61</v>
@@ -29692,7 +29692,7 @@
         <v>728</v>
       </c>
       <c r="D309" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E309" s="0" t="s">
         <v>547</v>
@@ -29953,10 +29953,10 @@
         <v>734</v>
       </c>
       <c r="F312" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G312" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H312" s="0" t="s">
         <v>731</v>
@@ -30110,7 +30110,7 @@
     </row>
     <row r="314">
       <c r="A314" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B314" s="0" t="s">
         <v>49</v>
@@ -30196,7 +30196,7 @@
     </row>
     <row r="315">
       <c r="A315" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B315" s="0" t="s">
         <v>49</v>
@@ -30366,7 +30366,7 @@
     </row>
     <row r="317">
       <c r="A317" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B317" s="0" t="s">
         <v>61</v>
@@ -30452,7 +30452,7 @@
     </row>
     <row r="318">
       <c r="A318" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B318" s="0" t="s">
         <v>61</v>
@@ -30538,7 +30538,7 @@
     </row>
     <row r="319">
       <c r="A319" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B319" s="0" t="s">
         <v>61</v>
@@ -30553,10 +30553,10 @@
         <v>37</v>
       </c>
       <c r="F319" s="0" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G319" s="0" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H319" s="0" t="s">
         <v>543</v>
@@ -30624,7 +30624,7 @@
     </row>
     <row r="320">
       <c r="A320" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B320" s="0" t="s">
         <v>61</v>
@@ -30639,10 +30639,10 @@
         <v>37</v>
       </c>
       <c r="F320" s="0" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G320" s="0" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H320" s="0" t="s">
         <v>543</v>
@@ -30710,7 +30710,7 @@
     </row>
     <row r="321">
       <c r="A321" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B321" s="0" t="s">
         <v>61</v>
@@ -30725,10 +30725,10 @@
         <v>37</v>
       </c>
       <c r="F321" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G321" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H321" s="0" t="s">
         <v>402</v>
@@ -30796,7 +30796,7 @@
     </row>
     <row r="322">
       <c r="A322" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B322" s="0" t="s">
         <v>61</v>
@@ -30811,10 +30811,10 @@
         <v>37</v>
       </c>
       <c r="F322" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G322" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H322" s="0" t="s">
         <v>402</v>
@@ -30897,10 +30897,10 @@
         <v>750</v>
       </c>
       <c r="F323" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G323" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H323" s="0" t="s">
         <v>751</v>
@@ -30983,10 +30983,10 @@
         <v>750</v>
       </c>
       <c r="F324" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G324" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H324" s="0" t="s">
         <v>751</v>
@@ -31054,7 +31054,7 @@
     </row>
     <row r="325">
       <c r="A325" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B325" s="0" t="s">
         <v>61</v>
@@ -31138,7 +31138,7 @@
     </row>
     <row r="326">
       <c r="A326" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B326" s="0" t="s">
         <v>61</v>
@@ -31222,7 +31222,7 @@
     </row>
     <row r="327">
       <c r="A327" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B327" s="0" t="s">
         <v>61</v>
@@ -31308,7 +31308,7 @@
     </row>
     <row r="328">
       <c r="A328" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B328" s="0" t="s">
         <v>61</v>
@@ -31409,10 +31409,10 @@
         <v>760</v>
       </c>
       <c r="F329" s="0" t="s">
+        <v>148</v>
+      </c>
+      <c r="G329" s="0" t="s">
         <v>149</v>
-      </c>
-      <c r="G329" s="0" t="s">
-        <v>150</v>
       </c>
       <c r="J329" s="11">
         <v>46386.125</v>
@@ -31474,7 +31474,7 @@
     </row>
     <row r="330">
       <c r="A330" s="0" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B330" s="0" t="s">
         <v>61</v>
@@ -31489,13 +31489,13 @@
         <v>87</v>
       </c>
       <c r="F330" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G330" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H330" s="0" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J330" s="11"/>
       <c r="K330" s="0" t="s">
@@ -31561,7 +31561,7 @@
     </row>
     <row r="331">
       <c r="A331" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B331" s="0" t="s">
         <v>61</v>
@@ -31576,13 +31576,13 @@
         <v>73</v>
       </c>
       <c r="F331" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G331" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H331" s="0" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J331" s="11"/>
       <c r="K331" s="0" t="s">
@@ -31663,7 +31663,7 @@
         <v>85</v>
       </c>
       <c r="G332" s="0" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H332" s="0" t="s">
         <v>764</v>
@@ -32000,10 +32000,10 @@
         <v>769</v>
       </c>
       <c r="F336" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G336" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J336" s="11">
         <v>46403.125</v>
@@ -32083,7 +32083,7 @@
         <v>304</v>
       </c>
       <c r="F337" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G337" s="0" t="s">
         <v>79</v>
@@ -32169,7 +32169,7 @@
         <v>304</v>
       </c>
       <c r="F338" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G338" s="0" t="s">
         <v>79</v>
@@ -32249,7 +32249,7 @@
         <v>772</v>
       </c>
       <c r="D339" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E339" s="0" t="s">
         <v>216</v>
@@ -32324,7 +32324,7 @@
     </row>
     <row r="340">
       <c r="A340" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B340" s="0" t="s">
         <v>34</v>
@@ -32333,10 +32333,10 @@
         <v>774</v>
       </c>
       <c r="D340" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="E340" s="0" t="s">
         <v>140</v>
-      </c>
-      <c r="E340" s="0" t="s">
-        <v>141</v>
       </c>
       <c r="F340" s="0" t="s">
         <v>243</v>
@@ -32417,7 +32417,7 @@
         <v>775</v>
       </c>
       <c r="D341" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E341" s="0" t="s">
         <v>216</v>
@@ -32494,7 +32494,7 @@
     </row>
     <row r="342">
       <c r="A342" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B342" s="0" t="s">
         <v>61</v>
@@ -32509,7 +32509,7 @@
         <v>37</v>
       </c>
       <c r="F342" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G342" s="0" t="s">
         <v>526</v>
@@ -32669,7 +32669,7 @@
         <v>780</v>
       </c>
       <c r="D344" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E344" s="0" t="s">
         <v>216</v>
@@ -32746,7 +32746,7 @@
     </row>
     <row r="345">
       <c r="A345" s="0" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B345" s="0" t="s">
         <v>61</v>
@@ -32764,7 +32764,7 @@
         <v>60</v>
       </c>
       <c r="G345" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H345" s="0" t="s">
         <v>781</v>
@@ -32847,13 +32847,13 @@
         <v>51</v>
       </c>
       <c r="E346" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="F346" s="0" t="s">
         <v>130</v>
       </c>
-      <c r="F346" s="0" t="s">
-        <v>131</v>
-      </c>
       <c r="G346" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H346" s="0" t="s">
         <v>785</v>
@@ -33177,7 +33177,7 @@
         <v>795</v>
       </c>
       <c r="F350" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G350" s="0" t="s">
         <v>526</v>
@@ -33426,10 +33426,10 @@
         <v>803</v>
       </c>
       <c r="F353" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G353" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J353" s="11">
         <v>46399.125</v>
@@ -33491,7 +33491,7 @@
     </row>
     <row r="354">
       <c r="A354" s="0" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B354" s="0" t="s">
         <v>34</v>
@@ -33741,7 +33741,7 @@
     </row>
     <row r="357">
       <c r="A357" s="0" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B357" s="0" t="s">
         <v>61</v>
@@ -33753,7 +33753,7 @@
         <v>51</v>
       </c>
       <c r="E357" s="0" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F357" s="0" t="s">
         <v>79</v>
@@ -33830,7 +33830,7 @@
     </row>
     <row r="358">
       <c r="A358" s="0" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B358" s="0" t="s">
         <v>61</v>
@@ -33845,10 +33845,10 @@
         <v>810</v>
       </c>
       <c r="F358" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G358" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H358" s="0" t="s">
         <v>756</v>
@@ -34017,7 +34017,7 @@
         <v>815</v>
       </c>
       <c r="E360" s="0" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F360" s="0" t="s">
         <v>428</v>
@@ -34094,7 +34094,7 @@
         <v>816</v>
       </c>
       <c r="D361" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E361" s="0" t="s">
         <v>216</v>
@@ -34255,7 +34255,7 @@
     </row>
     <row r="363">
       <c r="A363" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B363" s="0" t="s">
         <v>34</v>
@@ -34354,10 +34354,10 @@
         <v>511</v>
       </c>
       <c r="F364" s="0" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G364" s="0" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H364" s="0" t="s">
         <v>281</v>
@@ -34524,7 +34524,7 @@
         <v>693</v>
       </c>
       <c r="F366" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G366" s="0" t="s">
         <v>526</v>
@@ -34696,7 +34696,7 @@
         <v>827</v>
       </c>
       <c r="F368" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G368" s="0" t="s">
         <v>526</v>
@@ -34788,7 +34788,7 @@
         <v>200</v>
       </c>
       <c r="H369" s="0" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="J369" s="11">
         <v>46391.125</v>
@@ -34865,7 +34865,7 @@
         <v>63</v>
       </c>
       <c r="E370" s="0" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F370" s="0" t="s">
         <v>74</v>
@@ -34957,7 +34957,7 @@
         <v>60</v>
       </c>
       <c r="G371" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H371" s="0" t="s">
         <v>834</v>
@@ -35035,7 +35035,7 @@
         <v>839</v>
       </c>
       <c r="H372" s="0" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="J372" s="11">
         <v>46391.125</v>
@@ -35337,7 +35337,7 @@
     </row>
     <row r="376">
       <c r="A376" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B376" s="0" t="s">
         <v>34</v>
@@ -35423,7 +35423,7 @@
     </row>
     <row r="377">
       <c r="A377" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B377" s="0" t="s">
         <v>61</v>
@@ -35506,7 +35506,7 @@
     </row>
     <row r="378">
       <c r="A378" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B378" s="0" t="s">
         <v>61</v>
@@ -35856,7 +35856,7 @@
         <v>60</v>
       </c>
       <c r="G382" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J382" s="11"/>
       <c r="K382" s="0" t="s">
@@ -36005,7 +36005,7 @@
     </row>
     <row r="384">
       <c r="A384" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B384" s="0" t="s">
         <v>34</v>
@@ -36272,7 +36272,7 @@
         <v>869</v>
       </c>
       <c r="D387" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E387" s="0" t="s">
         <v>487</v>
@@ -36364,10 +36364,10 @@
         <v>503</v>
       </c>
       <c r="F388" s="0" t="s">
+        <v>148</v>
+      </c>
+      <c r="G388" s="0" t="s">
         <v>149</v>
-      </c>
-      <c r="G388" s="0" t="s">
-        <v>150</v>
       </c>
       <c r="H388" s="0" t="s">
         <v>872</v>
@@ -36450,10 +36450,10 @@
         <v>59</v>
       </c>
       <c r="F389" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G389" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H389" s="0" t="s">
         <v>874</v>
@@ -36521,7 +36521,7 @@
     </row>
     <row r="390">
       <c r="A390" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B390" s="0" t="s">
         <v>34</v>
@@ -36536,10 +36536,10 @@
         <v>37</v>
       </c>
       <c r="F390" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G390" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H390" s="0" t="s">
         <v>874</v>
@@ -36706,10 +36706,10 @@
         <v>322</v>
       </c>
       <c r="F392" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G392" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H392" s="0" t="s">
         <v>878</v>
@@ -37119,7 +37119,7 @@
     </row>
     <row r="397">
       <c r="A397" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B397" s="0" t="s">
         <v>34</v>
@@ -37134,10 +37134,10 @@
         <v>888</v>
       </c>
       <c r="F397" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G397" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H397" s="0" t="s">
         <v>886</v>
@@ -37203,7 +37203,7 @@
     </row>
     <row r="398">
       <c r="A398" s="0" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B398" s="0" t="s">
         <v>34</v>
@@ -37218,10 +37218,10 @@
         <v>890</v>
       </c>
       <c r="F398" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G398" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H398" s="0" t="s">
         <v>344</v>
@@ -37290,7 +37290,7 @@
     </row>
     <row r="399">
       <c r="A399" s="0" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B399" s="0" t="s">
         <v>34</v>
@@ -37302,10 +37302,10 @@
         <v>51</v>
       </c>
       <c r="E399" s="0" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F399" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G399" s="0" t="s">
         <v>332</v>
@@ -37379,7 +37379,7 @@
     </row>
     <row r="400">
       <c r="A400" s="0" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B400" s="0" t="s">
         <v>34</v>
@@ -37388,16 +37388,16 @@
         <v>893</v>
       </c>
       <c r="D400" s="0" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E400" s="0" t="s">
         <v>894</v>
       </c>
       <c r="F400" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G400" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H400" s="0" t="s">
         <v>895</v>
@@ -37466,7 +37466,7 @@
     </row>
     <row r="401">
       <c r="A401" s="0" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B401" s="0" t="s">
         <v>34</v>
@@ -37475,7 +37475,7 @@
         <v>896</v>
       </c>
       <c r="D401" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E401" s="0" t="s">
         <v>897</v>
@@ -37562,10 +37562,10 @@
         <v>899</v>
       </c>
       <c r="D402" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="E402" s="0" t="s">
         <v>123</v>
-      </c>
-      <c r="E402" s="0" t="s">
-        <v>124</v>
       </c>
       <c r="F402" s="0" t="s">
         <v>60</v>
@@ -37646,10 +37646,10 @@
         <v>900</v>
       </c>
       <c r="D403" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="E403" s="0" t="s">
         <v>123</v>
-      </c>
-      <c r="E403" s="0" t="s">
-        <v>124</v>
       </c>
       <c r="F403" s="0" t="s">
         <v>60</v>
@@ -37819,10 +37819,10 @@
         <v>92</v>
       </c>
       <c r="F405" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G405" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H405" s="0" t="s">
         <v>527</v>
@@ -37890,7 +37890,7 @@
     </row>
     <row r="406">
       <c r="A406" s="0" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B406" s="0" t="s">
         <v>34</v>
@@ -37977,7 +37977,7 @@
     </row>
     <row r="407">
       <c r="A407" s="0" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B407" s="0" t="s">
         <v>34</v>
@@ -38162,10 +38162,10 @@
         <v>322</v>
       </c>
       <c r="F409" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G409" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J409" s="11">
         <v>46407.125</v>
@@ -38230,7 +38230,7 @@
     </row>
     <row r="410">
       <c r="A410" s="0" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B410" s="0" t="s">
         <v>34</v>
@@ -38415,10 +38415,10 @@
         <v>916</v>
       </c>
       <c r="F412" s="0" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G412" s="0" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J412" s="11">
         <v>46399.125</v>
@@ -38498,10 +38498,10 @@
         <v>521</v>
       </c>
       <c r="F413" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G413" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H413" s="0" t="s">
         <v>918</v>
@@ -38653,7 +38653,7 @@
     </row>
     <row r="415">
       <c r="A415" s="0" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B415" s="0" t="s">
         <v>61</v>
@@ -38740,7 +38740,7 @@
     </row>
     <row r="416">
       <c r="A416" s="0" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B416" s="0" t="s">
         <v>61</v>
@@ -38749,16 +38749,16 @@
         <v>924</v>
       </c>
       <c r="D416" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E416" s="0" t="s">
         <v>925</v>
       </c>
       <c r="F416" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G416" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H416" s="0" t="s">
         <v>224</v>
@@ -38924,7 +38924,7 @@
         <v>928</v>
       </c>
       <c r="D418" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E418" s="0" t="s">
         <v>929</v>
@@ -39011,13 +39011,13 @@
         <v>51</v>
       </c>
       <c r="E419" s="0" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F419" s="0" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G419" s="0" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H419" s="0" t="s">
         <v>932</v>
@@ -39085,7 +39085,7 @@
     </row>
     <row r="420">
       <c r="A420" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B420" s="0" t="s">
         <v>61</v>
@@ -39169,7 +39169,7 @@
     </row>
     <row r="421">
       <c r="A421" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B421" s="0" t="s">
         <v>61</v>
@@ -39253,7 +39253,7 @@
     </row>
     <row r="422">
       <c r="A422" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B422" s="0" t="s">
         <v>61</v>
@@ -39268,7 +39268,7 @@
         <v>260</v>
       </c>
       <c r="F422" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G422" s="0" t="s">
         <v>93</v>
@@ -39337,7 +39337,7 @@
     </row>
     <row r="423">
       <c r="A423" s="0" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B423" s="0" t="s">
         <v>61</v>
@@ -39352,10 +39352,10 @@
         <v>938</v>
       </c>
       <c r="F423" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G423" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H423" s="0" t="s">
         <v>923</v>
@@ -39424,7 +39424,7 @@
     </row>
     <row r="424">
       <c r="A424" s="0" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B424" s="0" t="s">
         <v>61</v>
@@ -39511,7 +39511,7 @@
     </row>
     <row r="425">
       <c r="A425" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B425" s="0" t="s">
         <v>61</v>
@@ -39532,7 +39532,7 @@
         <v>300</v>
       </c>
       <c r="H425" s="0" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="J425" s="11">
         <v>46373.125</v>
@@ -39597,7 +39597,7 @@
     </row>
     <row r="426">
       <c r="A426" s="0" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B426" s="0" t="s">
         <v>61</v>
@@ -39612,7 +39612,7 @@
         <v>260</v>
       </c>
       <c r="F426" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G426" s="0" t="s">
         <v>526</v>
@@ -39684,7 +39684,7 @@
     </row>
     <row r="427">
       <c r="A427" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B427" s="0" t="s">
         <v>61</v>
@@ -39699,10 +39699,10 @@
         <v>73</v>
       </c>
       <c r="F427" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G427" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H427" s="0" t="s">
         <v>945</v>
@@ -39770,7 +39770,7 @@
     </row>
     <row r="428">
       <c r="A428" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B428" s="0" t="s">
         <v>61</v>
@@ -39854,7 +39854,7 @@
     </row>
     <row r="429">
       <c r="A429" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B429" s="0" t="s">
         <v>61</v>
@@ -39938,7 +39938,7 @@
     </row>
     <row r="430">
       <c r="A430" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B430" s="0" t="s">
         <v>61</v>
@@ -40024,7 +40024,7 @@
     </row>
     <row r="431">
       <c r="A431" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B431" s="0" t="s">
         <v>61</v>
@@ -40108,7 +40108,7 @@
     </row>
     <row r="432">
       <c r="A432" s="0" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B432" s="0" t="s">
         <v>61</v>
@@ -40123,7 +40123,7 @@
         <v>260</v>
       </c>
       <c r="F432" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G432" s="0" t="s">
         <v>526</v>
@@ -40195,7 +40195,7 @@
     </row>
     <row r="433">
       <c r="A433" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B433" s="0" t="s">
         <v>61</v>
@@ -40210,10 +40210,10 @@
         <v>87</v>
       </c>
       <c r="F433" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G433" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H433" s="0" t="s">
         <v>945</v>
@@ -40281,7 +40281,7 @@
     </row>
     <row r="434">
       <c r="A434" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B434" s="0" t="s">
         <v>61</v>
@@ -40374,7 +40374,7 @@
         <v>953</v>
       </c>
       <c r="D435" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E435" s="0" t="s">
         <v>175</v>
@@ -40458,7 +40458,7 @@
         <v>955</v>
       </c>
       <c r="D436" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E436" s="0" t="s">
         <v>956</v>
@@ -40544,7 +40544,7 @@
         <v>958</v>
       </c>
       <c r="D437" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E437" s="0" t="s">
         <v>175</v>
@@ -40628,7 +40628,7 @@
         <v>960</v>
       </c>
       <c r="D438" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E438" s="0" t="s">
         <v>961</v>
@@ -40715,7 +40715,7 @@
         <v>963</v>
       </c>
       <c r="D439" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E439" s="0" t="s">
         <v>191</v>
@@ -41122,7 +41122,7 @@
     </row>
     <row r="444">
       <c r="A444" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B444" s="0" t="s">
         <v>34</v>
@@ -41137,10 +41137,10 @@
         <v>37</v>
       </c>
       <c r="F444" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G444" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="J444" s="11">
         <v>46394.125</v>
@@ -41214,10 +41214,10 @@
         <v>972</v>
       </c>
       <c r="D445" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="E445" s="0" t="s">
         <v>123</v>
-      </c>
-      <c r="E445" s="0" t="s">
-        <v>124</v>
       </c>
       <c r="F445" s="0" t="s">
         <v>38</v>
@@ -41300,10 +41300,10 @@
         <v>974</v>
       </c>
       <c r="D446" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="E446" s="0" t="s">
         <v>123</v>
-      </c>
-      <c r="E446" s="0" t="s">
-        <v>124</v>
       </c>
       <c r="F446" s="0" t="s">
         <v>38</v>
@@ -41478,10 +41478,10 @@
         <v>977</v>
       </c>
       <c r="F448" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G448" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H448" s="0" t="s">
         <v>535</v>
@@ -41562,10 +41562,10 @@
         <v>979</v>
       </c>
       <c r="F449" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G449" s="0" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H449" s="0" t="s">
         <v>980</v>
@@ -41575,7 +41575,7 @@
         <v>40</v>
       </c>
       <c r="L449" s="0" t="s">
-        <v>120</v>
+        <v>170</v>
       </c>
       <c r="M449" s="0" t="s">
         <v>39</v>
@@ -41884,7 +41884,7 @@
     </row>
     <row r="453">
       <c r="A453" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B453" s="0" t="s">
         <v>61</v>
@@ -41899,10 +41899,10 @@
         <v>37</v>
       </c>
       <c r="F453" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G453" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H453" s="0" t="s">
         <v>989</v>
@@ -41970,7 +41970,7 @@
     </row>
     <row r="454">
       <c r="A454" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B454" s="0" t="s">
         <v>61</v>
@@ -41985,10 +41985,10 @@
         <v>37</v>
       </c>
       <c r="F454" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G454" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H454" s="0" t="s">
         <v>989</v>
@@ -42056,7 +42056,7 @@
     </row>
     <row r="455">
       <c r="A455" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B455" s="0" t="s">
         <v>61</v>
@@ -42142,7 +42142,7 @@
     </row>
     <row r="456">
       <c r="A456" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B456" s="0" t="s">
         <v>61</v>
@@ -42249,7 +42249,7 @@
         <v>74</v>
       </c>
       <c r="H457" s="0" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="J457" s="11">
         <v>46399.125</v>
@@ -42329,10 +42329,10 @@
         <v>998</v>
       </c>
       <c r="F458" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G458" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H458" s="0" t="s">
         <v>999</v>
@@ -42646,7 +42646,7 @@
     </row>
     <row r="462">
       <c r="A462" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B462" s="0" t="s">
         <v>61</v>
@@ -42732,7 +42732,7 @@
     </row>
     <row r="463">
       <c r="A463" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B463" s="0" t="s">
         <v>61</v>
@@ -42760,7 +42760,7 @@
         <v>40</v>
       </c>
       <c r="L463" s="0" t="s">
-        <v>120</v>
+        <v>170</v>
       </c>
       <c r="M463" s="0" t="s">
         <v>39</v>
@@ -42828,13 +42828,13 @@
         <v>51</v>
       </c>
       <c r="E464" s="0" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F464" s="0" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G464" s="0" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H464" s="0" t="s">
         <v>1013</v>
@@ -42902,7 +42902,7 @@
     </row>
     <row r="465">
       <c r="A465" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B465" s="0" t="s">
         <v>61</v>
@@ -42988,7 +42988,7 @@
     </row>
     <row r="466">
       <c r="A466" s="0" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B466" s="0" t="s">
         <v>61</v>
@@ -43419,10 +43419,10 @@
         <v>1025</v>
       </c>
       <c r="F471" s="0" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G471" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J471" s="11">
         <v>46360.125</v>
@@ -43502,10 +43502,10 @@
         <v>339</v>
       </c>
       <c r="F472" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G472" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J472" s="11">
         <v>46356.125</v>
@@ -43585,10 +43585,10 @@
         <v>339</v>
       </c>
       <c r="F473" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G473" s="0" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J473" s="11">
         <v>46356.125</v>
@@ -44006,10 +44006,10 @@
         <v>1034</v>
       </c>
       <c r="F478" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G478" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J478" s="11">
         <v>46369.125</v>
@@ -44157,7 +44157,7 @@
     </row>
     <row r="480">
       <c r="A480" s="0" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B480" s="0" t="s">
         <v>61</v>
@@ -44668,10 +44668,10 @@
         <v>1049</v>
       </c>
       <c r="F486" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G486" s="0" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J486" s="11"/>
       <c r="K486" s="0" t="s">
@@ -44735,10 +44735,10 @@
         <v>1052</v>
       </c>
       <c r="F487" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G487" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="J487" s="11"/>
       <c r="K487" s="0" t="s">

</xml_diff>